<commit_message>
Meta-facturen gekoppeld via transactie-ID's (activiteitenlog)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qy9hDxpZfcAYZj3ievLnBb
</commit_message>
<xml_diff>
--- a/boekhouding/rapporten/SmartPaw_Q3-2026.xlsx
+++ b/boekhouding/rapporten/SmartPaw_Q3-2026.xlsx
@@ -586,7 +586,7 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>104</v>
+        <v>77</v>
       </c>
     </row>
     <row r="14">
@@ -7137,7 +7137,7 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>Bewijs per verrichting: 0 gekoppeld, 78 verklaard (geen factuur nodig, niet in deze lijst), 104 ontbreken. Facturen zitten in de map Facturen_Q3-2026 (bestandsnaam = datum_leverancier_bedrag).</t>
+          <t>Bewijs per verrichting: 27 gekoppeld, 78 verklaard (geen factuur nodig, niet in deze lijst), 77 ontbreken. Facturen zitten in de map Facturen_Q3-2026 (bestandsnaam = datum_leverancier_bedrag).</t>
         </is>
       </c>
     </row>
@@ -7181,11 +7181,11 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">FACEBK *X87X6SV7A2 IED04 X2K5 Dublin Betaling met </t>
+          <t>GOOGLE*WORKSPACE SMART IED02 R296 CC GOOGLE.COM Be</t>
         </is>
       </c>
       <c r="C4" s="9" t="n">
-        <v>-800</v>
+        <v>-75.90000000000001</v>
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
@@ -7207,15 +7207,15 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>GOOGLE*WORKSPACE SMART IED02 R296 CC GOOGLE.COM Be</t>
+          <t>Yuki Works NV via Mollie</t>
         </is>
       </c>
       <c r="C5" s="9" t="n">
-        <v>-75.90000000000001</v>
+        <v>-2.42</v>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
@@ -7233,15 +7233,15 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>Yuki Works NV via Mollie</t>
+          <t>Google ADS4790542578</t>
         </is>
       </c>
       <c r="C6" s="9" t="n">
-        <v>-2.42</v>
+        <v>-158.5</v>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
@@ -7254,20 +7254,20 @@
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Google ADS4790542578</t>
+          <t>RETURNGO</t>
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>-158.5</v>
+        <v>-86</v>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>NONEU</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
@@ -7280,20 +7280,20 @@
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>RETURNGO</t>
+          <t>Pro-Count</t>
         </is>
       </c>
       <c r="C8" s="9" t="n">
-        <v>-86</v>
+        <v>-242</v>
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>NONEU</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
@@ -7337,11 +7337,11 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Pro-Count</t>
+          <t>Widem Logistics NV</t>
         </is>
       </c>
       <c r="C10" s="9" t="n">
-        <v>-242</v>
+        <v>-527.83</v>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
@@ -7363,11 +7363,11 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>Widem Logistics NV</t>
+          <t>Findajob bv</t>
         </is>
       </c>
       <c r="C11" s="9" t="n">
-        <v>-527.83</v>
+        <v>-75.78</v>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
@@ -7389,15 +7389,15 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Findajob bv</t>
+          <t>Henri Steyaert</t>
         </is>
       </c>
       <c r="C12" s="9" t="n">
-        <v>-75.78</v>
+        <v>-91.84</v>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>NAKIJKEN</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
@@ -7415,15 +7415,15 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Henri Steyaert</t>
+          <t>Findajob bv</t>
         </is>
       </c>
       <c r="C13" s="9" t="n">
-        <v>-91.84</v>
+        <v>-18.95</v>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>NAKIJKEN</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
@@ -7436,20 +7436,20 @@
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Findajob bv</t>
+          <t>Company Pro plan fee</t>
         </is>
       </c>
       <c r="C14" s="9" t="n">
-        <v>-18.95</v>
+        <v>-35</v>
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>GEEN</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
@@ -7462,16 +7462,16 @@
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">FACEBK *W9EF8UH8A2 IED04 X2K5 Dublin Betaling met </t>
+          <t>HOLO AI</t>
         </is>
       </c>
       <c r="C15" s="9" t="n">
-        <v>-800</v>
+        <v>-41.98</v>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
@@ -7488,20 +7488,20 @@
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Company Pro plan fee</t>
+          <t>WIDEM LOGISTICS NV</t>
         </is>
       </c>
       <c r="C16" s="9" t="n">
-        <v>-35</v>
+        <v>-261.04</v>
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>GEEN</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
@@ -7514,20 +7514,20 @@
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">FACEBK *RQQRHTR7A2 IED04 X2K5 Dublin Betaling met </t>
+          <t>WIDEM LOGISTICS NV</t>
         </is>
       </c>
       <c r="C17" s="9" t="n">
-        <v>-278.57</v>
+        <v>-364.58</v>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
@@ -7540,20 +7540,20 @@
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>HOLO AI</t>
+          <t>KLAVIYO INC. SOFTWARE</t>
         </is>
       </c>
       <c r="C18" s="9" t="n">
-        <v>-41.98</v>
+        <v>-53.5</v>
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>NONEU</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr">
@@ -7566,20 +7566,20 @@
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>WIDEM LOGISTICS NV</t>
+          <t>SHOPIFY* 556521062</t>
         </is>
       </c>
       <c r="C19" s="9" t="n">
-        <v>-261.04</v>
+        <v>-141.39</v>
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
@@ -7592,20 +7592,20 @@
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>WIDEM LOGISTICS NV</t>
+          <t>Google ADS4790542578</t>
         </is>
       </c>
       <c r="C20" s="9" t="n">
-        <v>-364.58</v>
+        <v>-500</v>
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
@@ -7618,16 +7618,16 @@
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>KLAVIYO INC. SOFTWARE</t>
+          <t>HIGGSFIELD INC. US94105 SAN FRANCISCO Betaling met</t>
         </is>
       </c>
       <c r="C21" s="9" t="n">
-        <v>-53.5</v>
+        <v>-72</v>
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
@@ -7644,20 +7644,20 @@
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>SHOPIFY* 556521062</t>
+          <t>SP PACKAGINGDISCOUNTER</t>
         </is>
       </c>
       <c r="C22" s="9" t="n">
-        <v>-141.39</v>
+        <v>-665</v>
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>NAKIJKEN</t>
         </is>
       </c>
       <c r="E22" s="8" t="inlineStr">
@@ -7670,20 +7670,20 @@
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>Google ADS4790542578</t>
+          <t>SP PACKAGINGDISCOUNTER</t>
         </is>
       </c>
       <c r="C23" s="9" t="n">
-        <v>-500</v>
+        <v>-360</v>
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>NAKIJKEN</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
@@ -7696,20 +7696,20 @@
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">FACEBK *AF4S7TM7A2 IED04 X2K5 Dublin Betaling met </t>
+          <t>BPOST NV BE1000 BRUXELLES Betaling met KBC-Debetka</t>
         </is>
       </c>
       <c r="C24" s="9" t="n">
-        <v>-800</v>
+        <v>-5.6</v>
       </c>
       <c r="D24" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr">
@@ -7722,20 +7722,20 @@
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">FACEBK *G99QSTM8A2 IED04 X2K5 Dublin Betaling met </t>
+          <t>YAKI NOODLE BAR BE9000 GENT Betaling met KBC-Debet</t>
         </is>
       </c>
       <c r="C25" s="9" t="n">
-        <v>-800</v>
+        <v>-15</v>
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>BE21NA</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
@@ -7748,20 +7748,20 @@
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>HIGGSFIELD INC. US94105 SAN FRANCISCO Betaling met</t>
+          <t>AMBULANTE ZELFSTANDIGEN VZW</t>
         </is>
       </c>
       <c r="C26" s="9" t="n">
-        <v>-72</v>
+        <v>-210</v>
       </c>
       <c r="D26" s="8" t="inlineStr">
         <is>
-          <t>NONEU</t>
+          <t>NAKIJKEN</t>
         </is>
       </c>
       <c r="E26" s="8" t="inlineStr">
@@ -7774,20 +7774,20 @@
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>SP PACKAGINGDISCOUNTER</t>
+          <t xml:space="preserve">Shopify Hardware Store IED04 Xn32 Dublin Betaling </t>
         </is>
       </c>
       <c r="C27" s="9" t="n">
-        <v>-665</v>
+        <v>-59</v>
       </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
-          <t>NAKIJKEN</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
@@ -7800,20 +7800,20 @@
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B28" s="8" t="inlineStr">
         <is>
-          <t>SP PACKAGINGDISCOUNTER</t>
+          <t>KBC Verzekeringen</t>
         </is>
       </c>
       <c r="C28" s="9" t="n">
-        <v>-360</v>
+        <v>-18.47</v>
       </c>
       <c r="D28" s="8" t="inlineStr">
         <is>
-          <t>NAKIJKEN</t>
+          <t>GEEN</t>
         </is>
       </c>
       <c r="E28" s="8" t="inlineStr">
@@ -7826,16 +7826,16 @@
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>BPOST NV BE1000 BRUXELLES Betaling met KBC-Debetka</t>
+          <t>FINDAJOB BV</t>
         </is>
       </c>
       <c r="C29" s="9" t="n">
-        <v>-5.6</v>
+        <v>-293.64</v>
       </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
@@ -7852,20 +7852,20 @@
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B30" s="8" t="inlineStr">
         <is>
-          <t>YAKI NOODLE BAR BE9000 GENT Betaling met KBC-Debet</t>
+          <t>BPOST NV BE1000 BRUXELLES Betaling met KBC-Debetka</t>
         </is>
       </c>
       <c r="C30" s="9" t="n">
-        <v>-15</v>
+        <v>-7.1</v>
       </c>
       <c r="D30" s="8" t="inlineStr">
         <is>
-          <t>BE21NA</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="E30" s="8" t="inlineStr">
@@ -7878,20 +7878,20 @@
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">FACEBK *25EEEVR7A2 IED04 X2K5 Dublin Betaling met </t>
+          <t>bpost parcel</t>
         </is>
       </c>
       <c r="C31" s="9" t="n">
-        <v>-800</v>
+        <v>-7.1</v>
       </c>
       <c r="D31" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
@@ -7904,20 +7904,20 @@
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>AMBULANTE ZELFSTANDIGEN VZW</t>
+          <t xml:space="preserve">Plus Gent BE9000 Gent Betaling met KBC-Debetkaart </t>
         </is>
       </c>
       <c r="C32" s="9" t="n">
-        <v>-210</v>
+        <v>-47.1</v>
       </c>
       <c r="D32" s="8" t="inlineStr">
         <is>
-          <t>NAKIJKEN</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="E32" s="8" t="inlineStr">
@@ -7930,20 +7930,20 @@
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shopify Hardware Store IED04 Xn32 Dublin Betaling </t>
+          <t>Google ADS4790542578</t>
         </is>
       </c>
       <c r="C33" s="9" t="n">
-        <v>-59</v>
+        <v>-198.56</v>
       </c>
       <c r="D33" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
@@ -7956,20 +7956,20 @@
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>KBC Verzekeringen</t>
+          <t>bpost parcel</t>
         </is>
       </c>
       <c r="C34" s="9" t="n">
-        <v>-18.47</v>
+        <v>-7.85</v>
       </c>
       <c r="D34" s="8" t="inlineStr">
         <is>
-          <t>GEEN</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="E34" s="8" t="inlineStr">
@@ -7982,20 +7982,20 @@
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>FINDAJOB BV</t>
+          <t>GOOGLE*WORKSPACE SMART IED02 R296 CC GOOGLE.COM Be</t>
         </is>
       </c>
       <c r="C35" s="9" t="n">
-        <v>-293.64</v>
+        <v>-75.90000000000001</v>
       </c>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E35" s="8" t="inlineStr">
@@ -8008,16 +8008,16 @@
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B36" s="8" t="inlineStr">
         <is>
-          <t>BPOST NV BE1000 BRUXELLES Betaling met KBC-Debetka</t>
+          <t>Yuki Works NV via Mollie</t>
         </is>
       </c>
       <c r="C36" s="9" t="n">
-        <v>-7.1</v>
+        <v>-2.42</v>
       </c>
       <c r="D36" s="8" t="inlineStr">
         <is>
@@ -8034,20 +8034,20 @@
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
-          <t>bpost parcel</t>
+          <t>SHOPIFY* 569354127</t>
         </is>
       </c>
       <c r="C37" s="9" t="n">
-        <v>-7.1</v>
+        <v>-174.81</v>
       </c>
       <c r="D37" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E37" s="8" t="inlineStr">
@@ -8060,20 +8060,20 @@
     <row r="38">
       <c r="A38" s="8" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B38" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Plus Gent BE9000 Gent Betaling met KBC-Debetkaart </t>
+          <t>Company Pro plan fee</t>
         </is>
       </c>
       <c r="C38" s="9" t="n">
-        <v>-47.1</v>
+        <v>-35</v>
       </c>
       <c r="D38" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>GEEN</t>
         </is>
       </c>
       <c r="E38" s="8" t="inlineStr">
@@ -8086,20 +8086,20 @@
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">FACEBK *Y2RWNU98A2 IED04 X2K5 Dublin Betaling met </t>
+          <t>Action 2009 BE8560 Wevelgem Betaling met Apple Pay</t>
         </is>
       </c>
       <c r="C39" s="9" t="n">
-        <v>-800</v>
+        <v>-10.02</v>
       </c>
       <c r="D39" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="E39" s="8" t="inlineStr">
@@ -8112,20 +8112,20 @@
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B40" s="8" t="inlineStr">
         <is>
-          <t>Google ADS4790542578</t>
+          <t>AMBULANTE ZELFSTANDIGEN VZW</t>
         </is>
       </c>
       <c r="C40" s="9" t="n">
-        <v>-198.56</v>
+        <v>-230</v>
       </c>
       <c r="D40" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>NAKIJKEN</t>
         </is>
       </c>
       <c r="E40" s="8" t="inlineStr">
@@ -8138,20 +8138,20 @@
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B41" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">FACEBK *CTEE3XH8A2 IED04 X2K5 Dublin Betaling met </t>
+          <t xml:space="preserve">Hotel on Booking.com NL1017 CE AMSTERDAM Betaling </t>
         </is>
       </c>
       <c r="C41" s="9" t="n">
-        <v>-800</v>
+        <v>-94.25</v>
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>GEEN</t>
         </is>
       </c>
       <c r="E41" s="8" t="inlineStr">
@@ -8164,20 +8164,20 @@
     <row r="42">
       <c r="A42" s="8" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B42" s="8" t="inlineStr">
         <is>
-          <t>bpost parcel</t>
+          <t>AMBULANTE ZELFSTANDIGEN VZW</t>
         </is>
       </c>
       <c r="C42" s="9" t="n">
-        <v>-7.85</v>
+        <v>-230</v>
       </c>
       <c r="D42" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>NAKIJKEN</t>
         </is>
       </c>
       <c r="E42" s="8" t="inlineStr">
@@ -8190,16 +8190,16 @@
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B43" s="8" t="inlineStr">
         <is>
-          <t>GOOGLE*WORKSPACE SMART IED02 R296 CC GOOGLE.COM Be</t>
+          <t>SHOPIFY* 571029665</t>
         </is>
       </c>
       <c r="C43" s="9" t="n">
-        <v>-75.90000000000001</v>
+        <v>-32</v>
       </c>
       <c r="D43" s="8" t="inlineStr">
         <is>
@@ -8216,20 +8216,20 @@
     <row r="44">
       <c r="A44" s="8" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B44" s="8" t="inlineStr">
         <is>
-          <t>Yuki Works NV via Mollie</t>
+          <t>KLAVIYO INC. SOFTWARE</t>
         </is>
       </c>
       <c r="C44" s="9" t="n">
-        <v>-2.42</v>
+        <v>-52.94</v>
       </c>
       <c r="D44" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>NONEU</t>
         </is>
       </c>
       <c r="E44" s="8" t="inlineStr">
@@ -8242,20 +8242,20 @@
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">FACEBK *LWJTNVM7A2 IED04 X2K5 Dublin Betaling met </t>
+          <t>Drukbedrijf.nl NL1114AE Amsterdam Betaling met KBC</t>
         </is>
       </c>
       <c r="C45" s="9" t="n">
-        <v>-800</v>
+        <v>-174.28</v>
       </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>NAKIJKEN</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr">
@@ -8268,20 +8268,20 @@
     <row r="46">
       <c r="A46" s="8" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B46" s="8" t="inlineStr">
         <is>
-          <t>SHOPIFY* 569354127</t>
+          <t>THE SANTIBAL BE8700 TIELT Betaling met KBC-Debetka</t>
         </is>
       </c>
       <c r="C46" s="9" t="n">
-        <v>-174.81</v>
+        <v>-27</v>
       </c>
       <c r="D46" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>BE21NA</t>
         </is>
       </c>
       <c r="E46" s="8" t="inlineStr">
@@ -8294,20 +8294,20 @@
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B47" s="8" t="inlineStr">
         <is>
-          <t>Company Pro plan fee</t>
+          <t>bpost parcel</t>
         </is>
       </c>
       <c r="C47" s="9" t="n">
-        <v>-35</v>
+        <v>-5.4</v>
       </c>
       <c r="D47" s="8" t="inlineStr">
         <is>
-          <t>GEEN</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="E47" s="8" t="inlineStr">
@@ -8320,20 +8320,20 @@
     <row r="48">
       <c r="A48" s="8" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B48" s="8" t="inlineStr">
         <is>
-          <t>Action 2009 BE8560 Wevelgem Betaling met Apple Pay</t>
+          <t xml:space="preserve">NENUPHAR BE9051 AFSNEE Betaling met Apple Pay via </t>
         </is>
       </c>
       <c r="C48" s="9" t="n">
-        <v>-10.02</v>
+        <v>-249</v>
       </c>
       <c r="D48" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>BE21NA</t>
         </is>
       </c>
       <c r="E48" s="8" t="inlineStr">
@@ -8346,20 +8346,20 @@
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B49" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">FACEBK *XWUSXWR7A2 IED04 X2K5 Dublin Betaling met </t>
+          <t>HIGGSFIELD INC. US94105 SAN FRANCISCO Betaling met</t>
         </is>
       </c>
       <c r="C49" s="9" t="n">
-        <v>-757.53</v>
+        <v>-72</v>
       </c>
       <c r="D49" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>NONEU</t>
         </is>
       </c>
       <c r="E49" s="8" t="inlineStr">
@@ -8372,20 +8372,20 @@
     <row r="50">
       <c r="A50" s="8" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B50" s="8" t="inlineStr">
         <is>
-          <t>AMBULANTE ZELFSTANDIGEN VZW</t>
+          <t>Findajob bv</t>
         </is>
       </c>
       <c r="C50" s="9" t="n">
-        <v>-230</v>
+        <v>-94.72</v>
       </c>
       <c r="D50" s="8" t="inlineStr">
         <is>
-          <t>NAKIJKEN</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="E50" s="8" t="inlineStr">
@@ -8398,20 +8398,20 @@
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B51" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hotel on Booking.com NL1017 CE AMSTERDAM Betaling </t>
+          <t>SHOPIFY* 576277386</t>
         </is>
       </c>
       <c r="C51" s="9" t="n">
-        <v>-94.25</v>
+        <v>-12.27</v>
       </c>
       <c r="D51" s="8" t="inlineStr">
         <is>
-          <t>GEEN</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E51" s="8" t="inlineStr">
@@ -8424,20 +8424,20 @@
     <row r="52">
       <c r="A52" s="8" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B52" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">FACEBK *F7VQBWM8A2 IED04 X2K5 Dublin Betaling met </t>
+          <t>Findajob bv</t>
         </is>
       </c>
       <c r="C52" s="9" t="n">
-        <v>-800</v>
+        <v>-248.35</v>
       </c>
       <c r="D52" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="E52" s="8" t="inlineStr">
@@ -8450,20 +8450,20 @@
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B53" s="8" t="inlineStr">
         <is>
-          <t>AMBULANTE ZELFSTANDIGEN VZW</t>
+          <t>Advancemedia</t>
         </is>
       </c>
       <c r="C53" s="9" t="n">
-        <v>-230</v>
+        <v>-3650</v>
       </c>
       <c r="D53" s="8" t="inlineStr">
         <is>
-          <t>NAKIJKEN</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E53" s="8" t="inlineStr">
@@ -8476,20 +8476,20 @@
     <row r="54">
       <c r="A54" s="8" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B54" s="8" t="inlineStr">
         <is>
-          <t>SHOPIFY* 571029665</t>
+          <t>Widem Logistics NV</t>
         </is>
       </c>
       <c r="C54" s="9" t="n">
-        <v>-32</v>
+        <v>-1783.71</v>
       </c>
       <c r="D54" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="E54" s="8" t="inlineStr">
@@ -8502,20 +8502,20 @@
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B55" s="8" t="inlineStr">
         <is>
-          <t>KLAVIYO INC. SOFTWARE</t>
+          <t>KBC Verzekeringen</t>
         </is>
       </c>
       <c r="C55" s="9" t="n">
-        <v>-52.94</v>
+        <v>-18.47</v>
       </c>
       <c r="D55" s="8" t="inlineStr">
         <is>
-          <t>NONEU</t>
+          <t>GEEN</t>
         </is>
       </c>
       <c r="E55" s="8" t="inlineStr">
@@ -8528,20 +8528,20 @@
     <row r="56">
       <c r="A56" s="8" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B56" s="8" t="inlineStr">
         <is>
-          <t>Drukbedrijf.nl NL1114AE Amsterdam Betaling met KBC</t>
+          <t>GOOGLE*WORKSPACE SMART IED02 R296 CC GOOGLE.COM Be</t>
         </is>
       </c>
       <c r="C56" s="9" t="n">
-        <v>-174.28</v>
+        <v>-75.90000000000001</v>
       </c>
       <c r="D56" s="8" t="inlineStr">
         <is>
-          <t>NAKIJKEN</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E56" s="8" t="inlineStr">
@@ -8554,20 +8554,20 @@
     <row r="57">
       <c r="A57" s="8" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B57" s="8" t="inlineStr">
         <is>
-          <t>THE SANTIBAL BE8700 TIELT Betaling met KBC-Debetka</t>
+          <t>Yuki Works NV via Mollie</t>
         </is>
       </c>
       <c r="C57" s="9" t="n">
-        <v>-27</v>
+        <v>-2.42</v>
       </c>
       <c r="D57" s="8" t="inlineStr">
         <is>
-          <t>BE21NA</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="E57" s="8" t="inlineStr">
@@ -8580,16 +8580,16 @@
     <row r="58">
       <c r="A58" s="8" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B58" s="8" t="inlineStr">
         <is>
-          <t>FACEBK *JHMLRWM8A2</t>
+          <t>METAPAY*MV4B</t>
         </is>
       </c>
       <c r="C58" s="9" t="n">
-        <v>-800</v>
+        <v>-22.29</v>
       </c>
       <c r="D58" s="8" t="inlineStr">
         <is>
@@ -8606,20 +8606,20 @@
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B59" s="8" t="inlineStr">
         <is>
-          <t>bpost parcel</t>
+          <t>Second part order Furvac 750 pcs</t>
         </is>
       </c>
       <c r="C59" s="9" t="n">
-        <v>-5.4</v>
+        <v>-8637.91</v>
       </c>
       <c r="D59" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>INVOER</t>
         </is>
       </c>
       <c r="E59" s="8" t="inlineStr">
@@ -8632,20 +8632,20 @@
     <row r="60">
       <c r="A60" s="8" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B60" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">FACEBK *TK743YR7A2 IED04 X2K5 DUBLIN Betaling met </t>
+          <t>Company Pro plan fee</t>
         </is>
       </c>
       <c r="C60" s="9" t="n">
-        <v>-800</v>
+        <v>-35</v>
       </c>
       <c r="D60" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>GEEN</t>
         </is>
       </c>
       <c r="E60" s="8" t="inlineStr">
@@ -8658,20 +8658,20 @@
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B61" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">NENUPHAR BE9051 AFSNEE Betaling met Apple Pay via </t>
+          <t>Widem Logistics NV</t>
         </is>
       </c>
       <c r="C61" s="9" t="n">
-        <v>-249</v>
+        <v>-110.77</v>
       </c>
       <c r="D61" s="8" t="inlineStr">
         <is>
-          <t>BE21NA</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="E61" s="8" t="inlineStr">
@@ -8684,20 +8684,20 @@
     <row r="62">
       <c r="A62" s="8" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B62" s="8" t="inlineStr">
         <is>
-          <t>HIGGSFIELD INC. US94105 SAN FRANCISCO Betaling met</t>
+          <t>WIDEM LOGISTICS NV</t>
         </is>
       </c>
       <c r="C62" s="9" t="n">
-        <v>-72</v>
+        <v>-2361.28</v>
       </c>
       <c r="D62" s="8" t="inlineStr">
         <is>
-          <t>NONEU</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="E62" s="8" t="inlineStr">
@@ -8710,7 +8710,7 @@
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B63" s="8" t="inlineStr">
@@ -8719,7 +8719,7 @@
         </is>
       </c>
       <c r="C63" s="9" t="n">
-        <v>-94.72</v>
+        <v>-472.21</v>
       </c>
       <c r="D63" s="8" t="inlineStr">
         <is>
@@ -8736,20 +8736,20 @@
     <row r="64">
       <c r="A64" s="8" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B64" s="8" t="inlineStr">
         <is>
-          <t>SHOPIFY* 576277386</t>
+          <t>Widem Logistics NV</t>
         </is>
       </c>
       <c r="C64" s="9" t="n">
-        <v>-12.27</v>
+        <v>-3135</v>
       </c>
       <c r="D64" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="E64" s="8" t="inlineStr">
@@ -8762,20 +8762,20 @@
     <row r="65">
       <c r="A65" s="8" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B65" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">FACEBK *32NABX98A2 IED04 X2K5 Dublin Betaling met </t>
+          <t>Widem Logistics NV</t>
         </is>
       </c>
       <c r="C65" s="9" t="n">
-        <v>-800</v>
+        <v>-261.03</v>
       </c>
       <c r="D65" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="E65" s="8" t="inlineStr">
@@ -8788,20 +8788,20 @@
     <row r="66">
       <c r="A66" s="8" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B66" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">FACEBK *5F9L8Y58A2 IED04 X2K5 Dublin Betaling met </t>
+          <t>Widem Logistics NV</t>
         </is>
       </c>
       <c r="C66" s="9" t="n">
-        <v>-800</v>
+        <v>-364.57</v>
       </c>
       <c r="D66" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="E66" s="8" t="inlineStr">
@@ -8814,20 +8814,20 @@
     <row r="67">
       <c r="A67" s="8" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B67" s="8" t="inlineStr">
         <is>
-          <t>Findajob bv</t>
+          <t>HOLO AI</t>
         </is>
       </c>
       <c r="C67" s="9" t="n">
-        <v>-248.35</v>
+        <v>-41.33</v>
       </c>
       <c r="D67" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E67" s="8" t="inlineStr">
@@ -8840,16 +8840,16 @@
     <row r="68">
       <c r="A68" s="8" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B68" s="8" t="inlineStr">
         <is>
-          <t>Advancemedia</t>
+          <t>SHOPIFY* 586058249</t>
         </is>
       </c>
       <c r="C68" s="9" t="n">
-        <v>-3650</v>
+        <v>-136.02</v>
       </c>
       <c r="D68" s="8" t="inlineStr">
         <is>
@@ -8866,20 +8866,20 @@
     <row r="69">
       <c r="A69" s="8" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B69" s="8" t="inlineStr">
         <is>
-          <t>Widem Logistics NV</t>
+          <t>KLAVIYO INC. SOFTWARE</t>
         </is>
       </c>
       <c r="C69" s="9" t="n">
-        <v>-1783.71</v>
+        <v>-61.21</v>
       </c>
       <c r="D69" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>NONEU</t>
         </is>
       </c>
       <c r="E69" s="8" t="inlineStr">
@@ -8892,20 +8892,20 @@
     <row r="70">
       <c r="A70" s="8" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B70" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">FACEBK *J93Z3Y98A2 IED04 X2K5 Dublin Betaling met </t>
+          <t>Haddok BE9000 Gent, Belg Betaling met KBC-Debetkaa</t>
         </is>
       </c>
       <c r="C70" s="9" t="n">
-        <v>-800</v>
+        <v>-121.5</v>
       </c>
       <c r="D70" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>BE21NA</t>
         </is>
       </c>
       <c r="E70" s="8" t="inlineStr">
@@ -8918,20 +8918,20 @@
     <row r="71">
       <c r="A71" s="8" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B71" s="8" t="inlineStr">
         <is>
-          <t>KBC Verzekeringen</t>
+          <t xml:space="preserve">PAY*PATRON BE9000 GENT Betaling met Apple Pay via </t>
         </is>
       </c>
       <c r="C71" s="9" t="n">
-        <v>-18.47</v>
+        <v>-8.1</v>
       </c>
       <c r="D71" s="8" t="inlineStr">
         <is>
-          <t>GEEN</t>
+          <t>BE21NA</t>
         </is>
       </c>
       <c r="E71" s="8" t="inlineStr">
@@ -8944,20 +8944,20 @@
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B72" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">FACEBK *QHUESYM7A2 IED04 X2K5 Dublin Betaling met </t>
+          <t>POM-OostV Bedrijven BE9000 Gent Betaling met KBC-D</t>
         </is>
       </c>
       <c r="C72" s="9" t="n">
-        <v>-800</v>
+        <v>-148</v>
       </c>
       <c r="D72" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>NAKIJKEN</t>
         </is>
       </c>
       <c r="E72" s="8" t="inlineStr">
@@ -8970,20 +8970,20 @@
     <row r="73">
       <c r="A73" s="8" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B73" s="8" t="inlineStr">
         <is>
-          <t>GOOGLE*WORKSPACE SMART IED02 R296 CC GOOGLE.COM Be</t>
+          <t>HIGGSFIELD INC. US94105 SAN FRANCISCO Betaling met</t>
         </is>
       </c>
       <c r="C73" s="9" t="n">
-        <v>-75.90000000000001</v>
+        <v>-72</v>
       </c>
       <c r="D73" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>NONEU</t>
         </is>
       </c>
       <c r="E73" s="8" t="inlineStr">
@@ -8996,20 +8996,20 @@
     <row r="74">
       <c r="A74" s="8" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B74" s="8" t="inlineStr">
         <is>
-          <t>Yuki Works NV via Mollie</t>
+          <t>KBC Verzekeringen</t>
         </is>
       </c>
       <c r="C74" s="9" t="n">
-        <v>-2.42</v>
+        <v>-18.47</v>
       </c>
       <c r="D74" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>GEEN</t>
         </is>
       </c>
       <c r="E74" s="8" t="inlineStr">
@@ -9022,20 +9022,20 @@
     <row r="75">
       <c r="A75" s="8" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B75" s="8" t="inlineStr">
         <is>
-          <t>METAPAY*MV4B</t>
+          <t>Findajob bv</t>
         </is>
       </c>
       <c r="C75" s="9" t="n">
-        <v>-22.29</v>
+        <v>-218.55</v>
       </c>
       <c r="D75" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="E75" s="8" t="inlineStr">
@@ -9048,20 +9048,20 @@
     <row r="76">
       <c r="A76" s="8" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B76" s="8" t="inlineStr">
         <is>
-          <t>Second part order Furvac 750 pcs</t>
+          <t>Findajob bv</t>
         </is>
       </c>
       <c r="C76" s="9" t="n">
-        <v>-8637.91</v>
+        <v>-437.1</v>
       </c>
       <c r="D76" s="8" t="inlineStr">
         <is>
-          <t>INVOER</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="E76" s="8" t="inlineStr">
@@ -9074,20 +9074,20 @@
     <row r="77">
       <c r="A77" s="8" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B77" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">FACEBK *7RKG93W7A4 IED04 X2K5 Dublin Betaling met </t>
+          <t>Pro-Count</t>
         </is>
       </c>
       <c r="C77" s="9" t="n">
-        <v>-800</v>
+        <v>-242</v>
       </c>
       <c r="D77" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="E77" s="8" t="inlineStr">
@@ -9100,20 +9100,20 @@
     <row r="78">
       <c r="A78" s="8" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B78" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">FACEBK *45UMKZM8A2 IED04 X2K5 Dublin Betaling met </t>
+          <t>bpost</t>
         </is>
       </c>
       <c r="C78" s="9" t="n">
-        <v>-800</v>
+        <v>-6.78</v>
       </c>
       <c r="D78" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="E78" s="8" t="inlineStr">
@@ -9126,20 +9126,20 @@
     <row r="79">
       <c r="A79" s="8" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B79" s="8" t="inlineStr">
         <is>
-          <t>Company Pro plan fee</t>
+          <t>Widem Logistics NV</t>
         </is>
       </c>
       <c r="C79" s="9" t="n">
-        <v>-35</v>
+        <v>-3251.79</v>
       </c>
       <c r="D79" s="8" t="inlineStr">
         <is>
-          <t>GEEN</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="E79" s="8" t="inlineStr">
@@ -9152,16 +9152,16 @@
     <row r="80">
       <c r="A80" s="8" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B80" s="8" t="inlineStr">
         <is>
-          <t>Widem Logistics NV</t>
+          <t>Findajob bv</t>
         </is>
       </c>
       <c r="C80" s="9" t="n">
-        <v>-110.77</v>
+        <v>-238.42</v>
       </c>
       <c r="D80" s="8" t="inlineStr">
         <is>
@@ -9178,146 +9178,166 @@
     <row r="81">
       <c r="A81" s="8" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B81" s="8" t="inlineStr">
         <is>
-          <t>WIDEM LOGISTICS NV</t>
+          <t xml:space="preserve">FACEBK *X87X6SV7A2 IED04 X2K5 Dublin Betaling met </t>
         </is>
       </c>
       <c r="C81" s="9" t="n">
-        <v>-2361.28</v>
+        <v>-800</v>
       </c>
       <c r="D81" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E81" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F81" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F81" s="8" t="inlineStr">
+        <is>
+          <t>Meta-kwitantie 27253725940979469-27253726004312796 (2026-07-01) – in Lucy/Yuki</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="8" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B82" s="8" t="inlineStr">
         <is>
-          <t>Findajob bv</t>
+          <t xml:space="preserve">FACEBK *W9EF8UH8A2 IED04 X2K5 Dublin Betaling met </t>
         </is>
       </c>
       <c r="C82" s="9" t="n">
-        <v>-472.21</v>
+        <v>-800</v>
       </c>
       <c r="D82" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E82" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F82" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F82" s="8" t="inlineStr">
+        <is>
+          <t>Meta-kwitantie 27355189934166399-27530401703311892 (2026-07-06) – in Lucy/Yuki</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="8" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B83" s="8" t="inlineStr">
         <is>
-          <t>Widem Logistics NV</t>
+          <t xml:space="preserve">FACEBK *RQQRHTR7A2 IED04 X2K5 Dublin Betaling met </t>
         </is>
       </c>
       <c r="C83" s="9" t="n">
-        <v>-3135</v>
+        <v>-278.57</v>
       </c>
       <c r="D83" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E83" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F83" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F83" s="8" t="inlineStr">
+        <is>
+          <t>Meta-kwitantie 27328965953455467-27376759048676154 (2026-07-08) – in Lucy/Yuki</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="8" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B84" s="8" t="inlineStr">
         <is>
-          <t>Widem Logistics NV</t>
+          <t xml:space="preserve">FACEBK *AF4S7TM7A2 IED04 X2K5 Dublin Betaling met </t>
         </is>
       </c>
       <c r="C84" s="9" t="n">
-        <v>-261.03</v>
+        <v>-800</v>
       </c>
       <c r="D84" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E84" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F84" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F84" s="8" t="inlineStr">
+        <is>
+          <t>Meta-kwitantie 27593360840349303-27416226398062750 (2026-07-13) – in Lucy/Yuki</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="8" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B85" s="8" t="inlineStr">
         <is>
-          <t>Widem Logistics NV</t>
+          <t xml:space="preserve">FACEBK *G99QSTM8A2 IED04 X2K5 Dublin Betaling met </t>
         </is>
       </c>
       <c r="C85" s="9" t="n">
-        <v>-364.57</v>
+        <v>-800</v>
       </c>
       <c r="D85" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E85" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F85" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F85" s="8" t="inlineStr">
+        <is>
+          <t>Meta-kwitantie 27669559296062797-27482434021441995 (2026-07-19) – in Lucy/Yuki</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="8" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B86" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">FACEBK *L3G8L3A8A4 IED04 X2K5 Dublin Betaling met </t>
+          <t xml:space="preserve">FACEBK *25EEEVR7A2 IED04 X2K5 Dublin Betaling met </t>
         </is>
       </c>
       <c r="C86" s="9" t="n">
-        <v>-555.08</v>
+        <v>-800</v>
       </c>
       <c r="D86" s="8" t="inlineStr">
         <is>
@@ -9326,24 +9346,28 @@
       </c>
       <c r="E86" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F86" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F86" s="8" t="inlineStr">
+        <is>
+          <t>Meta-kwitantie 27560767960275267-27538964052455655 (2026-07-25) – in Lucy/Yuki</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="8" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B87" s="8" t="inlineStr">
         <is>
-          <t>HOLO AI</t>
+          <t xml:space="preserve">FACEBK *Y2RWNU98A2 IED04 X2K5 Dublin Betaling met </t>
         </is>
       </c>
       <c r="C87" s="9" t="n">
-        <v>-41.33</v>
+        <v>-800</v>
       </c>
       <c r="D87" s="8" t="inlineStr">
         <is>
@@ -9352,24 +9376,28 @@
       </c>
       <c r="E87" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F87" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F87" s="8" t="inlineStr">
+        <is>
+          <t>Meta-kwitantie 27610339325318122-27705458205806234 (2026-07-29) – in Lucy/Yuki</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="8" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B88" s="8" t="inlineStr">
         <is>
-          <t>SHOPIFY* 586058249</t>
+          <t xml:space="preserve">FACEBK *CTEE3XH8A2 IED04 X2K5 Dublin Betaling met </t>
         </is>
       </c>
       <c r="C88" s="9" t="n">
-        <v>-136.02</v>
+        <v>-800</v>
       </c>
       <c r="D88" s="8" t="inlineStr">
         <is>
@@ -9378,20 +9406,24 @@
       </c>
       <c r="E88" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F88" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F88" s="8" t="inlineStr">
+        <is>
+          <t>Meta-kwitantie 27848362231515836-27831764456508946 (2026-08-01) – in Lucy/Yuki</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="8" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B89" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">FACEBK *FZ5UX3A8A4 IED04 X2K5 DUBLIN Betaling met </t>
+          <t xml:space="preserve">FACEBK *LWJTNVM7A2 IED04 X2K5 Dublin Betaling met </t>
         </is>
       </c>
       <c r="C89" s="9" t="n">
@@ -9404,72 +9436,84 @@
       </c>
       <c r="E89" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F89" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F89" s="8" t="inlineStr">
+        <is>
+          <t>Meta-kwitantie 27711775655174490-27869145762770808 (2026-08-04) – in Lucy/Yuki</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="8" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B90" s="8" t="inlineStr">
         <is>
-          <t>KLAVIYO INC. SOFTWARE</t>
+          <t xml:space="preserve">FACEBK *XWUSXWR7A2 IED04 X2K5 Dublin Betaling met </t>
         </is>
       </c>
       <c r="C90" s="9" t="n">
-        <v>-61.21</v>
+        <v>-757.53</v>
       </c>
       <c r="D90" s="8" t="inlineStr">
         <is>
-          <t>NONEU</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E90" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F90" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F90" s="8" t="inlineStr">
+        <is>
+          <t>Meta-kwitantie 27916096561409061-27967802372905150 (2026-08-08) – in Lucy/Yuki</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="8" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B91" s="8" t="inlineStr">
         <is>
-          <t>Haddok BE9000 Gent, Belg Betaling met KBC-Debetkaa</t>
+          <t xml:space="preserve">FACEBK *F7VQBWM8A2 IED04 X2K5 Dublin Betaling met </t>
         </is>
       </c>
       <c r="C91" s="9" t="n">
-        <v>-121.5</v>
+        <v>-800</v>
       </c>
       <c r="D91" s="8" t="inlineStr">
         <is>
-          <t>BE21NA</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E91" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F91" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F91" s="8" t="inlineStr">
+        <is>
+          <t>Meta-kwitantie 28001385692880151-27949550744730309 (2026-08-10) – in Lucy/Yuki</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="8" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B92" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">FACEBK *EY2TK3N7A4 IED04 X2K5 DUBLIN Betaling met </t>
+          <t>FACEBK *JHMLRWM8A2</t>
         </is>
       </c>
       <c r="C92" s="9" t="n">
@@ -9482,20 +9526,24 @@
       </c>
       <c r="E92" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F92" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F92" s="8" t="inlineStr">
+        <is>
+          <t>Meta-kwitantie 27840792075606180-27840792262272828 (2026-08-14) – in Lucy/Yuki</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="8" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="B93" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">FACEBK *52WHD3S7A4 IED04 X2K5 DUBLIN Betaling met </t>
+          <t xml:space="preserve">FACEBK *TK743YR7A2 IED04 X2K5 DUBLIN Betaling met </t>
         </is>
       </c>
       <c r="C93" s="9" t="n">
@@ -9508,98 +9556,114 @@
       </c>
       <c r="E93" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F93" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F93" s="8" t="inlineStr">
+        <is>
+          <t>Meta-kwitantie 28061581953527195-27855281750823885 (2026-08-17) – in Lucy/Yuki</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="8" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B94" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">PAY*PATRON BE9000 GENT Betaling met Apple Pay via </t>
+          <t xml:space="preserve">FACEBK *32NABX98A2 IED04 X2K5 Dublin Betaling met </t>
         </is>
       </c>
       <c r="C94" s="9" t="n">
-        <v>-8.1</v>
+        <v>-800</v>
       </c>
       <c r="D94" s="8" t="inlineStr">
         <is>
-          <t>BE21NA</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E94" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F94" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F94" s="8" t="inlineStr">
+        <is>
+          <t>Meta-kwitantie 28134158839602835-28081838734834842 (2026-08-20) – in Lucy/Yuki</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="8" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B95" s="8" t="inlineStr">
         <is>
-          <t>POM-OostV Bedrijven BE9000 Gent Betaling met KBC-D</t>
+          <t xml:space="preserve">FACEBK *5F9L8Y58A2 IED04 X2K5 Dublin Betaling met </t>
         </is>
       </c>
       <c r="C95" s="9" t="n">
-        <v>-148</v>
+        <v>-800</v>
       </c>
       <c r="D95" s="8" t="inlineStr">
         <is>
-          <t>NAKIJKEN</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E95" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F95" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F95" s="8" t="inlineStr">
+        <is>
+          <t>Meta-kwitantie 27978323681853020-27946942661657785 (2026-08-23) – in Lucy/Yuki</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="8" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B96" s="8" t="inlineStr">
         <is>
-          <t>HIGGSFIELD INC. US94105 SAN FRANCISCO Betaling met</t>
+          <t xml:space="preserve">FACEBK *J93Z3Y98A2 IED04 X2K5 Dublin Betaling met </t>
         </is>
       </c>
       <c r="C96" s="9" t="n">
-        <v>-72</v>
+        <v>-800</v>
       </c>
       <c r="D96" s="8" t="inlineStr">
         <is>
-          <t>NONEU</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E96" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F96" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F96" s="8" t="inlineStr">
+        <is>
+          <t>Meta-kwitantie 28174602315558490-28023493624002692 (2026-08-26) – in Lucy/Yuki</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="8" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B97" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">FACEBK *VRFKQ5W7A4 IED04 X2K5 DUBLIN Betaling met </t>
+          <t xml:space="preserve">FACEBK *QHUESYM7A2 IED04 X2K5 Dublin Betaling met </t>
         </is>
       </c>
       <c r="C97" s="9" t="n">
@@ -9612,20 +9676,24 @@
       </c>
       <c r="E97" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F97" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F97" s="8" t="inlineStr">
+        <is>
+          <t>Meta-kwitantie 28241109438907778-28269737452711639 (2026-08-30) – in Lucy/Yuki</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="8" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B98" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">FACEBK *QFMU25N7A4 IED04 X2K5 DUBLIN Betaling met </t>
+          <t xml:space="preserve">FACEBK *7RKG93W7A4 IED04 X2K5 Dublin Betaling met </t>
         </is>
       </c>
       <c r="C98" s="9" t="n">
@@ -9638,20 +9706,24 @@
       </c>
       <c r="E98" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F98" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F98" s="8" t="inlineStr">
+        <is>
+          <t>Meta-kwitantie 28057913993893989-28264454399906607 (2026-09-02) – in Lucy/Yuki</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="8" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B99" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">FACEBK *ZDGTF5N7A4 IED04 X2K5 DUBLIN Betaling met </t>
+          <t xml:space="preserve">FACEBK *45UMKZM8A2 IED04 X2K5 Dublin Betaling met </t>
         </is>
       </c>
       <c r="C99" s="9" t="n">
@@ -9664,192 +9736,224 @@
       </c>
       <c r="E99" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F99" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F99" s="8" t="inlineStr">
+        <is>
+          <t>Meta-kwitantie 28135330259485690-28135330349485681 (2026-09-05) – in Lucy/Yuki</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="8" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B100" s="8" t="inlineStr">
         <is>
-          <t>KBC Verzekeringen</t>
+          <t xml:space="preserve">FACEBK *L3G8L3A8A4 IED04 X2K5 Dublin Betaling met </t>
         </is>
       </c>
       <c r="C100" s="9" t="n">
-        <v>-18.47</v>
+        <v>-555.08</v>
       </c>
       <c r="D100" s="8" t="inlineStr">
         <is>
-          <t>GEEN</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E100" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F100" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F100" s="8" t="inlineStr">
+        <is>
+          <t>Meta-kwitantie 28354522874233099-28372066432478744 (2026-09-08) – in Lucy/Yuki</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="8" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B101" s="8" t="inlineStr">
         <is>
-          <t>Findajob bv</t>
+          <t xml:space="preserve">FACEBK *FZ5UX3A8A4 IED04 X2K5 DUBLIN Betaling met </t>
         </is>
       </c>
       <c r="C101" s="9" t="n">
-        <v>-218.55</v>
+        <v>-800</v>
       </c>
       <c r="D101" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E101" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F101" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F101" s="8" t="inlineStr">
+        <is>
+          <t>Meta-kwitantie 28388089664209746-28211277685224280 (2026-09-10) – in Lucy/Yuki</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="8" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B102" s="8" t="inlineStr">
         <is>
-          <t>Findajob bv</t>
+          <t xml:space="preserve">FACEBK *EY2TK3N7A4 IED04 X2K5 DUBLIN Betaling met </t>
         </is>
       </c>
       <c r="C102" s="9" t="n">
-        <v>-437.1</v>
+        <v>-800</v>
       </c>
       <c r="D102" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E102" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F102" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F102" s="8" t="inlineStr">
+        <is>
+          <t>Meta-kwitantie 28254286180923430-28254286254256756 (2026-09-13) – in Lucy/Yuki</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="8" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B103" s="8" t="inlineStr">
         <is>
-          <t>Pro-Count</t>
+          <t xml:space="preserve">FACEBK *52WHD3S7A4 IED04 X2K5 DUBLIN Betaling met </t>
         </is>
       </c>
       <c r="C103" s="9" t="n">
-        <v>-242</v>
+        <v>-800</v>
       </c>
       <c r="D103" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F103" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F103" s="8" t="inlineStr">
+        <is>
+          <t>Meta-kwitantie 28488005980884780-28343182888700429 (2026-09-17) – in Lucy/Yuki</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="8" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B104" s="8" t="inlineStr">
         <is>
-          <t>bpost</t>
+          <t xml:space="preserve">FACEBK *VRFKQ5W7A4 IED04 X2K5 DUBLIN Betaling met </t>
         </is>
       </c>
       <c r="C104" s="9" t="n">
-        <v>-6.78</v>
+        <v>-800</v>
       </c>
       <c r="D104" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F104" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F104" s="8" t="inlineStr">
+        <is>
+          <t>Meta-kwitantie 28548539494831435-28333791032972949 (2026-09-20) – in Lucy/Yuki</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="8" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="B105" s="8" t="inlineStr">
         <is>
-          <t>Widem Logistics NV</t>
+          <t xml:space="preserve">FACEBK *QFMU25N7A4 IED04 X2K5 DUBLIN Betaling met </t>
         </is>
       </c>
       <c r="C105" s="9" t="n">
-        <v>-3251.79</v>
+        <v>-800</v>
       </c>
       <c r="D105" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E105" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F105" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F105" s="8" t="inlineStr">
+        <is>
+          <t>Meta-kwitantie 28412552321763489-28417867054565341 (2026-09-24) – in Lucy/Yuki</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="8" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B106" s="8" t="inlineStr">
         <is>
-          <t>Findajob bv</t>
+          <t xml:space="preserve">FACEBK *ZDGTF5N7A4 IED04 X2K5 DUBLIN Betaling met </t>
         </is>
       </c>
       <c r="C106" s="9" t="n">
-        <v>-238.42</v>
+        <v>-800</v>
       </c>
       <c r="D106" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E106" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F106" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F106" s="8" t="inlineStr">
+        <is>
+          <t>Meta-kwitantie 28496207413397975-28665230016495716 (2026-09-27) – in Lucy/Yuki</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="8" t="inlineStr">
@@ -9872,10 +9976,14 @@
       </c>
       <c r="E107" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F107" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F107" s="8" t="inlineStr">
+        <is>
+          <t>Meta-kwitantie 28690004364018280-28524841167201264 (2026-09-30) – in Lucy/Yuki</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Ochtendcheck 27/10: Jess-voorschot gekoppeld, boek Q4 en rapporten bijgewerkt
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WLjvFbtqAZDvUMthyPjkEk
</commit_message>
<xml_diff>
--- a/boekhouding/rapporten/SmartPaw_Q3-2026.xlsx
+++ b/boekhouding/rapporten/SmartPaw_Q3-2026.xlsx
@@ -7099,7 +7099,7 @@
         </is>
       </c>
       <c r="C6" s="9" t="n">
-        <v>-0</v>
+        <v>-27.86</v>
       </c>
       <c r="D6" s="9" t="n">
         <v>10610.49</v>
@@ -7108,7 +7108,7 @@
         <v>-10040.65</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>569.84</v>
+        <v>541.98</v>
       </c>
       <c r="G6" s="8" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Aankoopdagboek na ruimere Yuki-ophaling (Widem 26012021 in Yuki)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WLjvFcZoD9WegLqrYozzyo
</commit_message>
<xml_diff>
--- a/boekhouding/rapporten/SmartPaw_Q3-2026.xlsx
+++ b/boekhouding/rapporten/SmartPaw_Q3-2026.xlsx
@@ -589,7 +589,7 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="14">
@@ -6749,7 +6749,7 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>Aankoopdagboek Q3 2026: 11 te boeken, 73 al in Yuki (ter controle), 17 zonder factuur. Grootboekrekeningen volgens jullie rekeningschema; btw-codes: eigen code + roosters.</t>
+          <t>Aankoopdagboek Q3 2026: 10 te boeken, 74 al in Yuki (ter controle), 17 zonder factuur. Grootboekrekeningen volgens jullie rekeningschema; btw-codes: eigen code + roosters.</t>
         </is>
       </c>
     </row>
@@ -6923,70 +6923,70 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>Widem Logistics NV</t>
+          <t>UAB Holo LT (Vilnius, LT)</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr"/>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>26012021</t>
+          <t>HOLO-202607-E80C0</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>612730</t>
+          <t>611080</t>
         </is>
       </c>
       <c r="G5" s="8" t="inlineStr">
         <is>
-          <t>TRANSPORTEN AAN DERDEN</t>
+          <t>ABONNEMENTEN</t>
         </is>
       </c>
       <c r="H5" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>EUDV</t>
         </is>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
-          <t>82 · 59</t>
+          <t>88 · 55 · 59</t>
         </is>
       </c>
       <c r="J5" s="9" t="n">
-        <v>2590.91</v>
+        <v>41.98</v>
       </c>
       <c r="K5" s="9" t="n">
-        <v>544.09</v>
+        <v>0</v>
       </c>
       <c r="L5" s="9" t="n">
-        <v>0</v>
+        <v>8.82</v>
       </c>
       <c r="M5" s="9" t="n">
-        <v>3135</v>
+        <v>41.98</v>
       </c>
       <c r="N5" s="8" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="O5" s="8" t="inlineStr">
         <is>
-          <t>550000 KBC zichtrekening</t>
+          <t>434000 Mastercard Henri (6682)</t>
         </is>
       </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
-          <t>Widem 26012021 (mail 2026-07-07)</t>
+          <t>2026-07-08_HoloAI_47.19USD.pdf</t>
         </is>
       </c>
       <c r="Q5" s="8" t="inlineStr">
         <is>
-          <t>Yuki: 21%</t>
+          <t>Yuki: intracommunautair diensten (verlegd)</t>
         </is>
       </c>
     </row>
@@ -6998,70 +6998,70 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>UAB Holo LT (Vilnius, LT)</t>
+          <t>KBC Verzekeringen (polis 37630975, BA bedrijfspolis aansprakelijkheid)</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr"/>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>HOLO-202607-E80C0</t>
+          <t>37630975</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>611080</t>
+          <t>613210</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>ABONNEMENTEN</t>
+          <t>BURGERLIJKE AANSPRAKELIJKHEID</t>
         </is>
       </c>
       <c r="H6" s="8" t="inlineStr">
         <is>
-          <t>EUDV</t>
+          <t>GEEN</t>
         </is>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
-          <t>88 · 55 · 59</t>
+          <t>82</t>
         </is>
       </c>
       <c r="J6" s="9" t="n">
-        <v>41.98</v>
+        <v>18.47</v>
       </c>
       <c r="K6" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L6" s="9" t="n">
-        <v>8.82</v>
+        <v>0</v>
       </c>
       <c r="M6" s="9" t="n">
-        <v>41.98</v>
+        <v>18.47</v>
       </c>
       <c r="N6" s="8" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="O6" s="8" t="inlineStr">
         <is>
-          <t>434000 Mastercard Henri (6682)</t>
+          <t>550000 KBC zichtrekening</t>
         </is>
       </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
-          <t>2026-07-08_HoloAI_47.19USD.pdf</t>
+          <t>KBC_BA-polis_37630975_2026-08-27.pdf</t>
         </is>
       </c>
       <c r="Q6" s="8" t="inlineStr">
         <is>
-          <t>Yuki: intracommunautair diensten (verlegd)</t>
+          <t>Yuki: geen btw / vrijgesteld</t>
         </is>
       </c>
     </row>
@@ -7078,65 +7078,65 @@
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>KBC Verzekeringen (polis 37630975, BA bedrijfspolis aansprakelijkheid)</t>
+          <t>Klaviyo Inc</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr"/>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>37630975</t>
+          <t>T9T7QHZO-0012</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>613210</t>
+          <t>611080</t>
         </is>
       </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>BURGERLIJKE AANSPRAKELIJKHEID</t>
+          <t>ABONNEMENTEN</t>
         </is>
       </c>
       <c r="H7" s="8" t="inlineStr">
         <is>
-          <t>GEEN</t>
+          <t>NEUDV</t>
         </is>
       </c>
       <c r="I7" s="8" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>87 · 56 · 59</t>
         </is>
       </c>
       <c r="J7" s="9" t="n">
-        <v>18.47</v>
+        <v>53.5</v>
       </c>
       <c r="K7" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L7" s="9" t="n">
-        <v>0</v>
+        <v>11.23</v>
       </c>
       <c r="M7" s="9" t="n">
-        <v>18.47</v>
+        <v>53.5</v>
       </c>
       <c r="N7" s="8" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="O7" s="8" t="inlineStr">
         <is>
-          <t>550000 KBC zichtrekening</t>
+          <t>434000 Mastercard Henri (6682)</t>
         </is>
       </c>
       <c r="P7" s="8" t="inlineStr">
         <is>
-          <t>KBC_BA-polis_37630975_2026-08-27.pdf</t>
+          <t>Klaviyo T9T7QHZO-0012 (mail 2026-07-10)</t>
         </is>
       </c>
       <c r="Q7" s="8" t="inlineStr">
         <is>
-          <t>Yuki: geen btw / vrijgesteld</t>
+          <t>Yuki: btw verlegd (dienst buiten EU)</t>
         </is>
       </c>
     </row>
@@ -7148,55 +7148,55 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>Klaviyo Inc</t>
+          <t>Packaging Discounter B.V.</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr"/>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>T9T7QHZO-0012</t>
+          <t>28109678</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>611080</t>
+          <t>601000</t>
         </is>
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t>ABONNEMENTEN</t>
+          <t>Aankopen van hulpstoffen</t>
         </is>
       </c>
       <c r="H8" s="8" t="inlineStr">
         <is>
-          <t>NEUDV</t>
+          <t>EUG</t>
         </is>
       </c>
       <c r="I8" s="8" t="inlineStr">
         <is>
-          <t>87 · 56 · 59</t>
+          <t>86 · 55 · 59</t>
         </is>
       </c>
       <c r="J8" s="9" t="n">
-        <v>53.5</v>
+        <v>665</v>
       </c>
       <c r="K8" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L8" s="9" t="n">
-        <v>11.23</v>
+        <v>139.65</v>
       </c>
       <c r="M8" s="9" t="n">
-        <v>53.5</v>
+        <v>665</v>
       </c>
       <c r="N8" s="8" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="O8" s="8" t="inlineStr">
@@ -7206,12 +7206,12 @@
       </c>
       <c r="P8" s="8" t="inlineStr">
         <is>
-          <t>Klaviyo T9T7QHZO-0012 (mail 2026-07-10)</t>
+          <t>Packaging Discounter 28109678 (mail 2026-07-20)</t>
         </is>
       </c>
       <c r="Q8" s="8" t="inlineStr">
         <is>
-          <t>Yuki: btw verlegd (dienst buiten EU)</t>
+          <t>NAKIJKEN: Yuki: intracommunautair goederen, als de factuur btw verlegd vermeldt; anders buitenlandse btw, niet aftrekbaar</t>
         </is>
       </c>
     </row>
@@ -7223,70 +7223,70 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>Packaging Discounter B.V.</t>
+          <t>KBC Verzekeringen (polis 37630975, BA bedrijfspolis aansprakelijkheid)</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr"/>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>28109678</t>
+          <t>37630975</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>601000</t>
+          <t>613210</t>
         </is>
       </c>
       <c r="G9" s="8" t="inlineStr">
         <is>
-          <t>Aankopen van hulpstoffen</t>
+          <t>BURGERLIJKE AANSPRAKELIJKHEID</t>
         </is>
       </c>
       <c r="H9" s="8" t="inlineStr">
         <is>
-          <t>EUG</t>
+          <t>GEEN</t>
         </is>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
-          <t>86 · 55 · 59</t>
+          <t>82</t>
         </is>
       </c>
       <c r="J9" s="9" t="n">
-        <v>665</v>
+        <v>18.47</v>
       </c>
       <c r="K9" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L9" s="9" t="n">
-        <v>139.65</v>
+        <v>0</v>
       </c>
       <c r="M9" s="9" t="n">
-        <v>665</v>
+        <v>18.47</v>
       </c>
       <c r="N9" s="8" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="O9" s="8" t="inlineStr">
         <is>
-          <t>434000 Mastercard Henri (6682)</t>
+          <t>550000 KBC zichtrekening</t>
         </is>
       </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
-          <t>Packaging Discounter 28109678 (mail 2026-07-20)</t>
+          <t>KBC_BA-polis_37630975_2026-09-27.pdf</t>
         </is>
       </c>
       <c r="Q9" s="8" t="inlineStr">
         <is>
-          <t>NAKIJKEN: Yuki: intracommunautair goederen, als de factuur btw verlegd vermeldt; anders buitenlandse btw, niet aftrekbaar</t>
+          <t>Yuki: geen btw / vrijgesteld</t>
         </is>
       </c>
     </row>
@@ -7303,65 +7303,65 @@
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>KBC Verzekeringen (polis 37630975, BA bedrijfspolis aansprakelijkheid)</t>
+          <t>Klaviyo Inc</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr"/>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>37630975</t>
+          <t>T9T7QHZO-0013</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>613210</t>
+          <t>611080</t>
         </is>
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
-          <t>BURGERLIJKE AANSPRAKELIJKHEID</t>
+          <t>ABONNEMENTEN</t>
         </is>
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
-          <t>GEEN</t>
+          <t>NEUDV</t>
         </is>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>87 · 56 · 59</t>
         </is>
       </c>
       <c r="J10" s="9" t="n">
-        <v>18.47</v>
+        <v>52.94</v>
       </c>
       <c r="K10" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L10" s="9" t="n">
-        <v>0</v>
+        <v>11.12</v>
       </c>
       <c r="M10" s="9" t="n">
-        <v>18.47</v>
+        <v>52.94</v>
       </c>
       <c r="N10" s="8" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="O10" s="8" t="inlineStr">
         <is>
-          <t>550000 KBC zichtrekening</t>
+          <t>434000 Mastercard Henri (6682)</t>
         </is>
       </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
-          <t>KBC_BA-polis_37630975_2026-09-27.pdf</t>
+          <t>Klaviyo T9T7QHZO-0013 (mail 2026-08-10)</t>
         </is>
       </c>
       <c r="Q10" s="8" t="inlineStr">
         <is>
-          <t>Yuki: geen btw / vrijgesteld</t>
+          <t>Yuki: btw verlegd (dienst buiten EU)</t>
         </is>
       </c>
     </row>
@@ -7373,18 +7373,18 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>Klaviyo Inc</t>
+          <t>UAB Holo LT (Vilnius, LT)</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr"/>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>T9T7QHZO-0013</t>
+          <t>HOLO-202609-477F0</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
@@ -7399,29 +7399,29 @@
       </c>
       <c r="H11" s="8" t="inlineStr">
         <is>
-          <t>NEUDV</t>
+          <t>EUDV</t>
         </is>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
-          <t>87 · 56 · 59</t>
+          <t>88 · 55 · 59</t>
         </is>
       </c>
       <c r="J11" s="9" t="n">
-        <v>52.94</v>
+        <v>41.33</v>
       </c>
       <c r="K11" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L11" s="9" t="n">
-        <v>11.12</v>
+        <v>8.68</v>
       </c>
       <c r="M11" s="9" t="n">
-        <v>52.94</v>
+        <v>41.33</v>
       </c>
       <c r="N11" s="8" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="O11" s="8" t="inlineStr">
@@ -7431,12 +7431,12 @@
       </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
-          <t>Klaviyo T9T7QHZO-0013 (mail 2026-08-10)</t>
+          <t>2026-09-08_HoloAI_47.19USD.pdf</t>
         </is>
       </c>
       <c r="Q11" s="8" t="inlineStr">
         <is>
-          <t>Yuki: btw verlegd (dienst buiten EU)</t>
+          <t>Yuki: intracommunautair diensten (verlegd)</t>
         </is>
       </c>
     </row>
@@ -7448,18 +7448,18 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>UAB Holo LT (Vilnius, LT)</t>
+          <t>Klaviyo Inc</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr"/>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>HOLO-202609-477F0</t>
+          <t>T9T7QHZO-0014</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
@@ -7474,29 +7474,29 @@
       </c>
       <c r="H12" s="8" t="inlineStr">
         <is>
-          <t>EUDV</t>
+          <t>NEUDV</t>
         </is>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
-          <t>88 · 55 · 59</t>
+          <t>87 · 56 · 59</t>
         </is>
       </c>
       <c r="J12" s="9" t="n">
-        <v>41.33</v>
+        <v>61.21</v>
       </c>
       <c r="K12" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L12" s="9" t="n">
-        <v>8.68</v>
+        <v>12.85</v>
       </c>
       <c r="M12" s="9" t="n">
-        <v>41.33</v>
+        <v>61.21</v>
       </c>
       <c r="N12" s="8" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="O12" s="8" t="inlineStr">
@@ -7506,12 +7506,12 @@
       </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
-          <t>2026-09-08_HoloAI_47.19USD.pdf</t>
+          <t>Klaviyo T9T7QHZO-0014 (mail 2026-09-10)</t>
         </is>
       </c>
       <c r="Q12" s="8" t="inlineStr">
         <is>
-          <t>Yuki: intracommunautair diensten (verlegd)</t>
+          <t>Yuki: btw verlegd (dienst buiten EU)</t>
         </is>
       </c>
     </row>
@@ -7523,103 +7523,99 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Klaviyo Inc</t>
+          <t>Meta Platforms Ireland</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr"/>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>T9T7QHZO-0014</t>
+          <t>28690004364018280-28524841167201264</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t>611080</t>
+          <t>616502</t>
         </is>
       </c>
       <c r="G13" s="8" t="inlineStr">
         <is>
-          <t>ABONNEMENTEN</t>
+          <t>RECLAME MET MERK</t>
         </is>
       </c>
       <c r="H13" s="8" t="inlineStr">
         <is>
-          <t>NEUDV</t>
+          <t>EUDV</t>
         </is>
       </c>
       <c r="I13" s="8" t="inlineStr">
         <is>
-          <t>87 · 56 · 59</t>
+          <t>88 · 55 · 59</t>
         </is>
       </c>
       <c r="J13" s="9" t="n">
-        <v>61.21</v>
+        <v>800</v>
       </c>
       <c r="K13" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L13" s="9" t="n">
-        <v>12.85</v>
+        <v>168</v>
       </c>
       <c r="M13" s="9" t="n">
-        <v>61.21</v>
+        <v>800</v>
       </c>
       <c r="N13" s="8" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="O13" s="8" t="inlineStr">
         <is>
-          <t>434000 Mastercard Henri (6682)</t>
+          <t>550000 KBC zichtrekening</t>
         </is>
       </c>
       <c r="P13" s="8" t="inlineStr">
         <is>
-          <t>Klaviyo T9T7QHZO-0014 (mail 2026-09-10)</t>
+          <t>Meta-kwitantie 28690004364018280-28524841167201264 (2026-09-30) – in Lucy/Yuki</t>
         </is>
       </c>
       <c r="Q13" s="8" t="inlineStr">
         <is>
-          <t>Yuki: btw verlegd (dienst buiten EU)</t>
+          <t>Yuki: intracommunautair diensten (verlegd)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>te boeken</t>
+          <t>factuur ontbreekt</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Meta Platforms Ireland</t>
+          <t>Google ADS4790542578</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr"/>
-      <c r="E14" s="8" t="inlineStr">
-        <is>
-          <t>28690004364018280-28524841167201264</t>
-        </is>
-      </c>
+      <c r="E14" s="8" t="inlineStr"/>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>616502</t>
+          <t>616501</t>
         </is>
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
-          <t>RECLAME MET MERK</t>
+          <t>RECLAME ZONDER MERK</t>
         </is>
       </c>
       <c r="H14" s="8" t="inlineStr">
@@ -7633,32 +7629,28 @@
         </is>
       </c>
       <c r="J14" s="9" t="n">
-        <v>800</v>
+        <v>158.5</v>
       </c>
       <c r="K14" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L14" s="9" t="n">
-        <v>168</v>
+        <v>33.28</v>
       </c>
       <c r="M14" s="9" t="n">
-        <v>800</v>
+        <v>158.5</v>
       </c>
       <c r="N14" s="8" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="O14" s="8" t="inlineStr">
         <is>
-          <t>550000 KBC zichtrekening</t>
-        </is>
-      </c>
-      <c r="P14" s="8" t="inlineStr">
-        <is>
-          <t>Meta-kwitantie 28690004364018280-28524841167201264 (2026-09-30) – in Lucy/Yuki</t>
-        </is>
-      </c>
+          <t>434001 Mastercard Kaydee (2103)</t>
+        </is>
+      </c>
+      <c r="P14" s="8" t="inlineStr"/>
       <c r="Q14" s="8" t="inlineStr">
         <is>
           <t>Yuki: intracommunautair diensten (verlegd)</t>
@@ -7673,24 +7665,24 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>Google ADS4790542578</t>
+          <t>SHOPIFY* 556521062</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr"/>
       <c r="E15" s="8" t="inlineStr"/>
       <c r="F15" s="8" t="inlineStr">
         <is>
-          <t>616501</t>
+          <t>611080</t>
         </is>
       </c>
       <c r="G15" s="8" t="inlineStr">
         <is>
-          <t>RECLAME ZONDER MERK</t>
+          <t>ABONNEMENTEN</t>
         </is>
       </c>
       <c r="H15" s="8" t="inlineStr">
@@ -7704,25 +7696,25 @@
         </is>
       </c>
       <c r="J15" s="9" t="n">
-        <v>158.5</v>
+        <v>141.39</v>
       </c>
       <c r="K15" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L15" s="9" t="n">
-        <v>33.28</v>
+        <v>29.69</v>
       </c>
       <c r="M15" s="9" t="n">
-        <v>158.5</v>
+        <v>141.39</v>
       </c>
       <c r="N15" s="8" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="O15" s="8" t="inlineStr">
         <is>
-          <t>434001 Mastercard Kaydee (2103)</t>
+          <t>434000 Mastercard Henri (6682)</t>
         </is>
       </c>
       <c r="P15" s="8" t="inlineStr"/>
@@ -7740,24 +7732,24 @@
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>SHOPIFY* 556521062</t>
+          <t>Google ADS4790542578</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr"/>
       <c r="E16" s="8" t="inlineStr"/>
       <c r="F16" s="8" t="inlineStr">
         <is>
-          <t>611080</t>
+          <t>616501</t>
         </is>
       </c>
       <c r="G16" s="8" t="inlineStr">
         <is>
-          <t>ABONNEMENTEN</t>
+          <t>RECLAME ZONDER MERK</t>
         </is>
       </c>
       <c r="H16" s="8" t="inlineStr">
@@ -7771,25 +7763,25 @@
         </is>
       </c>
       <c r="J16" s="9" t="n">
-        <v>141.39</v>
+        <v>500</v>
       </c>
       <c r="K16" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L16" s="9" t="n">
-        <v>29.69</v>
+        <v>105</v>
       </c>
       <c r="M16" s="9" t="n">
-        <v>141.39</v>
+        <v>500</v>
       </c>
       <c r="N16" s="8" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="O16" s="8" t="inlineStr">
         <is>
-          <t>434000 Mastercard Henri (6682)</t>
+          <t>434001 Mastercard Kaydee (2103)</t>
         </is>
       </c>
       <c r="P16" s="8" t="inlineStr"/>
@@ -7807,62 +7799,62 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>Google ADS4790542578</t>
+          <t>SP PACKAGINGDISCOUNTER</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr"/>
       <c r="E17" s="8" t="inlineStr"/>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>616501</t>
+          <t>601000</t>
         </is>
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
-          <t>RECLAME ZONDER MERK</t>
+          <t>Aankopen van hulpstoffen</t>
         </is>
       </c>
       <c r="H17" s="8" t="inlineStr">
         <is>
-          <t>EUDV</t>
+          <t>EUG</t>
         </is>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
-          <t>88 · 55 · 59</t>
+          <t>86 · 55 · 59</t>
         </is>
       </c>
       <c r="J17" s="9" t="n">
-        <v>500</v>
+        <v>360</v>
       </c>
       <c r="K17" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L17" s="9" t="n">
-        <v>105</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="M17" s="9" t="n">
-        <v>500</v>
+        <v>360</v>
       </c>
       <c r="N17" s="8" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="O17" s="8" t="inlineStr">
         <is>
-          <t>434001 Mastercard Kaydee (2103)</t>
+          <t>434000 Mastercard Henri (6682)</t>
         </is>
       </c>
       <c r="P17" s="8" t="inlineStr"/>
       <c r="Q17" s="8" t="inlineStr">
         <is>
-          <t>Yuki: intracommunautair diensten (verlegd)</t>
+          <t>NAKIJKEN: Yuki: intracommunautair goederen, als de factuur btw verlegd vermeldt; anders buitenlandse btw, niet aftrekbaar</t>
         </is>
       </c>
     </row>
@@ -7874,62 +7866,62 @@
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>SP PACKAGINGDISCOUNTER</t>
+          <t>YAKI NOODLE BAR BE9000 GENT Betaling met KBC-Debet</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr"/>
       <c r="E18" s="8" t="inlineStr"/>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>601000</t>
+          <t>616680</t>
         </is>
       </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
-          <t>Aankopen van hulpstoffen</t>
+          <t>Restaurantkosten</t>
         </is>
       </c>
       <c r="H18" s="8" t="inlineStr">
         <is>
-          <t>EUG</t>
+          <t>BE21NA</t>
         </is>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
-          <t>86 · 55 · 59</t>
+          <t>82</t>
         </is>
       </c>
       <c r="J18" s="9" t="n">
-        <v>360</v>
+        <v>15</v>
       </c>
       <c r="K18" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L18" s="9" t="n">
-        <v>75.59999999999999</v>
+        <v>0</v>
       </c>
       <c r="M18" s="9" t="n">
-        <v>360</v>
+        <v>15</v>
       </c>
       <c r="N18" s="8" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="O18" s="8" t="inlineStr">
         <is>
-          <t>434000 Mastercard Henri (6682)</t>
+          <t>550000 KBC zichtrekening</t>
         </is>
       </c>
       <c r="P18" s="8" t="inlineStr"/>
       <c r="Q18" s="8" t="inlineStr">
         <is>
-          <t>NAKIJKEN: Yuki: intracommunautair goederen, als de factuur btw verlegd vermeldt; anders buitenlandse btw, niet aftrekbaar</t>
+          <t>Yuki: 0% aftrek (restaurant)</t>
         </is>
       </c>
     </row>
@@ -7941,38 +7933,38 @@
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>YAKI NOODLE BAR BE9000 GENT Betaling met KBC-Debet</t>
+          <t>AMBULANTE ZELFSTANDIGEN VZW</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr"/>
       <c r="E19" s="8" t="inlineStr"/>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>616680</t>
+          <t>616620</t>
         </is>
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>Restaurantkosten</t>
+          <t>Beurzen en tentoonstellingen</t>
         </is>
       </c>
       <c r="H19" s="8" t="inlineStr">
         <is>
-          <t>BE21NA</t>
+          <t>?</t>
         </is>
       </c>
       <c r="I19" s="8" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>?</t>
         </is>
       </c>
       <c r="J19" s="9" t="n">
-        <v>15</v>
+        <v>210</v>
       </c>
       <c r="K19" s="9" t="n">
         <v>0</v>
@@ -7981,11 +7973,11 @@
         <v>0</v>
       </c>
       <c r="M19" s="9" t="n">
-        <v>15</v>
+        <v>210</v>
       </c>
       <c r="N19" s="8" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="O19" s="8" t="inlineStr">
@@ -7996,7 +7988,7 @@
       <c r="P19" s="8" t="inlineStr"/>
       <c r="Q19" s="8" t="inlineStr">
         <is>
-          <t>Yuki: 0% aftrek (restaurant)</t>
+          <t>NAKIJKEN: btw-behandeling nakijken</t>
         </is>
       </c>
     </row>
@@ -8008,62 +8000,62 @@
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>AMBULANTE ZELFSTANDIGEN VZW</t>
+          <t>Google ADS4790542578</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr"/>
       <c r="E20" s="8" t="inlineStr"/>
       <c r="F20" s="8" t="inlineStr">
         <is>
-          <t>616620</t>
+          <t>616501</t>
         </is>
       </c>
       <c r="G20" s="8" t="inlineStr">
         <is>
-          <t>Beurzen en tentoonstellingen</t>
+          <t>RECLAME ZONDER MERK</t>
         </is>
       </c>
       <c r="H20" s="8" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>EUDV</t>
         </is>
       </c>
       <c r="I20" s="8" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>88 · 55 · 59</t>
         </is>
       </c>
       <c r="J20" s="9" t="n">
-        <v>210</v>
+        <v>198.56</v>
       </c>
       <c r="K20" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L20" s="9" t="n">
-        <v>0</v>
+        <v>41.7</v>
       </c>
       <c r="M20" s="9" t="n">
-        <v>210</v>
+        <v>198.56</v>
       </c>
       <c r="N20" s="8" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="O20" s="8" t="inlineStr">
         <is>
-          <t>550000 KBC zichtrekening</t>
+          <t>434001 Mastercard Kaydee (2103)</t>
         </is>
       </c>
       <c r="P20" s="8" t="inlineStr"/>
       <c r="Q20" s="8" t="inlineStr">
         <is>
-          <t>NAKIJKEN: btw-behandeling nakijken</t>
+          <t>Yuki: intracommunautair diensten (verlegd)</t>
         </is>
       </c>
     </row>
@@ -8075,24 +8067,24 @@
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>Google ADS4790542578</t>
+          <t>SHOPIFY* 569354127</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr"/>
       <c r="E21" s="8" t="inlineStr"/>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t>616501</t>
+          <t>611080</t>
         </is>
       </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
-          <t>RECLAME ZONDER MERK</t>
+          <t>ABONNEMENTEN</t>
         </is>
       </c>
       <c r="H21" s="8" t="inlineStr">
@@ -8106,25 +8098,25 @@
         </is>
       </c>
       <c r="J21" s="9" t="n">
-        <v>198.56</v>
+        <v>174.81</v>
       </c>
       <c r="K21" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L21" s="9" t="n">
-        <v>41.7</v>
+        <v>36.71</v>
       </c>
       <c r="M21" s="9" t="n">
-        <v>198.56</v>
+        <v>174.81</v>
       </c>
       <c r="N21" s="8" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="O21" s="8" t="inlineStr">
         <is>
-          <t>434001 Mastercard Kaydee (2103)</t>
+          <t>434000 Mastercard Henri (6682)</t>
         </is>
       </c>
       <c r="P21" s="8" t="inlineStr"/>
@@ -8142,62 +8134,62 @@
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>SHOPIFY* 569354127</t>
+          <t>AMBULANTE ZELFSTANDIGEN VZW</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr"/>
       <c r="E22" s="8" t="inlineStr"/>
       <c r="F22" s="8" t="inlineStr">
         <is>
-          <t>611080</t>
+          <t>616620</t>
         </is>
       </c>
       <c r="G22" s="8" t="inlineStr">
         <is>
-          <t>ABONNEMENTEN</t>
+          <t>Beurzen en tentoonstellingen</t>
         </is>
       </c>
       <c r="H22" s="8" t="inlineStr">
         <is>
-          <t>EUDV</t>
+          <t>?</t>
         </is>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
-          <t>88 · 55 · 59</t>
+          <t>?</t>
         </is>
       </c>
       <c r="J22" s="9" t="n">
-        <v>174.81</v>
+        <v>230</v>
       </c>
       <c r="K22" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L22" s="9" t="n">
-        <v>36.71</v>
+        <v>0</v>
       </c>
       <c r="M22" s="9" t="n">
-        <v>174.81</v>
+        <v>230</v>
       </c>
       <c r="N22" s="8" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="O22" s="8" t="inlineStr">
         <is>
-          <t>434000 Mastercard Henri (6682)</t>
+          <t>550000 KBC zichtrekening</t>
         </is>
       </c>
       <c r="P22" s="8" t="inlineStr"/>
       <c r="Q22" s="8" t="inlineStr">
         <is>
-          <t>Yuki: intracommunautair diensten (verlegd)</t>
+          <t>NAKIJKEN: btw-behandeling nakijken</t>
         </is>
       </c>
     </row>
@@ -8281,42 +8273,42 @@
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>AMBULANTE ZELFSTANDIGEN VZW</t>
+          <t>SHOPIFY* 571029665</t>
         </is>
       </c>
       <c r="D24" s="8" t="inlineStr"/>
       <c r="E24" s="8" t="inlineStr"/>
       <c r="F24" s="8" t="inlineStr">
         <is>
-          <t>616620</t>
+          <t>611080</t>
         </is>
       </c>
       <c r="G24" s="8" t="inlineStr">
         <is>
-          <t>Beurzen en tentoonstellingen</t>
+          <t>ABONNEMENTEN</t>
         </is>
       </c>
       <c r="H24" s="8" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>EUDV</t>
         </is>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>88 · 55 · 59</t>
         </is>
       </c>
       <c r="J24" s="9" t="n">
-        <v>230</v>
+        <v>32</v>
       </c>
       <c r="K24" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L24" s="9" t="n">
-        <v>0</v>
+        <v>6.72</v>
       </c>
       <c r="M24" s="9" t="n">
-        <v>230</v>
+        <v>32</v>
       </c>
       <c r="N24" s="8" t="inlineStr">
         <is>
@@ -8325,13 +8317,13 @@
       </c>
       <c r="O24" s="8" t="inlineStr">
         <is>
-          <t>550000 KBC zichtrekening</t>
+          <t>434000 Mastercard Henri (6682)</t>
         </is>
       </c>
       <c r="P24" s="8" t="inlineStr"/>
       <c r="Q24" s="8" t="inlineStr">
         <is>
-          <t>NAKIJKEN: btw-behandeling nakijken</t>
+          <t>Yuki: intracommunautair diensten (verlegd)</t>
         </is>
       </c>
     </row>
@@ -8343,62 +8335,62 @@
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>SHOPIFY* 571029665</t>
+          <t>THE SANTIBAL BE8700 TIELT Betaling met KBC-Debetka</t>
         </is>
       </c>
       <c r="D25" s="8" t="inlineStr"/>
       <c r="E25" s="8" t="inlineStr"/>
       <c r="F25" s="8" t="inlineStr">
         <is>
-          <t>611080</t>
+          <t>616680</t>
         </is>
       </c>
       <c r="G25" s="8" t="inlineStr">
         <is>
-          <t>ABONNEMENTEN</t>
+          <t>Restaurantkosten</t>
         </is>
       </c>
       <c r="H25" s="8" t="inlineStr">
         <is>
-          <t>EUDV</t>
+          <t>BE21NA</t>
         </is>
       </c>
       <c r="I25" s="8" t="inlineStr">
         <is>
-          <t>88 · 55 · 59</t>
+          <t>82</t>
         </is>
       </c>
       <c r="J25" s="9" t="n">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="K25" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L25" s="9" t="n">
-        <v>6.72</v>
+        <v>0</v>
       </c>
       <c r="M25" s="9" t="n">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="N25" s="8" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="O25" s="8" t="inlineStr">
         <is>
-          <t>434000 Mastercard Henri (6682)</t>
+          <t>550000 KBC zichtrekening</t>
         </is>
       </c>
       <c r="P25" s="8" t="inlineStr"/>
       <c r="Q25" s="8" t="inlineStr">
         <is>
-          <t>Yuki: intracommunautair diensten (verlegd)</t>
+          <t>Yuki: 0% aftrek (restaurant)</t>
         </is>
       </c>
     </row>
@@ -8410,62 +8402,62 @@
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
-          <t>THE SANTIBAL BE8700 TIELT Betaling met KBC-Debetka</t>
+          <t>SHOPIFY* 576277386</t>
         </is>
       </c>
       <c r="D26" s="8" t="inlineStr"/>
       <c r="E26" s="8" t="inlineStr"/>
       <c r="F26" s="8" t="inlineStr">
         <is>
-          <t>616680</t>
+          <t>611080</t>
         </is>
       </c>
       <c r="G26" s="8" t="inlineStr">
         <is>
-          <t>Restaurantkosten</t>
+          <t>ABONNEMENTEN</t>
         </is>
       </c>
       <c r="H26" s="8" t="inlineStr">
         <is>
-          <t>BE21NA</t>
+          <t>EUDV</t>
         </is>
       </c>
       <c r="I26" s="8" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>88 · 55 · 59</t>
         </is>
       </c>
       <c r="J26" s="9" t="n">
-        <v>27</v>
+        <v>12.27</v>
       </c>
       <c r="K26" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L26" s="9" t="n">
-        <v>0</v>
+        <v>2.58</v>
       </c>
       <c r="M26" s="9" t="n">
-        <v>27</v>
+        <v>12.27</v>
       </c>
       <c r="N26" s="8" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="O26" s="8" t="inlineStr">
         <is>
-          <t>550000 KBC zichtrekening</t>
+          <t>434000 Mastercard Henri (6682)</t>
         </is>
       </c>
       <c r="P26" s="8" t="inlineStr"/>
       <c r="Q26" s="8" t="inlineStr">
         <is>
-          <t>Yuki: 0% aftrek (restaurant)</t>
+          <t>Yuki: intracommunautair diensten (verlegd)</t>
         </is>
       </c>
     </row>
@@ -8477,12 +8469,12 @@
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>SHOPIFY* 576277386</t>
+          <t>METAPAY*MV4B</t>
         </is>
       </c>
       <c r="D27" s="8" t="inlineStr"/>
@@ -8508,25 +8500,25 @@
         </is>
       </c>
       <c r="J27" s="9" t="n">
-        <v>12.27</v>
+        <v>22.29</v>
       </c>
       <c r="K27" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L27" s="9" t="n">
-        <v>2.58</v>
+        <v>4.68</v>
       </c>
       <c r="M27" s="9" t="n">
-        <v>12.27</v>
+        <v>22.29</v>
       </c>
       <c r="N27" s="8" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="O27" s="8" t="inlineStr">
         <is>
-          <t>434000 Mastercard Henri (6682)</t>
+          <t>434001 Mastercard Kaydee (2103)</t>
         </is>
       </c>
       <c r="P27" s="8" t="inlineStr"/>
@@ -8544,12 +8536,12 @@
       </c>
       <c r="B28" s="8" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="C28" s="8" t="inlineStr">
         <is>
-          <t>METAPAY*MV4B</t>
+          <t>SHOPIFY* 586058249</t>
         </is>
       </c>
       <c r="D28" s="8" t="inlineStr"/>
@@ -8575,25 +8567,25 @@
         </is>
       </c>
       <c r="J28" s="9" t="n">
-        <v>22.29</v>
+        <v>136.02</v>
       </c>
       <c r="K28" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L28" s="9" t="n">
-        <v>4.68</v>
+        <v>28.56</v>
       </c>
       <c r="M28" s="9" t="n">
-        <v>22.29</v>
+        <v>136.02</v>
       </c>
       <c r="N28" s="8" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="O28" s="8" t="inlineStr">
         <is>
-          <t>434001 Mastercard Kaydee (2103)</t>
+          <t>434000 Mastercard Henri (6682)</t>
         </is>
       </c>
       <c r="P28" s="8" t="inlineStr"/>
@@ -8611,62 +8603,62 @@
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>SHOPIFY* 586058249</t>
+          <t xml:space="preserve">PAY*PATRON BE9000 GENT Betaling met Apple Pay via </t>
         </is>
       </c>
       <c r="D29" s="8" t="inlineStr"/>
       <c r="E29" s="8" t="inlineStr"/>
       <c r="F29" s="8" t="inlineStr">
         <is>
-          <t>611080</t>
+          <t>616680</t>
         </is>
       </c>
       <c r="G29" s="8" t="inlineStr">
         <is>
-          <t>ABONNEMENTEN</t>
+          <t>Restaurantkosten</t>
         </is>
       </c>
       <c r="H29" s="8" t="inlineStr">
         <is>
-          <t>EUDV</t>
+          <t>BE21NA</t>
         </is>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
-          <t>88 · 55 · 59</t>
+          <t>82</t>
         </is>
       </c>
       <c r="J29" s="9" t="n">
-        <v>136.02</v>
+        <v>8.1</v>
       </c>
       <c r="K29" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L29" s="9" t="n">
-        <v>28.56</v>
+        <v>0</v>
       </c>
       <c r="M29" s="9" t="n">
-        <v>136.02</v>
+        <v>8.1</v>
       </c>
       <c r="N29" s="8" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="O29" s="8" t="inlineStr">
         <is>
-          <t>434000 Mastercard Henri (6682)</t>
+          <t>550000 KBC zichtrekening</t>
         </is>
       </c>
       <c r="P29" s="8" t="inlineStr"/>
       <c r="Q29" s="8" t="inlineStr">
         <is>
-          <t>Yuki: intracommunautair diensten (verlegd)</t>
+          <t>Yuki: 0% aftrek (restaurant)</t>
         </is>
       </c>
     </row>
@@ -8683,33 +8675,33 @@
       </c>
       <c r="C30" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">PAY*PATRON BE9000 GENT Betaling met Apple Pay via </t>
+          <t>POM-OostV Bedrijven BE9000 Gent Betaling met KBC-D</t>
         </is>
       </c>
       <c r="D30" s="8" t="inlineStr"/>
       <c r="E30" s="8" t="inlineStr"/>
       <c r="F30" s="8" t="inlineStr">
         <is>
-          <t>616680</t>
+          <t>616651</t>
         </is>
       </c>
       <c r="G30" s="8" t="inlineStr">
         <is>
-          <t>Restaurantkosten</t>
+          <t>Beroepsbijdragen</t>
         </is>
       </c>
       <c r="H30" s="8" t="inlineStr">
         <is>
-          <t>BE21NA</t>
+          <t>?</t>
         </is>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>?</t>
         </is>
       </c>
       <c r="J30" s="9" t="n">
-        <v>8.1</v>
+        <v>148</v>
       </c>
       <c r="K30" s="9" t="n">
         <v>0</v>
@@ -8718,7 +8710,7 @@
         <v>0</v>
       </c>
       <c r="M30" s="9" t="n">
-        <v>8.1</v>
+        <v>148</v>
       </c>
       <c r="N30" s="8" t="inlineStr">
         <is>
@@ -8733,74 +8725,82 @@
       <c r="P30" s="8" t="inlineStr"/>
       <c r="Q30" s="8" t="inlineStr">
         <is>
-          <t>Yuki: 0% aftrek (restaurant)</t>
+          <t>NAKIJKEN: btw-behandeling nakijken</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>factuur ontbreekt</t>
+          <t>in Yuki</t>
         </is>
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>POM-OostV Bedrijven BE9000 Gent Betaling met KBC-D</t>
+          <t>Suzhou Compass Machinery &amp; Electric Co., Ltd. (CN)</t>
         </is>
       </c>
       <c r="D31" s="8" t="inlineStr"/>
-      <c r="E31" s="8" t="inlineStr"/>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>CPS20260619</t>
+        </is>
+      </c>
       <c r="F31" s="8" t="inlineStr">
         <is>
-          <t>616651</t>
+          <t>604000</t>
         </is>
       </c>
       <c r="G31" s="8" t="inlineStr">
         <is>
-          <t>Beroepsbijdragen</t>
+          <t>Aankopen van handelsgoederen</t>
         </is>
       </c>
       <c r="H31" s="8" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>INVOER</t>
         </is>
       </c>
       <c r="I31" s="8" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>87 · 56 · 59 (op invoeraangifte)</t>
         </is>
       </c>
       <c r="J31" s="9" t="n">
-        <v>148</v>
+        <v>8637.91</v>
       </c>
       <c r="K31" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L31" s="9" t="n">
-        <v>0</v>
+        <v>1813.96</v>
       </c>
       <c r="M31" s="9" t="n">
-        <v>148</v>
+        <v>8637.91</v>
       </c>
       <c r="N31" s="8" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="O31" s="8" t="inlineStr">
         <is>
-          <t>550000 KBC zichtrekening</t>
-        </is>
-      </c>
-      <c r="P31" s="8" t="inlineStr"/>
+          <t>550001 Revolut EUR</t>
+        </is>
+      </c>
+      <c r="P31" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-24_Compass_FurVac750_21784.75USD.pdf</t>
+        </is>
+      </c>
       <c r="Q31" s="8" t="inlineStr">
         <is>
-          <t>NAKIJKEN: btw-behandeling nakijken</t>
+          <t>Yuki: invoer met verlegging (art. 41, invoeraangifte Widem)</t>
         </is>
       </c>
     </row>
@@ -8812,70 +8812,70 @@
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
-          <t>Suzhou Compass Machinery &amp; Electric Co., Ltd. (CN)</t>
+          <t>Meta Platforms Ireland</t>
         </is>
       </c>
       <c r="D32" s="8" t="inlineStr"/>
       <c r="E32" s="8" t="inlineStr">
         <is>
-          <t>CPS20260619</t>
+          <t>27253725940979469-27253726004312796</t>
         </is>
       </c>
       <c r="F32" s="8" t="inlineStr">
         <is>
-          <t>604000</t>
+          <t>616502</t>
         </is>
       </c>
       <c r="G32" s="8" t="inlineStr">
         <is>
-          <t>Aankopen van handelsgoederen</t>
+          <t>RECLAME MET MERK</t>
         </is>
       </c>
       <c r="H32" s="8" t="inlineStr">
         <is>
-          <t>INVOER</t>
+          <t>EUDV</t>
         </is>
       </c>
       <c r="I32" s="8" t="inlineStr">
         <is>
-          <t>87 · 56 · 59 (op invoeraangifte)</t>
+          <t>88 · 55 · 59</t>
         </is>
       </c>
       <c r="J32" s="9" t="n">
-        <v>8637.91</v>
+        <v>800</v>
       </c>
       <c r="K32" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L32" s="9" t="n">
-        <v>1813.96</v>
+        <v>168</v>
       </c>
       <c r="M32" s="9" t="n">
-        <v>8637.91</v>
+        <v>800</v>
       </c>
       <c r="N32" s="8" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="O32" s="8" t="inlineStr">
         <is>
-          <t>550001 Revolut EUR</t>
+          <t>550000 KBC zichtrekening</t>
         </is>
       </c>
       <c r="P32" s="8" t="inlineStr">
         <is>
-          <t>2026-06-24_Compass_FurVac750_21784.75USD.pdf</t>
+          <t>Meta-kwitantie 27253725940979469-27253726004312796 (2026-07-01) – in Lucy/Yuki</t>
         </is>
       </c>
       <c r="Q32" s="8" t="inlineStr">
         <is>
-          <t>Yuki: invoer met verlegging (art. 41, invoeraangifte Widem)</t>
+          <t>Yuki: intracommunautair diensten (verlegd)</t>
         </is>
       </c>
     </row>
@@ -8892,23 +8892,23 @@
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>Meta Platforms Ireland</t>
+          <t>GOOGLE*WORKSPACE SMART IED02 R296 CC GOOGLE.COM Be</t>
         </is>
       </c>
       <c r="D33" s="8" t="inlineStr"/>
       <c r="E33" s="8" t="inlineStr">
         <is>
-          <t>27253725940979469-27253726004312796</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="F33" s="8" t="inlineStr">
         <is>
-          <t>616502</t>
+          <t>616501</t>
         </is>
       </c>
       <c r="G33" s="8" t="inlineStr">
         <is>
-          <t>RECLAME MET MERK</t>
+          <t>RECLAME ZONDER MERK</t>
         </is>
       </c>
       <c r="H33" s="8" t="inlineStr">
@@ -8922,16 +8922,16 @@
         </is>
       </c>
       <c r="J33" s="9" t="n">
-        <v>800</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="K33" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L33" s="9" t="n">
-        <v>168</v>
+        <v>15.94</v>
       </c>
       <c r="M33" s="9" t="n">
-        <v>800</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="N33" s="8" t="inlineStr">
         <is>
@@ -8945,7 +8945,7 @@
       </c>
       <c r="P33" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 27253725940979469-27253726004312796 (2026-07-01) – in Lucy/Yuki</t>
+          <t>in Yuki: Google Ireland Limited (2026-07-02)</t>
         </is>
       </c>
       <c r="Q33" s="8" t="inlineStr">
@@ -8967,46 +8967,46 @@
       </c>
       <c r="C34" s="8" t="inlineStr">
         <is>
-          <t>GOOGLE*WORKSPACE SMART IED02 R296 CC GOOGLE.COM Be</t>
+          <t>Yuki Works NV via Mollie</t>
         </is>
       </c>
       <c r="D34" s="8" t="inlineStr"/>
       <c r="E34" s="8" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="F34" s="8" t="inlineStr">
         <is>
-          <t>616501</t>
+          <t>611080</t>
         </is>
       </c>
       <c r="G34" s="8" t="inlineStr">
         <is>
-          <t>RECLAME ZONDER MERK</t>
+          <t>ABONNEMENTEN</t>
         </is>
       </c>
       <c r="H34" s="8" t="inlineStr">
         <is>
-          <t>EUDV</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
-          <t>88 · 55 · 59</t>
+          <t>82 · 59</t>
         </is>
       </c>
       <c r="J34" s="9" t="n">
-        <v>75.90000000000001</v>
+        <v>2</v>
       </c>
       <c r="K34" s="9" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="L34" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="L34" s="9" t="n">
-        <v>15.94</v>
-      </c>
       <c r="M34" s="9" t="n">
-        <v>75.90000000000001</v>
+        <v>2.42</v>
       </c>
       <c r="N34" s="8" t="inlineStr">
         <is>
@@ -9020,12 +9020,12 @@
       </c>
       <c r="P34" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Google Ireland Limited (2026-07-02)</t>
+          <t>in Yuki: Yuki works (2026-07-01)</t>
         </is>
       </c>
       <c r="Q34" s="8" t="inlineStr">
         <is>
-          <t>Yuki: intracommunautair diensten (verlegd)</t>
+          <t>Yuki: 21%</t>
         </is>
       </c>
     </row>
@@ -9037,18 +9037,18 @@
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>Yuki Works NV via Mollie</t>
+          <t>RETURNGO</t>
         </is>
       </c>
       <c r="D35" s="8" t="inlineStr"/>
       <c r="E35" s="8" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="F35" s="8" t="inlineStr">
@@ -9063,44 +9063,44 @@
       </c>
       <c r="H35" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>NEUDV</t>
         </is>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
-          <t>82 · 59</t>
+          <t>87 · 56 · 59</t>
         </is>
       </c>
       <c r="J35" s="9" t="n">
-        <v>2</v>
+        <v>86</v>
       </c>
       <c r="K35" s="9" t="n">
-        <v>0.42</v>
+        <v>0</v>
       </c>
       <c r="L35" s="9" t="n">
-        <v>0</v>
+        <v>18.06</v>
       </c>
       <c r="M35" s="9" t="n">
-        <v>2.42</v>
+        <v>86</v>
       </c>
       <c r="N35" s="8" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="O35" s="8" t="inlineStr">
         <is>
-          <t>550000 KBC zichtrekening</t>
+          <t>434000 Mastercard Henri (6682)</t>
         </is>
       </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Yuki works (2026-07-01)</t>
+          <t>in Yuki: Returngo (2026-04-23)</t>
         </is>
       </c>
       <c r="Q35" s="8" t="inlineStr">
         <is>
-          <t>Yuki: 21%</t>
+          <t>Yuki: btw verlegd (dienst buiten EU)</t>
         </is>
       </c>
     </row>
@@ -9112,62 +9112,70 @@
       </c>
       <c r="B36" s="8" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="C36" s="8" t="inlineStr">
         <is>
-          <t>RETURNGO</t>
+          <t>Pro-Count</t>
         </is>
       </c>
       <c r="D36" s="8" t="inlineStr"/>
-      <c r="E36" s="8" t="inlineStr"/>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
       <c r="F36" s="8" t="inlineStr">
         <is>
-          <t>611080</t>
+          <t>615200</t>
         </is>
       </c>
       <c r="G36" s="8" t="inlineStr">
         <is>
-          <t>ABONNEMENTEN</t>
+          <t>Erelonen boekhouders en accountants</t>
         </is>
       </c>
       <c r="H36" s="8" t="inlineStr">
         <is>
-          <t>NEUDV</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
-          <t>87 · 56 · 59</t>
+          <t>82 · 59</t>
         </is>
       </c>
       <c r="J36" s="9" t="n">
-        <v>86</v>
+        <v>200</v>
       </c>
       <c r="K36" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="L36" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="L36" s="9" t="n">
-        <v>18.06</v>
-      </c>
       <c r="M36" s="9" t="n">
-        <v>86</v>
+        <v>242</v>
       </c>
       <c r="N36" s="8" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="O36" s="8" t="inlineStr">
         <is>
-          <t>434000 Mastercard Henri (6682)</t>
-        </is>
-      </c>
-      <c r="P36" s="8" t="inlineStr"/>
+          <t>550000 KBC zichtrekening</t>
+        </is>
+      </c>
+      <c r="P36" s="8" t="inlineStr">
+        <is>
+          <t>in Yuki: Pro-Count (2026-07-06)</t>
+        </is>
+      </c>
       <c r="Q36" s="8" t="inlineStr">
         <is>
-          <t>Yuki: btw verlegd (dienst buiten EU)</t>
+          <t>Yuki: 21%</t>
         </is>
       </c>
     </row>
@@ -9259,7 +9267,7 @@
       </c>
       <c r="C38" s="8" t="inlineStr">
         <is>
-          <t>Pro-Count</t>
+          <t>Widem Logistics NV</t>
         </is>
       </c>
       <c r="D38" s="8" t="inlineStr"/>
@@ -9270,12 +9278,12 @@
       </c>
       <c r="F38" s="8" t="inlineStr">
         <is>
-          <t>615200</t>
+          <t>612730</t>
         </is>
       </c>
       <c r="G38" s="8" t="inlineStr">
         <is>
-          <t>Erelonen boekhouders en accountants</t>
+          <t>TRANSPORTEN AAN DERDEN</t>
         </is>
       </c>
       <c r="H38" s="8" t="inlineStr">
@@ -9289,16 +9297,16 @@
         </is>
       </c>
       <c r="J38" s="9" t="n">
-        <v>200</v>
+        <v>436.22</v>
       </c>
       <c r="K38" s="9" t="n">
-        <v>42</v>
+        <v>91.61</v>
       </c>
       <c r="L38" s="9" t="n">
         <v>0</v>
       </c>
       <c r="M38" s="9" t="n">
-        <v>242</v>
+        <v>527.83</v>
       </c>
       <c r="N38" s="8" t="inlineStr">
         <is>
@@ -9312,7 +9320,7 @@
       </c>
       <c r="P38" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Pro-Count (2026-07-06)</t>
+          <t>in Yuki: Widem Logistics (2026-07-06)</t>
         </is>
       </c>
       <c r="Q38" s="8" t="inlineStr">
@@ -9334,7 +9342,7 @@
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>Widem Logistics NV</t>
+          <t>Findajob bv</t>
         </is>
       </c>
       <c r="D39" s="8" t="inlineStr"/>
@@ -9345,12 +9353,12 @@
       </c>
       <c r="F39" s="8" t="inlineStr">
         <is>
-          <t>612730</t>
+          <t>617000</t>
         </is>
       </c>
       <c r="G39" s="8" t="inlineStr">
         <is>
-          <t>TRANSPORTEN AAN DERDEN</t>
+          <t>Uitzendkrachten</t>
         </is>
       </c>
       <c r="H39" s="8" t="inlineStr">
@@ -9364,16 +9372,16 @@
         </is>
       </c>
       <c r="J39" s="9" t="n">
-        <v>436.22</v>
+        <v>62.63</v>
       </c>
       <c r="K39" s="9" t="n">
-        <v>91.61</v>
+        <v>13.15</v>
       </c>
       <c r="L39" s="9" t="n">
         <v>0</v>
       </c>
       <c r="M39" s="9" t="n">
-        <v>527.83</v>
+        <v>75.78</v>
       </c>
       <c r="N39" s="8" t="inlineStr">
         <is>
@@ -9387,7 +9395,7 @@
       </c>
       <c r="P39" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Widem Logistics (2026-07-06)</t>
+          <t>in Yuki: Findajob (2026-07-06)</t>
         </is>
       </c>
       <c r="Q39" s="8" t="inlineStr">
@@ -9409,7 +9417,7 @@
       </c>
       <c r="C40" s="8" t="inlineStr">
         <is>
-          <t>Findajob bv</t>
+          <t>Henri Steyaert</t>
         </is>
       </c>
       <c r="D40" s="8" t="inlineStr"/>
@@ -9420,35 +9428,35 @@
       </c>
       <c r="F40" s="8" t="inlineStr">
         <is>
-          <t>617000</t>
+          <t>611080</t>
         </is>
       </c>
       <c r="G40" s="8" t="inlineStr">
         <is>
-          <t>Uitzendkrachten</t>
+          <t>ABONNEMENTEN</t>
         </is>
       </c>
       <c r="H40" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>?</t>
         </is>
       </c>
       <c r="I40" s="8" t="inlineStr">
         <is>
-          <t>82 · 59</t>
+          <t>?</t>
         </is>
       </c>
       <c r="J40" s="9" t="n">
-        <v>62.63</v>
+        <v>91.84</v>
       </c>
       <c r="K40" s="9" t="n">
-        <v>13.15</v>
+        <v>0</v>
       </c>
       <c r="L40" s="9" t="n">
         <v>0</v>
       </c>
       <c r="M40" s="9" t="n">
-        <v>75.78</v>
+        <v>91.84</v>
       </c>
       <c r="N40" s="8" t="inlineStr">
         <is>
@@ -9462,12 +9470,12 @@
       </c>
       <c r="P40" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Findajob (2026-07-06)</t>
+          <t>in Yuki: Henri Steyaert (2026-07-06)</t>
         </is>
       </c>
       <c r="Q40" s="8" t="inlineStr">
         <is>
-          <t>Yuki: 21%</t>
+          <t>NAKIJKEN: btw-behandeling nakijken</t>
         </is>
       </c>
     </row>
@@ -9484,7 +9492,7 @@
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t>Henri Steyaert</t>
+          <t>Findajob bv</t>
         </is>
       </c>
       <c r="D41" s="8" t="inlineStr"/>
@@ -9495,35 +9503,35 @@
       </c>
       <c r="F41" s="8" t="inlineStr">
         <is>
-          <t>611080</t>
+          <t>617000</t>
         </is>
       </c>
       <c r="G41" s="8" t="inlineStr">
         <is>
-          <t>ABONNEMENTEN</t>
+          <t>Uitzendkrachten</t>
         </is>
       </c>
       <c r="H41" s="8" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="I41" s="8" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>82 · 59</t>
         </is>
       </c>
       <c r="J41" s="9" t="n">
-        <v>91.84</v>
+        <v>15.66</v>
       </c>
       <c r="K41" s="9" t="n">
-        <v>0</v>
+        <v>3.29</v>
       </c>
       <c r="L41" s="9" t="n">
         <v>0</v>
       </c>
       <c r="M41" s="9" t="n">
-        <v>91.84</v>
+        <v>18.95</v>
       </c>
       <c r="N41" s="8" t="inlineStr">
         <is>
@@ -9537,12 +9545,12 @@
       </c>
       <c r="P41" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Henri Steyaert (2026-07-06)</t>
+          <t>in Yuki: Findajob (2026-07-06)</t>
         </is>
       </c>
       <c r="Q41" s="8" t="inlineStr">
         <is>
-          <t>NAKIJKEN: btw-behandeling nakijken</t>
+          <t>Yuki: 21%</t>
         </is>
       </c>
     </row>
@@ -9554,57 +9562,57 @@
       </c>
       <c r="B42" s="8" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="C42" s="8" t="inlineStr">
         <is>
-          <t>Findajob bv</t>
+          <t>Meta Platforms Ireland</t>
         </is>
       </c>
       <c r="D42" s="8" t="inlineStr"/>
       <c r="E42" s="8" t="inlineStr">
         <is>
+          <t>27355189934166399-27530401703311892</t>
+        </is>
+      </c>
+      <c r="F42" s="8" t="inlineStr">
+        <is>
+          <t>616502</t>
+        </is>
+      </c>
+      <c r="G42" s="8" t="inlineStr">
+        <is>
+          <t>RECLAME MET MERK</t>
+        </is>
+      </c>
+      <c r="H42" s="8" t="inlineStr">
+        <is>
+          <t>EUDV</t>
+        </is>
+      </c>
+      <c r="I42" s="8" t="inlineStr">
+        <is>
+          <t>88 · 55 · 59</t>
+        </is>
+      </c>
+      <c r="J42" s="9" t="n">
+        <v>800</v>
+      </c>
+      <c r="K42" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L42" s="9" t="n">
+        <v>168</v>
+      </c>
+      <c r="M42" s="9" t="n">
+        <v>800</v>
+      </c>
+      <c r="N42" s="8" t="inlineStr">
+        <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="F42" s="8" t="inlineStr">
-        <is>
-          <t>617000</t>
-        </is>
-      </c>
-      <c r="G42" s="8" t="inlineStr">
-        <is>
-          <t>Uitzendkrachten</t>
-        </is>
-      </c>
-      <c r="H42" s="8" t="inlineStr">
-        <is>
-          <t>BE21</t>
-        </is>
-      </c>
-      <c r="I42" s="8" t="inlineStr">
-        <is>
-          <t>82 · 59</t>
-        </is>
-      </c>
-      <c r="J42" s="9" t="n">
-        <v>15.66</v>
-      </c>
-      <c r="K42" s="9" t="n">
-        <v>3.29</v>
-      </c>
-      <c r="L42" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="M42" s="9" t="n">
-        <v>18.95</v>
-      </c>
-      <c r="N42" s="8" t="inlineStr">
-        <is>
-          <t>2026-07-05</t>
-        </is>
-      </c>
       <c r="O42" s="8" t="inlineStr">
         <is>
           <t>550000 KBC zichtrekening</t>
@@ -9612,12 +9620,12 @@
       </c>
       <c r="P42" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Findajob (2026-07-06)</t>
+          <t>Meta-kwitantie 27355189934166399-27530401703311892 (2026-07-06) – in Lucy/Yuki</t>
         </is>
       </c>
       <c r="Q42" s="8" t="inlineStr">
         <is>
-          <t>Yuki: 21%</t>
+          <t>Yuki: intracommunautair diensten (verlegd)</t>
         </is>
       </c>
     </row>
@@ -9629,55 +9637,55 @@
       </c>
       <c r="B43" s="8" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>Meta Platforms Ireland</t>
+          <t>Widem Logistics NV</t>
         </is>
       </c>
       <c r="D43" s="8" t="inlineStr"/>
       <c r="E43" s="8" t="inlineStr">
         <is>
-          <t>27355189934166399-27530401703311892</t>
+          <t>26012021</t>
         </is>
       </c>
       <c r="F43" s="8" t="inlineStr">
         <is>
-          <t>616502</t>
+          <t>612730</t>
         </is>
       </c>
       <c r="G43" s="8" t="inlineStr">
         <is>
-          <t>RECLAME MET MERK</t>
+          <t>TRANSPORTEN AAN DERDEN</t>
         </is>
       </c>
       <c r="H43" s="8" t="inlineStr">
         <is>
-          <t>EUDV</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="I43" s="8" t="inlineStr">
         <is>
-          <t>88 · 55 · 59</t>
+          <t>82 · 59</t>
         </is>
       </c>
       <c r="J43" s="9" t="n">
-        <v>800</v>
+        <v>2590.91</v>
       </c>
       <c r="K43" s="9" t="n">
+        <v>544.09</v>
+      </c>
+      <c r="L43" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="L43" s="9" t="n">
-        <v>168</v>
-      </c>
       <c r="M43" s="9" t="n">
-        <v>800</v>
+        <v>3135</v>
       </c>
       <c r="N43" s="8" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="O43" s="8" t="inlineStr">
@@ -9687,12 +9695,12 @@
       </c>
       <c r="P43" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 27355189934166399-27530401703311892 (2026-07-06) – in Lucy/Yuki</t>
+          <t>Widem 26012021 (mail 2026-07-07)</t>
         </is>
       </c>
       <c r="Q43" s="8" t="inlineStr">
         <is>
-          <t>Yuki: intracommunautair diensten (verlegd)</t>
+          <t>Yuki: 21%</t>
         </is>
       </c>
     </row>
@@ -15049,7 +15057,7 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>Bewijs per verrichting: 83 gekoppeld, 81 verklaard (geen factuur nodig, niet in deze lijst), 18 ontbreken. Facturen zitten in de map Facturen_Q3-2026 (bestandsnaam = datum_leverancier_bedrag).</t>
+          <t>Bewijs per verrichting: 84 gekoppeld, 81 verklaard (geen factuur nodig, niet in deze lijst), 17 ontbreken. Facturen zitten in de map Facturen_Q3-2026 (bestandsnaam = datum_leverancier_bedrag).</t>
         </is>
       </c>
     </row>
@@ -15114,20 +15122,20 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>RETURNGO</t>
+          <t>SHOPIFY* 556521062</t>
         </is>
       </c>
       <c r="C5" s="9" t="n">
-        <v>-86</v>
+        <v>-141.39</v>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>NONEU</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
@@ -15140,16 +15148,16 @@
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>SHOPIFY* 556521062</t>
+          <t>Google ADS4790542578</t>
         </is>
       </c>
       <c r="C6" s="9" t="n">
-        <v>-141.39</v>
+        <v>-500</v>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
@@ -15166,20 +15174,20 @@
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Google ADS4790542578</t>
+          <t>SP PACKAGINGDISCOUNTER</t>
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>-500</v>
+        <v>-360</v>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>NAKIJKEN</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
@@ -15192,20 +15200,20 @@
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>SP PACKAGINGDISCOUNTER</t>
+          <t>YAKI NOODLE BAR BE9000 GENT Betaling met KBC-Debet</t>
         </is>
       </c>
       <c r="C8" s="9" t="n">
-        <v>-360</v>
+        <v>-15</v>
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>NAKIJKEN</t>
+          <t>BE21NA</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
@@ -15218,20 +15226,20 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>YAKI NOODLE BAR BE9000 GENT Betaling met KBC-Debet</t>
+          <t>AMBULANTE ZELFSTANDIGEN VZW</t>
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>-15</v>
+        <v>-210</v>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>BE21NA</t>
+          <t>NAKIJKEN</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
@@ -15244,20 +15252,20 @@
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>AMBULANTE ZELFSTANDIGEN VZW</t>
+          <t>Google ADS4790542578</t>
         </is>
       </c>
       <c r="C10" s="9" t="n">
-        <v>-210</v>
+        <v>-198.56</v>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>NAKIJKEN</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
@@ -15270,16 +15278,16 @@
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>Google ADS4790542578</t>
+          <t>SHOPIFY* 569354127</t>
         </is>
       </c>
       <c r="C11" s="9" t="n">
-        <v>-198.56</v>
+        <v>-174.81</v>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
@@ -15296,20 +15304,20 @@
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>SHOPIFY* 569354127</t>
+          <t>AMBULANTE ZELFSTANDIGEN VZW</t>
         </is>
       </c>
       <c r="C12" s="9" t="n">
-        <v>-174.81</v>
+        <v>-230</v>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>NAKIJKEN</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
@@ -15353,15 +15361,15 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>AMBULANTE ZELFSTANDIGEN VZW</t>
+          <t>SHOPIFY* 571029665</t>
         </is>
       </c>
       <c r="C14" s="9" t="n">
-        <v>-230</v>
+        <v>-32</v>
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>NAKIJKEN</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
@@ -15374,20 +15382,20 @@
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>SHOPIFY* 571029665</t>
+          <t>THE SANTIBAL BE8700 TIELT Betaling met KBC-Debetka</t>
         </is>
       </c>
       <c r="C15" s="9" t="n">
-        <v>-32</v>
+        <v>-27</v>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>BE21NA</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
@@ -15400,20 +15408,20 @@
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>THE SANTIBAL BE8700 TIELT Betaling met KBC-Debetka</t>
+          <t>SHOPIFY* 576277386</t>
         </is>
       </c>
       <c r="C16" s="9" t="n">
-        <v>-27</v>
+        <v>-12.27</v>
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>BE21NA</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
@@ -15426,16 +15434,16 @@
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>SHOPIFY* 576277386</t>
+          <t>METAPAY*MV4B</t>
         </is>
       </c>
       <c r="C17" s="9" t="n">
-        <v>-12.27</v>
+        <v>-22.29</v>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
@@ -15452,16 +15460,16 @@
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>METAPAY*MV4B</t>
+          <t>SHOPIFY* 586058249</t>
         </is>
       </c>
       <c r="C18" s="9" t="n">
-        <v>-22.29</v>
+        <v>-136.02</v>
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
@@ -15478,20 +15486,20 @@
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>SHOPIFY* 586058249</t>
+          <t xml:space="preserve">PAY*PATRON BE9000 GENT Betaling met Apple Pay via </t>
         </is>
       </c>
       <c r="C19" s="9" t="n">
-        <v>-136.02</v>
+        <v>-8.1</v>
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>BE21NA</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
@@ -15509,15 +15517,15 @@
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">PAY*PATRON BE9000 GENT Betaling met Apple Pay via </t>
+          <t>POM-OostV Bedrijven BE9000 Gent Betaling met KBC-D</t>
         </is>
       </c>
       <c r="C20" s="9" t="n">
-        <v>-8.1</v>
+        <v>-148</v>
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>BE21NA</t>
+          <t>NAKIJKEN</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
@@ -15530,28 +15538,32 @@
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>POM-OostV Bedrijven BE9000 Gent Betaling met KBC-D</t>
+          <t xml:space="preserve">FACEBK *X87X6SV7A2 IED04 X2K5 Dublin Betaling met </t>
         </is>
       </c>
       <c r="C21" s="9" t="n">
-        <v>-148</v>
+        <v>-800</v>
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>NAKIJKEN</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F21" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>Meta-kwitantie 27253725940979469-27253726004312796 (2026-07-01) – in Lucy/Yuki</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
@@ -15561,11 +15573,11 @@
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">FACEBK *X87X6SV7A2 IED04 X2K5 Dublin Betaling met </t>
+          <t>GOOGLE*WORKSPACE SMART IED02 R296 CC GOOGLE.COM Be</t>
         </is>
       </c>
       <c r="C22" s="9" t="n">
-        <v>-800</v>
+        <v>-75.90000000000001</v>
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
@@ -15579,7 +15591,7 @@
       </c>
       <c r="F22" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 27253725940979469-27253726004312796 (2026-07-01) – in Lucy/Yuki</t>
+          <t>in Yuki: Google Ireland Limited (2026-07-02)</t>
         </is>
       </c>
     </row>
@@ -15591,15 +15603,15 @@
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>GOOGLE*WORKSPACE SMART IED02 R296 CC GOOGLE.COM Be</t>
+          <t>Yuki Works NV via Mollie</t>
         </is>
       </c>
       <c r="C23" s="9" t="n">
-        <v>-75.90000000000001</v>
+        <v>-2.42</v>
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
@@ -15609,27 +15621,27 @@
       </c>
       <c r="F23" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Google Ireland Limited (2026-07-02)</t>
+          <t>in Yuki: Yuki works (2026-07-01)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>Yuki Works NV via Mollie</t>
+          <t>RETURNGO</t>
         </is>
       </c>
       <c r="C24" s="9" t="n">
-        <v>-2.42</v>
+        <v>-86</v>
       </c>
       <c r="D24" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>NONEU</t>
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr">
@@ -15639,7 +15651,7 @@
       </c>
       <c r="F24" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Yuki works (2026-07-01)</t>
+          <t>in Yuki: Returngo (2026-04-23)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Aankoopdagboek: ook facturen in Yuki die nog niet betaald zijn
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WLjvFcZoD9WegLqrYozzyo
</commit_message>
<xml_diff>
--- a/boekhouding/rapporten/SmartPaw_Q3-2026.xlsx
+++ b/boekhouding/rapporten/SmartPaw_Q3-2026.xlsx
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Aankopen'!$A$3:$J$117</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Aankoopdagboek'!$A$3:$Q$104</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Aankoopdagboek'!$A$3:$Q$111</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -6724,7 +6724,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q121"/>
+  <dimension ref="A1:Q130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6749,7 +6749,7 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>Aankoopdagboek Q3 2026: 10 te boeken, 74 al in Yuki (ter controle), 17 zonder factuur. Grootboekrekeningen volgens jullie rekeningschema; btw-codes: eigen code + roosters.</t>
+          <t>Aankoopdagboek Q3 2026: 10 te boeken, 81 al in Yuki (ter controle), 17 zonder factuur. Grootboekrekeningen volgens jullie rekeningschema; btw-codes: eigen code + roosters.</t>
         </is>
       </c>
     </row>
@@ -12792,65 +12792,57 @@
       </c>
       <c r="C85" s="8" t="inlineStr">
         <is>
-          <t>Meta Platforms Ireland</t>
+          <t>Proximus</t>
         </is>
       </c>
       <c r="D85" s="8" t="inlineStr"/>
       <c r="E85" s="8" t="inlineStr">
         <is>
-          <t>28135330259485690-28135330349485681</t>
+          <t>7605427449</t>
         </is>
       </c>
       <c r="F85" s="8" t="inlineStr">
         <is>
-          <t>616502</t>
+          <t>657000</t>
         </is>
       </c>
       <c r="G85" s="8" t="inlineStr">
         <is>
-          <t>RECLAME MET MERK</t>
+          <t>Diverse financiële kosten</t>
         </is>
       </c>
       <c r="H85" s="8" t="inlineStr">
         <is>
-          <t>EUDV</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="I85" s="8" t="inlineStr">
         <is>
-          <t>88 · 55 · 59</t>
+          <t>82 · 59</t>
         </is>
       </c>
       <c r="J85" s="9" t="n">
-        <v>800</v>
+        <v>8.26</v>
       </c>
       <c r="K85" s="9" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="L85" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="L85" s="9" t="n">
-        <v>168</v>
-      </c>
       <c r="M85" s="9" t="n">
-        <v>800</v>
-      </c>
-      <c r="N85" s="8" t="inlineStr">
-        <is>
-          <t>2026-09-06</t>
-        </is>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="N85" s="8" t="inlineStr"/>
       <c r="O85" s="8" t="inlineStr">
         <is>
-          <t>550000 KBC zichtrekening</t>
-        </is>
-      </c>
-      <c r="P85" s="8" t="inlineStr">
-        <is>
-          <t>Meta-kwitantie 28135330259485690-28135330349485681 (2026-09-05) – in Lucy/Yuki</t>
-        </is>
-      </c>
+          <t xml:space="preserve"> nog te betalen (vervalt 2026-09-21)</t>
+        </is>
+      </c>
+      <c r="P85" s="8" t="inlineStr"/>
       <c r="Q85" s="8" t="inlineStr">
         <is>
-          <t>Yuki: intracommunautair diensten (verlegd)</t>
+          <t>Yuki: 21%</t>
         </is>
       </c>
     </row>
@@ -12862,55 +12854,55 @@
       </c>
       <c r="B86" s="8" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="C86" s="8" t="inlineStr">
         <is>
-          <t>WIDEM LOGISTICS NV</t>
+          <t>Meta Platforms Ireland</t>
         </is>
       </c>
       <c r="D86" s="8" t="inlineStr"/>
       <c r="E86" s="8" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>28135330259485690-28135330349485681</t>
         </is>
       </c>
       <c r="F86" s="8" t="inlineStr">
         <is>
-          <t>612730</t>
+          <t>616502</t>
         </is>
       </c>
       <c r="G86" s="8" t="inlineStr">
         <is>
-          <t>TRANSPORTEN AAN DERDEN</t>
+          <t>RECLAME MET MERK</t>
         </is>
       </c>
       <c r="H86" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>EUDV</t>
         </is>
       </c>
       <c r="I86" s="8" t="inlineStr">
         <is>
-          <t>82 · 59</t>
+          <t>88 · 55 · 59</t>
         </is>
       </c>
       <c r="J86" s="9" t="n">
-        <v>1951.47</v>
+        <v>800</v>
       </c>
       <c r="K86" s="9" t="n">
-        <v>409.81</v>
+        <v>0</v>
       </c>
       <c r="L86" s="9" t="n">
-        <v>0</v>
+        <v>168</v>
       </c>
       <c r="M86" s="9" t="n">
-        <v>2361.28</v>
+        <v>800</v>
       </c>
       <c r="N86" s="8" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="O86" s="8" t="inlineStr">
@@ -12920,12 +12912,12 @@
       </c>
       <c r="P86" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Widem Logistics (2026-09-09)</t>
+          <t>Meta-kwitantie 28135330259485690-28135330349485681 (2026-09-05) – in Lucy/Yuki</t>
         </is>
       </c>
       <c r="Q86" s="8" t="inlineStr">
         <is>
-          <t>Yuki: 21%</t>
+          <t>Yuki: intracommunautair diensten (verlegd)</t>
         </is>
       </c>
     </row>
@@ -12942,7 +12934,7 @@
       </c>
       <c r="C87" s="8" t="inlineStr">
         <is>
-          <t>Findajob bv</t>
+          <t>WIDEM LOGISTICS NV</t>
         </is>
       </c>
       <c r="D87" s="8" t="inlineStr"/>
@@ -12953,12 +12945,12 @@
       </c>
       <c r="F87" s="8" t="inlineStr">
         <is>
-          <t>617000</t>
+          <t>612730</t>
         </is>
       </c>
       <c r="G87" s="8" t="inlineStr">
         <is>
-          <t>Uitzendkrachten</t>
+          <t>TRANSPORTEN AAN DERDEN</t>
         </is>
       </c>
       <c r="H87" s="8" t="inlineStr">
@@ -12972,16 +12964,16 @@
         </is>
       </c>
       <c r="J87" s="9" t="n">
-        <v>390.26</v>
+        <v>1951.47</v>
       </c>
       <c r="K87" s="9" t="n">
-        <v>81.95</v>
+        <v>409.81</v>
       </c>
       <c r="L87" s="9" t="n">
         <v>0</v>
       </c>
       <c r="M87" s="9" t="n">
-        <v>472.21</v>
+        <v>2361.28</v>
       </c>
       <c r="N87" s="8" t="inlineStr">
         <is>
@@ -12995,7 +12987,7 @@
       </c>
       <c r="P87" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Findajob (2026-09-09)</t>
+          <t>in Yuki: Widem Logistics (2026-09-09)</t>
         </is>
       </c>
       <c r="Q87" s="8" t="inlineStr">
@@ -13017,7 +13009,7 @@
       </c>
       <c r="C88" s="8" t="inlineStr">
         <is>
-          <t>Widem Logistics NV</t>
+          <t>Findajob bv</t>
         </is>
       </c>
       <c r="D88" s="8" t="inlineStr"/>
@@ -13028,12 +13020,12 @@
       </c>
       <c r="F88" s="8" t="inlineStr">
         <is>
-          <t>612730</t>
+          <t>617000</t>
         </is>
       </c>
       <c r="G88" s="8" t="inlineStr">
         <is>
-          <t>TRANSPORTEN AAN DERDEN</t>
+          <t>Uitzendkrachten</t>
         </is>
       </c>
       <c r="H88" s="8" t="inlineStr">
@@ -13047,16 +13039,16 @@
         </is>
       </c>
       <c r="J88" s="9" t="n">
-        <v>215.73</v>
+        <v>390.26</v>
       </c>
       <c r="K88" s="9" t="n">
-        <v>45.3</v>
+        <v>81.95</v>
       </c>
       <c r="L88" s="9" t="n">
         <v>0</v>
       </c>
       <c r="M88" s="9" t="n">
-        <v>261.03</v>
+        <v>472.21</v>
       </c>
       <c r="N88" s="8" t="inlineStr">
         <is>
@@ -13070,7 +13062,7 @@
       </c>
       <c r="P88" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Widem Logistics (2026-09-09)</t>
+          <t>in Yuki: Findajob (2026-09-09)</t>
         </is>
       </c>
       <c r="Q88" s="8" t="inlineStr">
@@ -13122,16 +13114,16 @@
         </is>
       </c>
       <c r="J89" s="9" t="n">
-        <v>301.3</v>
+        <v>215.73</v>
       </c>
       <c r="K89" s="9" t="n">
-        <v>63.27</v>
+        <v>45.3</v>
       </c>
       <c r="L89" s="9" t="n">
         <v>0</v>
       </c>
       <c r="M89" s="9" t="n">
-        <v>364.57</v>
+        <v>261.03</v>
       </c>
       <c r="N89" s="8" t="inlineStr">
         <is>
@@ -13167,46 +13159,46 @@
       </c>
       <c r="C90" s="8" t="inlineStr">
         <is>
-          <t>Meta Platforms Ireland</t>
+          <t>Widem Logistics NV</t>
         </is>
       </c>
       <c r="D90" s="8" t="inlineStr"/>
       <c r="E90" s="8" t="inlineStr">
         <is>
-          <t>28354522874233099-28372066432478744</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="F90" s="8" t="inlineStr">
         <is>
-          <t>616502</t>
+          <t>612730</t>
         </is>
       </c>
       <c r="G90" s="8" t="inlineStr">
         <is>
-          <t>RECLAME MET MERK</t>
+          <t>TRANSPORTEN AAN DERDEN</t>
         </is>
       </c>
       <c r="H90" s="8" t="inlineStr">
         <is>
-          <t>EUDV</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="I90" s="8" t="inlineStr">
         <is>
-          <t>88 · 55 · 59</t>
+          <t>82 · 59</t>
         </is>
       </c>
       <c r="J90" s="9" t="n">
-        <v>555.08</v>
+        <v>301.3</v>
       </c>
       <c r="K90" s="9" t="n">
+        <v>63.27</v>
+      </c>
+      <c r="L90" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="L90" s="9" t="n">
-        <v>116.57</v>
-      </c>
       <c r="M90" s="9" t="n">
-        <v>555.08</v>
+        <v>364.57</v>
       </c>
       <c r="N90" s="8" t="inlineStr">
         <is>
@@ -13220,12 +13212,12 @@
       </c>
       <c r="P90" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28354522874233099-28372066432478744 (2026-09-08) – in Lucy/Yuki</t>
+          <t>in Yuki: Widem Logistics (2026-09-09)</t>
         </is>
       </c>
       <c r="Q90" s="8" t="inlineStr">
         <is>
-          <t>Yuki: intracommunautair diensten (verlegd)</t>
+          <t>Yuki: 21%</t>
         </is>
       </c>
     </row>
@@ -13237,7 +13229,7 @@
       </c>
       <c r="B91" s="8" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="C91" s="8" t="inlineStr">
@@ -13248,7 +13240,7 @@
       <c r="D91" s="8" t="inlineStr"/>
       <c r="E91" s="8" t="inlineStr">
         <is>
-          <t>28388089664209746-28211277685224280</t>
+          <t>28354522874233099-28372066432478744</t>
         </is>
       </c>
       <c r="F91" s="8" t="inlineStr">
@@ -13272,20 +13264,20 @@
         </is>
       </c>
       <c r="J91" s="9" t="n">
-        <v>800</v>
+        <v>555.08</v>
       </c>
       <c r="K91" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L91" s="9" t="n">
-        <v>168</v>
+        <v>116.57</v>
       </c>
       <c r="M91" s="9" t="n">
-        <v>800</v>
+        <v>555.08</v>
       </c>
       <c r="N91" s="8" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="O91" s="8" t="inlineStr">
@@ -13295,7 +13287,7 @@
       </c>
       <c r="P91" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28388089664209746-28211277685224280 (2026-09-10) – in Lucy/Yuki</t>
+          <t>Meta-kwitantie 28354522874233099-28372066432478744 (2026-09-08) – in Lucy/Yuki</t>
         </is>
       </c>
       <c r="Q91" s="8" t="inlineStr">
@@ -13312,70 +13304,62 @@
       </c>
       <c r="B92" s="8" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="C92" s="8" t="inlineStr">
         <is>
-          <t>Meta Platforms Ireland</t>
+          <t>Almost 3000</t>
         </is>
       </c>
       <c r="D92" s="8" t="inlineStr"/>
       <c r="E92" s="8" t="inlineStr">
         <is>
-          <t>28254286180923430-28254286254256756</t>
+          <t>Almost3000BV-011</t>
         </is>
       </c>
       <c r="F92" s="8" t="inlineStr">
         <is>
-          <t>616502</t>
+          <t>615300</t>
         </is>
       </c>
       <c r="G92" s="8" t="inlineStr">
         <is>
-          <t>RECLAME MET MERK</t>
+          <t>Overige erelonen</t>
         </is>
       </c>
       <c r="H92" s="8" t="inlineStr">
         <is>
-          <t>EUDV</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="I92" s="8" t="inlineStr">
         <is>
-          <t>88 · 55 · 59</t>
+          <t>82 · 59</t>
         </is>
       </c>
       <c r="J92" s="9" t="n">
-        <v>800</v>
+        <v>260</v>
       </c>
       <c r="K92" s="9" t="n">
+        <v>54.6</v>
+      </c>
+      <c r="L92" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="L92" s="9" t="n">
-        <v>168</v>
-      </c>
       <c r="M92" s="9" t="n">
-        <v>800</v>
-      </c>
-      <c r="N92" s="8" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
+        <v>314.6</v>
+      </c>
+      <c r="N92" s="8" t="inlineStr"/>
       <c r="O92" s="8" t="inlineStr">
         <is>
-          <t>550000 KBC zichtrekening</t>
-        </is>
-      </c>
-      <c r="P92" s="8" t="inlineStr">
-        <is>
-          <t>Meta-kwitantie 28254286180923430-28254286254256756 (2026-09-13) – in Lucy/Yuki</t>
-        </is>
-      </c>
+          <t xml:space="preserve"> nog te betalen (vervalt 2026-10-18)</t>
+        </is>
+      </c>
+      <c r="P92" s="8" t="inlineStr"/>
       <c r="Q92" s="8" t="inlineStr">
         <is>
-          <t>Yuki: intracommunautair diensten (verlegd)</t>
+          <t>Yuki: 21%</t>
         </is>
       </c>
     </row>
@@ -13387,55 +13371,55 @@
       </c>
       <c r="B93" s="8" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="C93" s="8" t="inlineStr">
         <is>
-          <t>Haddok BE9000 Gent, Belg Betaling met KBC-Debetkaa</t>
+          <t>Meta Platforms Ireland</t>
         </is>
       </c>
       <c r="D93" s="8" t="inlineStr"/>
       <c r="E93" s="8" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>28388089664209746-28211277685224280</t>
         </is>
       </c>
       <c r="F93" s="8" t="inlineStr">
         <is>
-          <t>611080</t>
+          <t>616502</t>
         </is>
       </c>
       <c r="G93" s="8" t="inlineStr">
         <is>
-          <t>ABONNEMENTEN</t>
+          <t>RECLAME MET MERK</t>
         </is>
       </c>
       <c r="H93" s="8" t="inlineStr">
         <is>
-          <t>BE21NA</t>
+          <t>EUDV</t>
         </is>
       </c>
       <c r="I93" s="8" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>88 · 55 · 59</t>
         </is>
       </c>
       <c r="J93" s="9" t="n">
-        <v>121.5</v>
+        <v>800</v>
       </c>
       <c r="K93" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L93" s="9" t="n">
-        <v>0</v>
+        <v>168</v>
       </c>
       <c r="M93" s="9" t="n">
-        <v>121.5</v>
+        <v>800</v>
       </c>
       <c r="N93" s="8" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="O93" s="8" t="inlineStr">
@@ -13445,12 +13429,12 @@
       </c>
       <c r="P93" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Haddok (2026-09-12)</t>
+          <t>Meta-kwitantie 28388089664209746-28211277685224280 (2026-09-10) – in Lucy/Yuki</t>
         </is>
       </c>
       <c r="Q93" s="8" t="inlineStr">
         <is>
-          <t>Yuki: 0% aftrek (restaurant)</t>
+          <t>Yuki: intracommunautair diensten (verlegd)</t>
         </is>
       </c>
     </row>
@@ -13462,55 +13446,55 @@
       </c>
       <c r="B94" s="8" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="C94" s="8" t="inlineStr">
         <is>
-          <t>Widem Logistics NV</t>
+          <t>Meta Platforms Ireland</t>
         </is>
       </c>
       <c r="D94" s="8" t="inlineStr"/>
       <c r="E94" s="8" t="inlineStr">
         <is>
-          <t>26015435</t>
+          <t>28254286180923430-28254286254256756</t>
         </is>
       </c>
       <c r="F94" s="8" t="inlineStr">
         <is>
-          <t>612730</t>
+          <t>616502</t>
         </is>
       </c>
       <c r="G94" s="8" t="inlineStr">
         <is>
-          <t>TRANSPORTEN AAN DERDEN</t>
+          <t>RECLAME MET MERK</t>
         </is>
       </c>
       <c r="H94" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>EUDV</t>
         </is>
       </c>
       <c r="I94" s="8" t="inlineStr">
         <is>
-          <t>82 · 59</t>
+          <t>88 · 55 · 59</t>
         </is>
       </c>
       <c r="J94" s="9" t="n">
-        <v>2687.43</v>
+        <v>800</v>
       </c>
       <c r="K94" s="9" t="n">
-        <v>564.36</v>
+        <v>0</v>
       </c>
       <c r="L94" s="9" t="n">
-        <v>0</v>
+        <v>168</v>
       </c>
       <c r="M94" s="9" t="n">
-        <v>3251.79</v>
+        <v>800</v>
       </c>
       <c r="N94" s="8" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="O94" s="8" t="inlineStr">
@@ -13520,12 +13504,12 @@
       </c>
       <c r="P94" s="8" t="inlineStr">
         <is>
-          <t>Widem 26015435 (mail 2026-09-15)</t>
+          <t>Meta-kwitantie 28254286180923430-28254286254256756 (2026-09-13) – in Lucy/Yuki</t>
         </is>
       </c>
       <c r="Q94" s="8" t="inlineStr">
         <is>
-          <t>Yuki: 21%</t>
+          <t>Yuki: intracommunautair diensten (verlegd)</t>
         </is>
       </c>
     </row>
@@ -13537,55 +13521,55 @@
       </c>
       <c r="B95" s="8" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="C95" s="8" t="inlineStr">
         <is>
-          <t>Meta Platforms Ireland</t>
+          <t>Haddok BE9000 Gent, Belg Betaling met KBC-Debetkaa</t>
         </is>
       </c>
       <c r="D95" s="8" t="inlineStr"/>
       <c r="E95" s="8" t="inlineStr">
         <is>
-          <t>28488005980884780-28343182888700429</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="F95" s="8" t="inlineStr">
         <is>
-          <t>616502</t>
+          <t>611080</t>
         </is>
       </c>
       <c r="G95" s="8" t="inlineStr">
         <is>
-          <t>RECLAME MET MERK</t>
+          <t>ABONNEMENTEN</t>
         </is>
       </c>
       <c r="H95" s="8" t="inlineStr">
         <is>
-          <t>EUDV</t>
+          <t>BE21NA</t>
         </is>
       </c>
       <c r="I95" s="8" t="inlineStr">
         <is>
-          <t>88 · 55 · 59</t>
+          <t>82</t>
         </is>
       </c>
       <c r="J95" s="9" t="n">
-        <v>800</v>
+        <v>121.5</v>
       </c>
       <c r="K95" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L95" s="9" t="n">
-        <v>168</v>
+        <v>0</v>
       </c>
       <c r="M95" s="9" t="n">
-        <v>800</v>
+        <v>121.5</v>
       </c>
       <c r="N95" s="8" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="O95" s="8" t="inlineStr">
@@ -13595,12 +13579,12 @@
       </c>
       <c r="P95" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28488005980884780-28343182888700429 (2026-09-17) – in Lucy/Yuki</t>
+          <t>in Yuki: Haddok (2026-09-12)</t>
         </is>
       </c>
       <c r="Q95" s="8" t="inlineStr">
         <is>
-          <t>Yuki: intracommunautair diensten (verlegd)</t>
+          <t>Yuki: 0% aftrek (restaurant)</t>
         </is>
       </c>
     </row>
@@ -13612,55 +13596,55 @@
       </c>
       <c r="B96" s="8" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="C96" s="8" t="inlineStr">
         <is>
-          <t>HIGGSFIELD INC. US94105 SAN FRANCISCO Betaling met</t>
+          <t>Widem Logistics NV</t>
         </is>
       </c>
       <c r="D96" s="8" t="inlineStr"/>
       <c r="E96" s="8" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>26015435</t>
         </is>
       </c>
       <c r="F96" s="8" t="inlineStr">
         <is>
-          <t>611080</t>
+          <t>612730</t>
         </is>
       </c>
       <c r="G96" s="8" t="inlineStr">
         <is>
-          <t>ABONNEMENTEN</t>
+          <t>TRANSPORTEN AAN DERDEN</t>
         </is>
       </c>
       <c r="H96" s="8" t="inlineStr">
         <is>
-          <t>NEUDV</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="I96" s="8" t="inlineStr">
         <is>
-          <t>87 · 56 · 59</t>
+          <t>82 · 59</t>
         </is>
       </c>
       <c r="J96" s="9" t="n">
-        <v>72</v>
+        <v>2687.43</v>
       </c>
       <c r="K96" s="9" t="n">
+        <v>564.36</v>
+      </c>
+      <c r="L96" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="L96" s="9" t="n">
-        <v>15.12</v>
-      </c>
       <c r="M96" s="9" t="n">
-        <v>72</v>
+        <v>3251.79</v>
       </c>
       <c r="N96" s="8" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="O96" s="8" t="inlineStr">
@@ -13670,12 +13654,12 @@
       </c>
       <c r="P96" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Higgsfield Inc (2026-09-20)</t>
+          <t>Widem 26015435 (mail 2026-09-15)</t>
         </is>
       </c>
       <c r="Q96" s="8" t="inlineStr">
         <is>
-          <t>Yuki: btw verlegd (dienst buiten EU)</t>
+          <t>Yuki: 21%</t>
         </is>
       </c>
     </row>
@@ -13687,70 +13671,62 @@
       </c>
       <c r="B97" s="8" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C97" s="8" t="inlineStr">
         <is>
-          <t>Meta Platforms Ireland</t>
+          <t>Thomas More Mechelen-Antwerpen</t>
         </is>
       </c>
       <c r="D97" s="8" t="inlineStr"/>
       <c r="E97" s="8" t="inlineStr">
         <is>
-          <t>28548539494831435-28333791032972949</t>
+          <t>TMM-62204778</t>
         </is>
       </c>
       <c r="F97" s="8" t="inlineStr">
         <is>
-          <t>616502</t>
+          <t>616651</t>
         </is>
       </c>
       <c r="G97" s="8" t="inlineStr">
         <is>
-          <t>RECLAME MET MERK</t>
+          <t>Beroepsbijdragen</t>
         </is>
       </c>
       <c r="H97" s="8" t="inlineStr">
         <is>
-          <t>EUDV</t>
+          <t>?</t>
         </is>
       </c>
       <c r="I97" s="8" t="inlineStr">
         <is>
-          <t>88 · 55 · 59</t>
+          <t>?</t>
         </is>
       </c>
       <c r="J97" s="9" t="n">
-        <v>800</v>
+        <v>75</v>
       </c>
       <c r="K97" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L97" s="9" t="n">
-        <v>168</v>
+        <v>0</v>
       </c>
       <c r="M97" s="9" t="n">
-        <v>800</v>
-      </c>
-      <c r="N97" s="8" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="N97" s="8" t="inlineStr"/>
       <c r="O97" s="8" t="inlineStr">
         <is>
-          <t>550000 KBC zichtrekening</t>
-        </is>
-      </c>
-      <c r="P97" s="8" t="inlineStr">
-        <is>
-          <t>Meta-kwitantie 28548539494831435-28333791032972949 (2026-09-20) – in Lucy/Yuki</t>
-        </is>
-      </c>
+          <t xml:space="preserve"> nog te betalen (vervalt 2026-10-17)</t>
+        </is>
+      </c>
+      <c r="P97" s="8" t="inlineStr"/>
       <c r="Q97" s="8" t="inlineStr">
         <is>
-          <t>Yuki: intracommunautair diensten (verlegd)</t>
+          <t>NAKIJKEN: btw-behandeling nakijken</t>
         </is>
       </c>
     </row>
@@ -13762,7 +13738,7 @@
       </c>
       <c r="B98" s="8" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C98" s="8" t="inlineStr">
@@ -13773,7 +13749,7 @@
       <c r="D98" s="8" t="inlineStr"/>
       <c r="E98" s="8" t="inlineStr">
         <is>
-          <t>28412552321763489-28417867054565341</t>
+          <t>28488005980884780-28343182888700429</t>
         </is>
       </c>
       <c r="F98" s="8" t="inlineStr">
@@ -13810,7 +13786,7 @@
       </c>
       <c r="N98" s="8" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="O98" s="8" t="inlineStr">
@@ -13820,7 +13796,7 @@
       </c>
       <c r="P98" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28412552321763489-28417867054565341 (2026-09-24) – in Lucy/Yuki</t>
+          <t>Meta-kwitantie 28488005980884780-28343182888700429 (2026-09-17) – in Lucy/Yuki</t>
         </is>
       </c>
       <c r="Q98" s="8" t="inlineStr">
@@ -13837,55 +13813,55 @@
       </c>
       <c r="B99" s="8" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="C99" s="8" t="inlineStr">
         <is>
-          <t>Meta Platforms Ireland</t>
+          <t>HIGGSFIELD INC. US94105 SAN FRANCISCO Betaling met</t>
         </is>
       </c>
       <c r="D99" s="8" t="inlineStr"/>
       <c r="E99" s="8" t="inlineStr">
         <is>
-          <t>28496207413397975-28665230016495716</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="F99" s="8" t="inlineStr">
         <is>
-          <t>616502</t>
+          <t>611080</t>
         </is>
       </c>
       <c r="G99" s="8" t="inlineStr">
         <is>
-          <t>RECLAME MET MERK</t>
+          <t>ABONNEMENTEN</t>
         </is>
       </c>
       <c r="H99" s="8" t="inlineStr">
         <is>
-          <t>EUDV</t>
+          <t>NEUDV</t>
         </is>
       </c>
       <c r="I99" s="8" t="inlineStr">
         <is>
-          <t>88 · 55 · 59</t>
+          <t>87 · 56 · 59</t>
         </is>
       </c>
       <c r="J99" s="9" t="n">
-        <v>800</v>
+        <v>72</v>
       </c>
       <c r="K99" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L99" s="9" t="n">
-        <v>168</v>
+        <v>15.12</v>
       </c>
       <c r="M99" s="9" t="n">
-        <v>800</v>
+        <v>72</v>
       </c>
       <c r="N99" s="8" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="O99" s="8" t="inlineStr">
@@ -13895,12 +13871,12 @@
       </c>
       <c r="P99" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28496207413397975-28665230016495716 (2026-09-27) – in Lucy/Yuki</t>
+          <t>in Yuki: Higgsfield Inc (2026-09-20)</t>
         </is>
       </c>
       <c r="Q99" s="8" t="inlineStr">
         <is>
-          <t>Yuki: intracommunautair diensten (verlegd)</t>
+          <t>Yuki: btw verlegd (dienst buiten EU)</t>
         </is>
       </c>
     </row>
@@ -13912,55 +13888,55 @@
       </c>
       <c r="B100" s="8" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="C100" s="8" t="inlineStr">
         <is>
-          <t>Findajob bv</t>
+          <t>Meta Platforms Ireland</t>
         </is>
       </c>
       <c r="D100" s="8" t="inlineStr"/>
       <c r="E100" s="8" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>28548539494831435-28333791032972949</t>
         </is>
       </c>
       <c r="F100" s="8" t="inlineStr">
         <is>
-          <t>617000</t>
+          <t>616502</t>
         </is>
       </c>
       <c r="G100" s="8" t="inlineStr">
         <is>
-          <t>Uitzendkrachten</t>
+          <t>RECLAME MET MERK</t>
         </is>
       </c>
       <c r="H100" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>EUDV</t>
         </is>
       </c>
       <c r="I100" s="8" t="inlineStr">
         <is>
-          <t>82 · 59</t>
+          <t>88 · 55 · 59</t>
         </is>
       </c>
       <c r="J100" s="9" t="n">
-        <v>180.62</v>
+        <v>800</v>
       </c>
       <c r="K100" s="9" t="n">
-        <v>37.93</v>
+        <v>0</v>
       </c>
       <c r="L100" s="9" t="n">
-        <v>0</v>
+        <v>168</v>
       </c>
       <c r="M100" s="9" t="n">
-        <v>218.55</v>
+        <v>800</v>
       </c>
       <c r="N100" s="8" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="O100" s="8" t="inlineStr">
@@ -13970,12 +13946,12 @@
       </c>
       <c r="P100" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Findajob (2026-09-29)</t>
+          <t>Meta-kwitantie 28548539494831435-28333791032972949 (2026-09-20) – in Lucy/Yuki</t>
         </is>
       </c>
       <c r="Q100" s="8" t="inlineStr">
         <is>
-          <t>Yuki: 21%</t>
+          <t>Yuki: intracommunautair diensten (verlegd)</t>
         </is>
       </c>
     </row>
@@ -13987,28 +13963,28 @@
       </c>
       <c r="B101" s="8" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C101" s="8" t="inlineStr">
         <is>
-          <t>Findajob bv</t>
+          <t>Widem Logistics</t>
         </is>
       </c>
       <c r="D101" s="8" t="inlineStr"/>
       <c r="E101" s="8" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>26016933</t>
         </is>
       </c>
       <c r="F101" s="8" t="inlineStr">
         <is>
-          <t>617000</t>
+          <t>612730</t>
         </is>
       </c>
       <c r="G101" s="8" t="inlineStr">
         <is>
-          <t>Uitzendkrachten</t>
+          <t>TRANSPORTEN AAN DERDEN</t>
         </is>
       </c>
       <c r="H101" s="8" t="inlineStr">
@@ -14022,32 +13998,24 @@
         </is>
       </c>
       <c r="J101" s="9" t="n">
-        <v>361.24</v>
+        <v>1009.43</v>
       </c>
       <c r="K101" s="9" t="n">
-        <v>75.86</v>
+        <v>211.98</v>
       </c>
       <c r="L101" s="9" t="n">
         <v>0</v>
       </c>
       <c r="M101" s="9" t="n">
-        <v>437.1</v>
-      </c>
-      <c r="N101" s="8" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
+        <v>1221.41</v>
+      </c>
+      <c r="N101" s="8" t="inlineStr"/>
       <c r="O101" s="8" t="inlineStr">
         <is>
-          <t>550000 KBC zichtrekening</t>
-        </is>
-      </c>
-      <c r="P101" s="8" t="inlineStr">
-        <is>
-          <t>in Yuki: Findajob (2026-09-29)</t>
-        </is>
-      </c>
+          <t xml:space="preserve"> nog te betalen (vervalt 2026-10-24)</t>
+        </is>
+      </c>
+      <c r="P101" s="8" t="inlineStr"/>
       <c r="Q101" s="8" t="inlineStr">
         <is>
           <t>Yuki: 21%</t>
@@ -14062,55 +14030,55 @@
       </c>
       <c r="B102" s="8" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C102" s="8" t="inlineStr">
         <is>
-          <t>Pro-Count</t>
+          <t>Meta Platforms Ireland</t>
         </is>
       </c>
       <c r="D102" s="8" t="inlineStr"/>
       <c r="E102" s="8" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>28412552321763489-28417867054565341</t>
         </is>
       </c>
       <c r="F102" s="8" t="inlineStr">
         <is>
-          <t>615200</t>
+          <t>616502</t>
         </is>
       </c>
       <c r="G102" s="8" t="inlineStr">
         <is>
-          <t>Erelonen boekhouders en accountants</t>
+          <t>RECLAME MET MERK</t>
         </is>
       </c>
       <c r="H102" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>EUDV</t>
         </is>
       </c>
       <c r="I102" s="8" t="inlineStr">
         <is>
-          <t>82 · 59</t>
+          <t>88 · 55 · 59</t>
         </is>
       </c>
       <c r="J102" s="9" t="n">
-        <v>200</v>
+        <v>800</v>
       </c>
       <c r="K102" s="9" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="L102" s="9" t="n">
-        <v>0</v>
+        <v>168</v>
       </c>
       <c r="M102" s="9" t="n">
-        <v>242</v>
+        <v>800</v>
       </c>
       <c r="N102" s="8" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="O102" s="8" t="inlineStr">
@@ -14120,12 +14088,12 @@
       </c>
       <c r="P102" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Pro-Count (2026-09-29)</t>
+          <t>Meta-kwitantie 28412552321763489-28417867054565341 (2026-09-24) – in Lucy/Yuki</t>
         </is>
       </c>
       <c r="Q102" s="8" t="inlineStr">
         <is>
-          <t>Yuki: 21%</t>
+          <t>Yuki: intracommunautair diensten (verlegd)</t>
         </is>
       </c>
     </row>
@@ -14137,55 +14105,55 @@
       </c>
       <c r="B103" s="8" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="C103" s="8" t="inlineStr">
         <is>
-          <t>bpost</t>
+          <t>Meta Platforms Ireland</t>
         </is>
       </c>
       <c r="D103" s="8" t="inlineStr"/>
       <c r="E103" s="8" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>28496207413397975-28665230016495716</t>
         </is>
       </c>
       <c r="F103" s="8" t="inlineStr">
         <is>
-          <t>611030</t>
+          <t>616502</t>
         </is>
       </c>
       <c r="G103" s="8" t="inlineStr">
         <is>
-          <t>PORTKOSTEN</t>
+          <t>RECLAME MET MERK</t>
         </is>
       </c>
       <c r="H103" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>EUDV</t>
         </is>
       </c>
       <c r="I103" s="8" t="inlineStr">
         <is>
-          <t>82 · 59</t>
+          <t>88 · 55 · 59</t>
         </is>
       </c>
       <c r="J103" s="9" t="n">
-        <v>5.6</v>
+        <v>800</v>
       </c>
       <c r="K103" s="9" t="n">
-        <v>1.18</v>
+        <v>0</v>
       </c>
       <c r="L103" s="9" t="n">
-        <v>0</v>
+        <v>168</v>
       </c>
       <c r="M103" s="9" t="n">
-        <v>6.78</v>
+        <v>800</v>
       </c>
       <c r="N103" s="8" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="O103" s="8" t="inlineStr">
@@ -14195,12 +14163,12 @@
       </c>
       <c r="P103" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Bpost (2026-09-29)</t>
+          <t>Meta-kwitantie 28496207413397975-28665230016495716 (2026-09-27) – in Lucy/Yuki</t>
         </is>
       </c>
       <c r="Q103" s="8" t="inlineStr">
         <is>
-          <t>Yuki: 21%</t>
+          <t>Yuki: intracommunautair diensten (verlegd)</t>
         </is>
       </c>
     </row>
@@ -14247,16 +14215,16 @@
         </is>
       </c>
       <c r="J104" s="9" t="n">
-        <v>197.04</v>
+        <v>180.62</v>
       </c>
       <c r="K104" s="9" t="n">
-        <v>41.38</v>
+        <v>37.93</v>
       </c>
       <c r="L104" s="9" t="n">
         <v>0</v>
       </c>
       <c r="M104" s="9" t="n">
-        <v>238.42</v>
+        <v>218.55</v>
       </c>
       <c r="N104" s="8" t="inlineStr">
         <is>
@@ -14279,203 +14247,557 @@
         </is>
       </c>
     </row>
+    <row r="105">
+      <c r="A105" s="8" t="inlineStr">
+        <is>
+          <t>in Yuki</t>
+        </is>
+      </c>
+      <c r="B105" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C105" s="8" t="inlineStr">
+        <is>
+          <t>Findajob bv</t>
+        </is>
+      </c>
+      <c r="D105" s="8" t="inlineStr"/>
+      <c r="E105" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="F105" s="8" t="inlineStr">
+        <is>
+          <t>617000</t>
+        </is>
+      </c>
+      <c r="G105" s="8" t="inlineStr">
+        <is>
+          <t>Uitzendkrachten</t>
+        </is>
+      </c>
+      <c r="H105" s="8" t="inlineStr">
+        <is>
+          <t>BE21</t>
+        </is>
+      </c>
+      <c r="I105" s="8" t="inlineStr">
+        <is>
+          <t>82 · 59</t>
+        </is>
+      </c>
+      <c r="J105" s="9" t="n">
+        <v>361.24</v>
+      </c>
+      <c r="K105" s="9" t="n">
+        <v>75.86</v>
+      </c>
+      <c r="L105" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M105" s="9" t="n">
+        <v>437.1</v>
+      </c>
+      <c r="N105" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="O105" s="8" t="inlineStr">
+        <is>
+          <t>550000 KBC zichtrekening</t>
+        </is>
+      </c>
+      <c r="P105" s="8" t="inlineStr">
+        <is>
+          <t>in Yuki: Findajob (2026-09-29)</t>
+        </is>
+      </c>
+      <c r="Q105" s="8" t="inlineStr">
+        <is>
+          <t>Yuki: 21%</t>
+        </is>
+      </c>
+    </row>
     <row r="106">
-      <c r="A106" s="6" t="inlineStr">
-        <is>
-          <t>Totaal per grootboekrekening</t>
+      <c r="A106" s="8" t="inlineStr">
+        <is>
+          <t>in Yuki</t>
+        </is>
+      </c>
+      <c r="B106" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C106" s="8" t="inlineStr">
+        <is>
+          <t>Pro-Count</t>
+        </is>
+      </c>
+      <c r="D106" s="8" t="inlineStr"/>
+      <c r="E106" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="F106" s="8" t="inlineStr">
+        <is>
+          <t>615200</t>
+        </is>
+      </c>
+      <c r="G106" s="8" t="inlineStr">
+        <is>
+          <t>Erelonen boekhouders en accountants</t>
+        </is>
+      </c>
+      <c r="H106" s="8" t="inlineStr">
+        <is>
+          <t>BE21</t>
+        </is>
+      </c>
+      <c r="I106" s="8" t="inlineStr">
+        <is>
+          <t>82 · 59</t>
+        </is>
+      </c>
+      <c r="J106" s="9" t="n">
+        <v>200</v>
+      </c>
+      <c r="K106" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="L106" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M106" s="9" t="n">
+        <v>242</v>
+      </c>
+      <c r="N106" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="O106" s="8" t="inlineStr">
+        <is>
+          <t>550000 KBC zichtrekening</t>
+        </is>
+      </c>
+      <c r="P106" s="8" t="inlineStr">
+        <is>
+          <t>in Yuki: Pro-Count (2026-09-29)</t>
+        </is>
+      </c>
+      <c r="Q106" s="8" t="inlineStr">
+        <is>
+          <t>Yuki: 21%</t>
         </is>
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="7" t="inlineStr">
-        <is>
-          <t>Rekening</t>
-        </is>
-      </c>
-      <c r="B107" s="7" t="inlineStr">
-        <is>
-          <t>Naam</t>
-        </is>
-      </c>
-      <c r="C107" s="7" t="inlineStr">
-        <is>
-          <t>Aantal</t>
-        </is>
-      </c>
-      <c r="D107" s="7" t="inlineStr">
-        <is>
-          <t>Maatstaf</t>
-        </is>
-      </c>
-      <c r="E107" s="7" t="inlineStr">
-        <is>
-          <t>Btw aftrekbaar</t>
+      <c r="A107" s="8" t="inlineStr">
+        <is>
+          <t>in Yuki</t>
+        </is>
+      </c>
+      <c r="B107" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C107" s="8" t="inlineStr">
+        <is>
+          <t>bpost</t>
+        </is>
+      </c>
+      <c r="D107" s="8" t="inlineStr"/>
+      <c r="E107" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="F107" s="8" t="inlineStr">
+        <is>
+          <t>611030</t>
+        </is>
+      </c>
+      <c r="G107" s="8" t="inlineStr">
+        <is>
+          <t>PORTKOSTEN</t>
+        </is>
+      </c>
+      <c r="H107" s="8" t="inlineStr">
+        <is>
+          <t>BE21</t>
+        </is>
+      </c>
+      <c r="I107" s="8" t="inlineStr">
+        <is>
+          <t>82 · 59</t>
+        </is>
+      </c>
+      <c r="J107" s="9" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="K107" s="9" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="L107" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M107" s="9" t="n">
+        <v>6.78</v>
+      </c>
+      <c r="N107" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="O107" s="8" t="inlineStr">
+        <is>
+          <t>550000 KBC zichtrekening</t>
+        </is>
+      </c>
+      <c r="P107" s="8" t="inlineStr">
+        <is>
+          <t>in Yuki: Bpost (2026-09-29)</t>
+        </is>
+      </c>
+      <c r="Q107" s="8" t="inlineStr">
+        <is>
+          <t>Yuki: 21%</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="8" t="inlineStr">
         <is>
-          <t>616502</t>
+          <t>in Yuki</t>
         </is>
       </c>
       <c r="B108" s="8" t="inlineStr">
         <is>
-          <t>RECLAME MET MERK</t>
-        </is>
-      </c>
-      <c r="C108" s="8" t="n">
-        <v>28</v>
-      </c>
-      <c r="D108" s="9" t="n">
-        <v>24441.18</v>
-      </c>
-      <c r="E108" s="9" t="n">
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C108" s="8" t="inlineStr">
+        <is>
+          <t>Findajob bv</t>
+        </is>
+      </c>
+      <c r="D108" s="8" t="inlineStr"/>
+      <c r="E108" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="F108" s="8" t="inlineStr">
+        <is>
+          <t>617000</t>
+        </is>
+      </c>
+      <c r="G108" s="8" t="inlineStr">
+        <is>
+          <t>Uitzendkrachten</t>
+        </is>
+      </c>
+      <c r="H108" s="8" t="inlineStr">
+        <is>
+          <t>BE21</t>
+        </is>
+      </c>
+      <c r="I108" s="8" t="inlineStr">
+        <is>
+          <t>82 · 59</t>
+        </is>
+      </c>
+      <c r="J108" s="9" t="n">
+        <v>197.04</v>
+      </c>
+      <c r="K108" s="9" t="n">
+        <v>41.38</v>
+      </c>
+      <c r="L108" s="9" t="n">
         <v>0</v>
+      </c>
+      <c r="M108" s="9" t="n">
+        <v>238.42</v>
+      </c>
+      <c r="N108" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="O108" s="8" t="inlineStr">
+        <is>
+          <t>550000 KBC zichtrekening</t>
+        </is>
+      </c>
+      <c r="P108" s="8" t="inlineStr">
+        <is>
+          <t>in Yuki: Findajob (2026-09-29)</t>
+        </is>
+      </c>
+      <c r="Q108" s="8" t="inlineStr">
+        <is>
+          <t>Yuki: 21%</t>
+        </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="8" t="inlineStr">
         <is>
-          <t>612730</t>
+          <t>in Yuki</t>
         </is>
       </c>
       <c r="B109" s="8" t="inlineStr">
         <is>
-          <t>TRANSPORTEN AAN DERDEN</t>
-        </is>
-      </c>
-      <c r="C109" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D109" s="9" t="n">
-        <v>10265.8</v>
-      </c>
-      <c r="E109" s="9" t="n">
-        <v>2155.8</v>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C109" s="8" t="inlineStr">
+        <is>
+          <t>Findajob</t>
+        </is>
+      </c>
+      <c r="D109" s="8" t="inlineStr"/>
+      <c r="E109" s="8" t="inlineStr">
+        <is>
+          <t>F001/202600701</t>
+        </is>
+      </c>
+      <c r="F109" s="8" t="inlineStr">
+        <is>
+          <t>617000</t>
+        </is>
+      </c>
+      <c r="G109" s="8" t="inlineStr">
+        <is>
+          <t>Uitzendkrachten</t>
+        </is>
+      </c>
+      <c r="H109" s="8" t="inlineStr">
+        <is>
+          <t>BE21</t>
+        </is>
+      </c>
+      <c r="I109" s="8" t="inlineStr">
+        <is>
+          <t>82 · 59</t>
+        </is>
+      </c>
+      <c r="J109" s="9" t="n">
+        <v>123.15</v>
+      </c>
+      <c r="K109" s="9" t="n">
+        <v>25.86</v>
+      </c>
+      <c r="L109" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M109" s="9" t="n">
+        <v>149.01</v>
+      </c>
+      <c r="N109" s="8" t="inlineStr"/>
+      <c r="O109" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> nog te betalen (vervalt 2026-10-07)</t>
+        </is>
+      </c>
+      <c r="P109" s="8" t="inlineStr"/>
+      <c r="Q109" s="8" t="inlineStr">
+        <is>
+          <t>Yuki: 21%</t>
+        </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="8" t="inlineStr">
         <is>
-          <t>604000</t>
+          <t>in Yuki</t>
         </is>
       </c>
       <c r="B110" s="8" t="inlineStr">
         <is>
-          <t>Aankopen van handelsgoederen</t>
-        </is>
-      </c>
-      <c r="C110" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D110" s="9" t="n">
-        <v>8637.91</v>
-      </c>
-      <c r="E110" s="9" t="n">
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C110" s="8" t="inlineStr">
+        <is>
+          <t>Findajob</t>
+        </is>
+      </c>
+      <c r="D110" s="8" t="inlineStr"/>
+      <c r="E110" s="8" t="inlineStr">
+        <is>
+          <t>F001/202600711</t>
+        </is>
+      </c>
+      <c r="F110" s="8" t="inlineStr">
+        <is>
+          <t>617000</t>
+        </is>
+      </c>
+      <c r="G110" s="8" t="inlineStr">
+        <is>
+          <t>Uitzendkrachten</t>
+        </is>
+      </c>
+      <c r="H110" s="8" t="inlineStr">
+        <is>
+          <t>BE21</t>
+        </is>
+      </c>
+      <c r="I110" s="8" t="inlineStr">
+        <is>
+          <t>82 · 59</t>
+        </is>
+      </c>
+      <c r="J110" s="9" t="n">
+        <v>131.36</v>
+      </c>
+      <c r="K110" s="9" t="n">
+        <v>27.59</v>
+      </c>
+      <c r="L110" s="9" t="n">
         <v>0</v>
+      </c>
+      <c r="M110" s="9" t="n">
+        <v>158.95</v>
+      </c>
+      <c r="N110" s="8" t="inlineStr"/>
+      <c r="O110" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> nog te betalen (vervalt 2026-10-08)</t>
+        </is>
+      </c>
+      <c r="P110" s="8" t="inlineStr"/>
+      <c r="Q110" s="8" t="inlineStr">
+        <is>
+          <t>Yuki: 21%</t>
+        </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="8" t="inlineStr">
         <is>
-          <t>617000</t>
+          <t>in Yuki</t>
         </is>
       </c>
       <c r="B111" s="8" t="inlineStr">
         <is>
-          <t>Uitzendkrachten</t>
-        </is>
-      </c>
-      <c r="C111" s="8" t="n">
-        <v>9</v>
-      </c>
-      <c r="D111" s="9" t="n">
-        <v>1733.66</v>
-      </c>
-      <c r="E111" s="9" t="n">
-        <v>364.06</v>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="8" t="inlineStr">
-        <is>
-          <t>611080</t>
-        </is>
-      </c>
-      <c r="B112" s="8" t="inlineStr">
-        <is>
-          <t>ABONNEMENTEN</t>
-        </is>
-      </c>
-      <c r="C112" s="8" t="n">
-        <v>24</v>
-      </c>
-      <c r="D112" s="9" t="n">
-        <v>1681.54</v>
-      </c>
-      <c r="E112" s="9" t="n">
-        <v>11.17</v>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C111" s="8" t="inlineStr">
+        <is>
+          <t>Widem Logistics</t>
+        </is>
+      </c>
+      <c r="D111" s="8" t="inlineStr"/>
+      <c r="E111" s="8" t="inlineStr">
+        <is>
+          <t>26017495</t>
+        </is>
+      </c>
+      <c r="F111" s="8" t="inlineStr">
+        <is>
+          <t>612730</t>
+        </is>
+      </c>
+      <c r="G111" s="8" t="inlineStr">
+        <is>
+          <t>TRANSPORTEN AAN DERDEN</t>
+        </is>
+      </c>
+      <c r="H111" s="8" t="inlineStr">
+        <is>
+          <t>BE21</t>
+        </is>
+      </c>
+      <c r="I111" s="8" t="inlineStr">
+        <is>
+          <t>82 · 59</t>
+        </is>
+      </c>
+      <c r="J111" s="9" t="n">
+        <v>1438.21</v>
+      </c>
+      <c r="K111" s="9" t="n">
+        <v>302.02</v>
+      </c>
+      <c r="L111" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M111" s="9" t="n">
+        <v>1740.23</v>
+      </c>
+      <c r="N111" s="8" t="inlineStr"/>
+      <c r="O111" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> nog te betalen (vervalt 2026-10-30)</t>
+        </is>
+      </c>
+      <c r="P111" s="8" t="inlineStr"/>
+      <c r="Q111" s="8" t="inlineStr">
+        <is>
+          <t>Yuki: 21%</t>
+        </is>
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="8" t="inlineStr">
-        <is>
-          <t>616501</t>
-        </is>
-      </c>
-      <c r="B113" s="8" t="inlineStr">
-        <is>
-          <t>RECLAME ZONDER MERK</t>
-        </is>
-      </c>
-      <c r="C113" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="D113" s="9" t="n">
-        <v>1084.76</v>
-      </c>
-      <c r="E113" s="9" t="n">
-        <v>0</v>
+      <c r="A113" s="6" t="inlineStr">
+        <is>
+          <t>Totaal per grootboekrekening</t>
+        </is>
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="8" t="inlineStr">
-        <is>
-          <t>601000</t>
-        </is>
-      </c>
-      <c r="B114" s="8" t="inlineStr">
-        <is>
-          <t>Aankopen van hulpstoffen</t>
-        </is>
-      </c>
-      <c r="C114" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D114" s="9" t="n">
-        <v>1025</v>
-      </c>
-      <c r="E114" s="9" t="n">
-        <v>0</v>
+      <c r="A114" s="7" t="inlineStr">
+        <is>
+          <t>Rekening</t>
+        </is>
+      </c>
+      <c r="B114" s="7" t="inlineStr">
+        <is>
+          <t>Naam</t>
+        </is>
+      </c>
+      <c r="C114" s="7" t="inlineStr">
+        <is>
+          <t>Aantal</t>
+        </is>
+      </c>
+      <c r="D114" s="7" t="inlineStr">
+        <is>
+          <t>Maatstaf</t>
+        </is>
+      </c>
+      <c r="E114" s="7" t="inlineStr">
+        <is>
+          <t>Btw aftrekbaar</t>
+        </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="8" t="inlineStr">
         <is>
-          <t>616620</t>
+          <t>616502</t>
         </is>
       </c>
       <c r="B115" s="8" t="inlineStr">
         <is>
-          <t>Beurzen en tentoonstellingen</t>
+          <t>RECLAME MET MERK</t>
         </is>
       </c>
       <c r="C115" s="8" t="n">
-        <v>3</v>
+        <v>28</v>
       </c>
       <c r="D115" s="9" t="n">
-        <v>670</v>
+        <v>24441.18</v>
       </c>
       <c r="E115" s="9" t="n">
         <v>0</v>
@@ -14484,103 +14806,103 @@
     <row r="116">
       <c r="A116" s="8" t="inlineStr">
         <is>
-          <t>615200</t>
+          <t>612730</t>
         </is>
       </c>
       <c r="B116" s="8" t="inlineStr">
         <is>
-          <t>Erelonen boekhouders en accountants</t>
+          <t>TRANSPORTEN AAN DERDEN</t>
         </is>
       </c>
       <c r="C116" s="8" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="D116" s="9" t="n">
-        <v>600</v>
+        <v>12713.44</v>
       </c>
       <c r="E116" s="9" t="n">
-        <v>126</v>
+        <v>2669.8</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="8" t="inlineStr">
         <is>
-          <t>611200</t>
+          <t>604000</t>
         </is>
       </c>
       <c r="B117" s="8" t="inlineStr">
         <is>
-          <t>Klein materiaal</t>
+          <t>Aankopen van handelsgoederen</t>
         </is>
       </c>
       <c r="C117" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D117" s="9" t="n">
-        <v>223.04</v>
+        <v>8637.91</v>
       </c>
       <c r="E117" s="9" t="n">
-        <v>10.24</v>
+        <v>0</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="8" t="inlineStr">
         <is>
-          <t>616651</t>
+          <t>617000</t>
         </is>
       </c>
       <c r="B118" s="8" t="inlineStr">
         <is>
-          <t>Beroepsbijdragen</t>
+          <t>Uitzendkrachten</t>
         </is>
       </c>
       <c r="C118" s="8" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D118" s="9" t="n">
-        <v>148</v>
+        <v>1988.17</v>
       </c>
       <c r="E118" s="9" t="n">
-        <v>0</v>
+        <v>417.51</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="8" t="inlineStr">
         <is>
-          <t>613210</t>
+          <t>611080</t>
         </is>
       </c>
       <c r="B119" s="8" t="inlineStr">
         <is>
-          <t>BURGERLIJKE AANSPRAKELIJKHEID</t>
+          <t>ABONNEMENTEN</t>
         </is>
       </c>
       <c r="C119" s="8" t="n">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="D119" s="9" t="n">
-        <v>55.41</v>
+        <v>1681.54</v>
       </c>
       <c r="E119" s="9" t="n">
-        <v>0</v>
+        <v>11.17</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="8" t="inlineStr">
         <is>
-          <t>616680</t>
+          <t>616501</t>
         </is>
       </c>
       <c r="B120" s="8" t="inlineStr">
         <is>
-          <t>Restaurantkosten</t>
+          <t>RECLAME ZONDER MERK</t>
         </is>
       </c>
       <c r="C120" s="8" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D120" s="9" t="n">
-        <v>50.1</v>
+        <v>1084.76</v>
       </c>
       <c r="E120" s="9" t="n">
         <v>0</v>
@@ -14589,26 +14911,215 @@
     <row r="121">
       <c r="A121" s="8" t="inlineStr">
         <is>
+          <t>601000</t>
+        </is>
+      </c>
+      <c r="B121" s="8" t="inlineStr">
+        <is>
+          <t>Aankopen van hulpstoffen</t>
+        </is>
+      </c>
+      <c r="C121" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D121" s="9" t="n">
+        <v>1025</v>
+      </c>
+      <c r="E121" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="8" t="inlineStr">
+        <is>
+          <t>616620</t>
+        </is>
+      </c>
+      <c r="B122" s="8" t="inlineStr">
+        <is>
+          <t>Beurzen en tentoonstellingen</t>
+        </is>
+      </c>
+      <c r="C122" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="D122" s="9" t="n">
+        <v>670</v>
+      </c>
+      <c r="E122" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="8" t="inlineStr">
+        <is>
+          <t>615200</t>
+        </is>
+      </c>
+      <c r="B123" s="8" t="inlineStr">
+        <is>
+          <t>Erelonen boekhouders en accountants</t>
+        </is>
+      </c>
+      <c r="C123" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="D123" s="9" t="n">
+        <v>600</v>
+      </c>
+      <c r="E123" s="9" t="n">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="8" t="inlineStr">
+        <is>
+          <t>615300</t>
+        </is>
+      </c>
+      <c r="B124" s="8" t="inlineStr">
+        <is>
+          <t>Overige erelonen</t>
+        </is>
+      </c>
+      <c r="C124" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D124" s="9" t="n">
+        <v>260</v>
+      </c>
+      <c r="E124" s="9" t="n">
+        <v>54.6</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="8" t="inlineStr">
+        <is>
+          <t>611200</t>
+        </is>
+      </c>
+      <c r="B125" s="8" t="inlineStr">
+        <is>
+          <t>Klein materiaal</t>
+        </is>
+      </c>
+      <c r="C125" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D125" s="9" t="n">
+        <v>223.04</v>
+      </c>
+      <c r="E125" s="9" t="n">
+        <v>10.24</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="8" t="inlineStr">
+        <is>
+          <t>616651</t>
+        </is>
+      </c>
+      <c r="B126" s="8" t="inlineStr">
+        <is>
+          <t>Beroepsbijdragen</t>
+        </is>
+      </c>
+      <c r="C126" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D126" s="9" t="n">
+        <v>223</v>
+      </c>
+      <c r="E126" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="8" t="inlineStr">
+        <is>
+          <t>613210</t>
+        </is>
+      </c>
+      <c r="B127" s="8" t="inlineStr">
+        <is>
+          <t>BURGERLIJKE AANSPRAKELIJKHEID</t>
+        </is>
+      </c>
+      <c r="C127" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="D127" s="9" t="n">
+        <v>55.41</v>
+      </c>
+      <c r="E127" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="8" t="inlineStr">
+        <is>
+          <t>616680</t>
+        </is>
+      </c>
+      <c r="B128" s="8" t="inlineStr">
+        <is>
+          <t>Restaurantkosten</t>
+        </is>
+      </c>
+      <c r="C128" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="D128" s="9" t="n">
+        <v>50.1</v>
+      </c>
+      <c r="E128" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="8" t="inlineStr">
+        <is>
           <t>611030</t>
         </is>
       </c>
-      <c r="B121" s="8" t="inlineStr">
+      <c r="B129" s="8" t="inlineStr">
         <is>
           <t>PORTKOSTEN</t>
         </is>
       </c>
-      <c r="C121" s="8" t="n">
+      <c r="C129" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="D121" s="9" t="n">
+      <c r="D129" s="9" t="n">
         <v>32.92</v>
       </c>
-      <c r="E121" s="9" t="n">
+      <c r="E129" s="9" t="n">
         <v>6.91</v>
       </c>
     </row>
+    <row r="130">
+      <c r="A130" s="8" t="inlineStr">
+        <is>
+          <t>657000</t>
+        </is>
+      </c>
+      <c r="B130" s="8" t="inlineStr">
+        <is>
+          <t>Diverse financiële kosten</t>
+        </is>
+      </c>
+      <c r="C130" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D130" s="9" t="n">
+        <v>8.26</v>
+      </c>
+      <c r="E130" s="9" t="n">
+        <v>1.74</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:Q104"/>
+  <autoFilter ref="A3:Q111"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Handmatige Yuki-betaling reserveert de bankverrichting
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WLjvFcZoD9WegLqrYozzyo
</commit_message>
<xml_diff>
--- a/boekhouding/rapporten/SmartPaw_Q3-2026.xlsx
+++ b/boekhouding/rapporten/SmartPaw_Q3-2026.xlsx
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Aankopen'!$A$3:$J$117</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Aankoopdagboek'!$A$3:$Q$111</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Aankoopdagboek'!$A$3:$Q$112</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -6724,7 +6724,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q130"/>
+  <dimension ref="A1:Q131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6749,7 +6749,7 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>Aankoopdagboek Q3 2026: 10 te boeken, 81 al in Yuki (ter controle), 17 zonder factuur. Grootboekrekeningen volgens jullie rekeningschema; btw-codes: eigen code + roosters.</t>
+          <t>Aankoopdagboek Q3 2026: 10 te boeken, 82 al in Yuki (ter controle), 17 zonder factuur. Grootboekrekeningen volgens jullie rekeningschema; btw-codes: eigen code + roosters.</t>
         </is>
       </c>
     </row>
@@ -13671,62 +13671,62 @@
       </c>
       <c r="B97" s="8" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C97" s="8" t="inlineStr">
         <is>
-          <t>Thomas More Mechelen-Antwerpen</t>
+          <t>Bpost</t>
         </is>
       </c>
       <c r="D97" s="8" t="inlineStr"/>
       <c r="E97" s="8" t="inlineStr">
         <is>
-          <t>TMM-62204778</t>
+          <t>268565664</t>
         </is>
       </c>
       <c r="F97" s="8" t="inlineStr">
         <is>
-          <t>616651</t>
+          <t>611030</t>
         </is>
       </c>
       <c r="G97" s="8" t="inlineStr">
         <is>
-          <t>Beroepsbijdragen</t>
+          <t>PORTKOSTEN</t>
         </is>
       </c>
       <c r="H97" s="8" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="I97" s="8" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>82 · 59</t>
         </is>
       </c>
       <c r="J97" s="9" t="n">
-        <v>75</v>
+        <v>5.6</v>
       </c>
       <c r="K97" s="9" t="n">
-        <v>0</v>
+        <v>1.18</v>
       </c>
       <c r="L97" s="9" t="n">
         <v>0</v>
       </c>
       <c r="M97" s="9" t="n">
-        <v>75</v>
+        <v>6.78</v>
       </c>
       <c r="N97" s="8" t="inlineStr"/>
       <c r="O97" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> nog te betalen (vervalt 2026-10-17)</t>
+          <t xml:space="preserve"> nog te betalen (vervalt 2026-10-16)</t>
         </is>
       </c>
       <c r="P97" s="8" t="inlineStr"/>
       <c r="Q97" s="8" t="inlineStr">
         <is>
-          <t>NAKIJKEN: btw-behandeling nakijken</t>
+          <t>Yuki: 21%</t>
         </is>
       </c>
     </row>
@@ -13743,65 +13743,57 @@
       </c>
       <c r="C98" s="8" t="inlineStr">
         <is>
-          <t>Meta Platforms Ireland</t>
+          <t>Thomas More Mechelen-Antwerpen</t>
         </is>
       </c>
       <c r="D98" s="8" t="inlineStr"/>
       <c r="E98" s="8" t="inlineStr">
         <is>
-          <t>28488005980884780-28343182888700429</t>
+          <t>TMM-62204778</t>
         </is>
       </c>
       <c r="F98" s="8" t="inlineStr">
         <is>
-          <t>616502</t>
+          <t>616651</t>
         </is>
       </c>
       <c r="G98" s="8" t="inlineStr">
         <is>
-          <t>RECLAME MET MERK</t>
+          <t>Beroepsbijdragen</t>
         </is>
       </c>
       <c r="H98" s="8" t="inlineStr">
         <is>
-          <t>EUDV</t>
+          <t>?</t>
         </is>
       </c>
       <c r="I98" s="8" t="inlineStr">
         <is>
-          <t>88 · 55 · 59</t>
+          <t>?</t>
         </is>
       </c>
       <c r="J98" s="9" t="n">
-        <v>800</v>
+        <v>75</v>
       </c>
       <c r="K98" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L98" s="9" t="n">
-        <v>168</v>
+        <v>0</v>
       </c>
       <c r="M98" s="9" t="n">
-        <v>800</v>
-      </c>
-      <c r="N98" s="8" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="N98" s="8" t="inlineStr"/>
       <c r="O98" s="8" t="inlineStr">
         <is>
-          <t>550000 KBC zichtrekening</t>
-        </is>
-      </c>
-      <c r="P98" s="8" t="inlineStr">
-        <is>
-          <t>Meta-kwitantie 28488005980884780-28343182888700429 (2026-09-17) – in Lucy/Yuki</t>
-        </is>
-      </c>
+          <t xml:space="preserve"> nog te betalen (vervalt 2026-10-17)</t>
+        </is>
+      </c>
+      <c r="P98" s="8" t="inlineStr"/>
       <c r="Q98" s="8" t="inlineStr">
         <is>
-          <t>Yuki: intracommunautair diensten (verlegd)</t>
+          <t>NAKIJKEN: btw-behandeling nakijken</t>
         </is>
       </c>
     </row>
@@ -13813,55 +13805,55 @@
       </c>
       <c r="B99" s="8" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C99" s="8" t="inlineStr">
         <is>
-          <t>HIGGSFIELD INC. US94105 SAN FRANCISCO Betaling met</t>
+          <t>Meta Platforms Ireland</t>
         </is>
       </c>
       <c r="D99" s="8" t="inlineStr"/>
       <c r="E99" s="8" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>28488005980884780-28343182888700429</t>
         </is>
       </c>
       <c r="F99" s="8" t="inlineStr">
         <is>
-          <t>611080</t>
+          <t>616502</t>
         </is>
       </c>
       <c r="G99" s="8" t="inlineStr">
         <is>
-          <t>ABONNEMENTEN</t>
+          <t>RECLAME MET MERK</t>
         </is>
       </c>
       <c r="H99" s="8" t="inlineStr">
         <is>
-          <t>NEUDV</t>
+          <t>EUDV</t>
         </is>
       </c>
       <c r="I99" s="8" t="inlineStr">
         <is>
-          <t>87 · 56 · 59</t>
+          <t>88 · 55 · 59</t>
         </is>
       </c>
       <c r="J99" s="9" t="n">
-        <v>72</v>
+        <v>800</v>
       </c>
       <c r="K99" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L99" s="9" t="n">
-        <v>15.12</v>
+        <v>168</v>
       </c>
       <c r="M99" s="9" t="n">
-        <v>72</v>
+        <v>800</v>
       </c>
       <c r="N99" s="8" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="O99" s="8" t="inlineStr">
@@ -13871,12 +13863,12 @@
       </c>
       <c r="P99" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Higgsfield Inc (2026-09-20)</t>
+          <t>Meta-kwitantie 28488005980884780-28343182888700429 (2026-09-17) – in Lucy/Yuki</t>
         </is>
       </c>
       <c r="Q99" s="8" t="inlineStr">
         <is>
-          <t>Yuki: btw verlegd (dienst buiten EU)</t>
+          <t>Yuki: intracommunautair diensten (verlegd)</t>
         </is>
       </c>
     </row>
@@ -13893,46 +13885,46 @@
       </c>
       <c r="C100" s="8" t="inlineStr">
         <is>
-          <t>Meta Platforms Ireland</t>
+          <t>HIGGSFIELD INC. US94105 SAN FRANCISCO Betaling met</t>
         </is>
       </c>
       <c r="D100" s="8" t="inlineStr"/>
       <c r="E100" s="8" t="inlineStr">
         <is>
-          <t>28548539494831435-28333791032972949</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="F100" s="8" t="inlineStr">
         <is>
-          <t>616502</t>
+          <t>611080</t>
         </is>
       </c>
       <c r="G100" s="8" t="inlineStr">
         <is>
-          <t>RECLAME MET MERK</t>
+          <t>ABONNEMENTEN</t>
         </is>
       </c>
       <c r="H100" s="8" t="inlineStr">
         <is>
-          <t>EUDV</t>
+          <t>NEUDV</t>
         </is>
       </c>
       <c r="I100" s="8" t="inlineStr">
         <is>
-          <t>88 · 55 · 59</t>
+          <t>87 · 56 · 59</t>
         </is>
       </c>
       <c r="J100" s="9" t="n">
-        <v>800</v>
+        <v>72</v>
       </c>
       <c r="K100" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L100" s="9" t="n">
-        <v>168</v>
+        <v>15.12</v>
       </c>
       <c r="M100" s="9" t="n">
-        <v>800</v>
+        <v>72</v>
       </c>
       <c r="N100" s="8" t="inlineStr">
         <is>
@@ -13946,12 +13938,12 @@
       </c>
       <c r="P100" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28548539494831435-28333791032972949 (2026-09-20) – in Lucy/Yuki</t>
+          <t>in Yuki: Higgsfield Inc (2026-09-20)</t>
         </is>
       </c>
       <c r="Q100" s="8" t="inlineStr">
         <is>
-          <t>Yuki: intracommunautair diensten (verlegd)</t>
+          <t>Yuki: btw verlegd (dienst buiten EU)</t>
         </is>
       </c>
     </row>
@@ -13963,62 +13955,70 @@
       </c>
       <c r="B101" s="8" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="C101" s="8" t="inlineStr">
         <is>
-          <t>Widem Logistics</t>
+          <t>Meta Platforms Ireland</t>
         </is>
       </c>
       <c r="D101" s="8" t="inlineStr"/>
       <c r="E101" s="8" t="inlineStr">
         <is>
-          <t>26016933</t>
+          <t>28548539494831435-28333791032972949</t>
         </is>
       </c>
       <c r="F101" s="8" t="inlineStr">
         <is>
-          <t>612730</t>
+          <t>616502</t>
         </is>
       </c>
       <c r="G101" s="8" t="inlineStr">
         <is>
-          <t>TRANSPORTEN AAN DERDEN</t>
+          <t>RECLAME MET MERK</t>
         </is>
       </c>
       <c r="H101" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>EUDV</t>
         </is>
       </c>
       <c r="I101" s="8" t="inlineStr">
         <is>
-          <t>82 · 59</t>
+          <t>88 · 55 · 59</t>
         </is>
       </c>
       <c r="J101" s="9" t="n">
-        <v>1009.43</v>
+        <v>800</v>
       </c>
       <c r="K101" s="9" t="n">
-        <v>211.98</v>
+        <v>0</v>
       </c>
       <c r="L101" s="9" t="n">
-        <v>0</v>
+        <v>168</v>
       </c>
       <c r="M101" s="9" t="n">
-        <v>1221.41</v>
-      </c>
-      <c r="N101" s="8" t="inlineStr"/>
+        <v>800</v>
+      </c>
+      <c r="N101" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
       <c r="O101" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> nog te betalen (vervalt 2026-10-24)</t>
-        </is>
-      </c>
-      <c r="P101" s="8" t="inlineStr"/>
+          <t>550000 KBC zichtrekening</t>
+        </is>
+      </c>
+      <c r="P101" s="8" t="inlineStr">
+        <is>
+          <t>Meta-kwitantie 28548539494831435-28333791032972949 (2026-09-20) – in Lucy/Yuki</t>
+        </is>
+      </c>
       <c r="Q101" s="8" t="inlineStr">
         <is>
-          <t>Yuki: 21%</t>
+          <t>Yuki: intracommunautair diensten (verlegd)</t>
         </is>
       </c>
     </row>
@@ -14035,65 +14035,57 @@
       </c>
       <c r="C102" s="8" t="inlineStr">
         <is>
-          <t>Meta Platforms Ireland</t>
+          <t>Widem Logistics</t>
         </is>
       </c>
       <c r="D102" s="8" t="inlineStr"/>
       <c r="E102" s="8" t="inlineStr">
         <is>
-          <t>28412552321763489-28417867054565341</t>
+          <t>26016933</t>
         </is>
       </c>
       <c r="F102" s="8" t="inlineStr">
         <is>
-          <t>616502</t>
+          <t>612730</t>
         </is>
       </c>
       <c r="G102" s="8" t="inlineStr">
         <is>
-          <t>RECLAME MET MERK</t>
+          <t>TRANSPORTEN AAN DERDEN</t>
         </is>
       </c>
       <c r="H102" s="8" t="inlineStr">
         <is>
-          <t>EUDV</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="I102" s="8" t="inlineStr">
         <is>
-          <t>88 · 55 · 59</t>
+          <t>82 · 59</t>
         </is>
       </c>
       <c r="J102" s="9" t="n">
-        <v>800</v>
+        <v>1009.43</v>
       </c>
       <c r="K102" s="9" t="n">
+        <v>211.98</v>
+      </c>
+      <c r="L102" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="L102" s="9" t="n">
-        <v>168</v>
-      </c>
       <c r="M102" s="9" t="n">
-        <v>800</v>
-      </c>
-      <c r="N102" s="8" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
+        <v>1221.41</v>
+      </c>
+      <c r="N102" s="8" t="inlineStr"/>
       <c r="O102" s="8" t="inlineStr">
         <is>
-          <t>550000 KBC zichtrekening</t>
-        </is>
-      </c>
-      <c r="P102" s="8" t="inlineStr">
-        <is>
-          <t>Meta-kwitantie 28412552321763489-28417867054565341 (2026-09-24) – in Lucy/Yuki</t>
-        </is>
-      </c>
+          <t xml:space="preserve"> nog te betalen (vervalt 2026-10-24)</t>
+        </is>
+      </c>
+      <c r="P102" s="8" t="inlineStr"/>
       <c r="Q102" s="8" t="inlineStr">
         <is>
-          <t>Yuki: intracommunautair diensten (verlegd)</t>
+          <t>Yuki: 21%</t>
         </is>
       </c>
     </row>
@@ -14105,7 +14097,7 @@
       </c>
       <c r="B103" s="8" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C103" s="8" t="inlineStr">
@@ -14116,7 +14108,7 @@
       <c r="D103" s="8" t="inlineStr"/>
       <c r="E103" s="8" t="inlineStr">
         <is>
-          <t>28496207413397975-28665230016495716</t>
+          <t>28412552321763489-28417867054565341</t>
         </is>
       </c>
       <c r="F103" s="8" t="inlineStr">
@@ -14153,7 +14145,7 @@
       </c>
       <c r="N103" s="8" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="O103" s="8" t="inlineStr">
@@ -14163,7 +14155,7 @@
       </c>
       <c r="P103" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28496207413397975-28665230016495716 (2026-09-27) – in Lucy/Yuki</t>
+          <t>Meta-kwitantie 28412552321763489-28417867054565341 (2026-09-24) – in Lucy/Yuki</t>
         </is>
       </c>
       <c r="Q103" s="8" t="inlineStr">
@@ -14180,55 +14172,55 @@
       </c>
       <c r="B104" s="8" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="C104" s="8" t="inlineStr">
         <is>
-          <t>Findajob bv</t>
+          <t>Meta Platforms Ireland</t>
         </is>
       </c>
       <c r="D104" s="8" t="inlineStr"/>
       <c r="E104" s="8" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>28496207413397975-28665230016495716</t>
         </is>
       </c>
       <c r="F104" s="8" t="inlineStr">
         <is>
-          <t>617000</t>
+          <t>616502</t>
         </is>
       </c>
       <c r="G104" s="8" t="inlineStr">
         <is>
-          <t>Uitzendkrachten</t>
+          <t>RECLAME MET MERK</t>
         </is>
       </c>
       <c r="H104" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>EUDV</t>
         </is>
       </c>
       <c r="I104" s="8" t="inlineStr">
         <is>
-          <t>82 · 59</t>
+          <t>88 · 55 · 59</t>
         </is>
       </c>
       <c r="J104" s="9" t="n">
-        <v>180.62</v>
+        <v>800</v>
       </c>
       <c r="K104" s="9" t="n">
-        <v>37.93</v>
+        <v>0</v>
       </c>
       <c r="L104" s="9" t="n">
-        <v>0</v>
+        <v>168</v>
       </c>
       <c r="M104" s="9" t="n">
-        <v>218.55</v>
+        <v>800</v>
       </c>
       <c r="N104" s="8" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="O104" s="8" t="inlineStr">
@@ -14238,12 +14230,12 @@
       </c>
       <c r="P104" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Findajob (2026-09-29)</t>
+          <t>Meta-kwitantie 28496207413397975-28665230016495716 (2026-09-27) – in Lucy/Yuki</t>
         </is>
       </c>
       <c r="Q104" s="8" t="inlineStr">
         <is>
-          <t>Yuki: 21%</t>
+          <t>Yuki: intracommunautair diensten (verlegd)</t>
         </is>
       </c>
     </row>
@@ -14290,16 +14282,16 @@
         </is>
       </c>
       <c r="J105" s="9" t="n">
-        <v>361.24</v>
+        <v>180.62</v>
       </c>
       <c r="K105" s="9" t="n">
-        <v>75.86</v>
+        <v>37.93</v>
       </c>
       <c r="L105" s="9" t="n">
         <v>0</v>
       </c>
       <c r="M105" s="9" t="n">
-        <v>437.1</v>
+        <v>218.55</v>
       </c>
       <c r="N105" s="8" t="inlineStr">
         <is>
@@ -14335,7 +14327,7 @@
       </c>
       <c r="C106" s="8" t="inlineStr">
         <is>
-          <t>Pro-Count</t>
+          <t>Findajob bv</t>
         </is>
       </c>
       <c r="D106" s="8" t="inlineStr"/>
@@ -14346,12 +14338,12 @@
       </c>
       <c r="F106" s="8" t="inlineStr">
         <is>
-          <t>615200</t>
+          <t>617000</t>
         </is>
       </c>
       <c r="G106" s="8" t="inlineStr">
         <is>
-          <t>Erelonen boekhouders en accountants</t>
+          <t>Uitzendkrachten</t>
         </is>
       </c>
       <c r="H106" s="8" t="inlineStr">
@@ -14365,16 +14357,16 @@
         </is>
       </c>
       <c r="J106" s="9" t="n">
-        <v>200</v>
+        <v>361.24</v>
       </c>
       <c r="K106" s="9" t="n">
-        <v>42</v>
+        <v>75.86</v>
       </c>
       <c r="L106" s="9" t="n">
         <v>0</v>
       </c>
       <c r="M106" s="9" t="n">
-        <v>242</v>
+        <v>437.1</v>
       </c>
       <c r="N106" s="8" t="inlineStr">
         <is>
@@ -14388,7 +14380,7 @@
       </c>
       <c r="P106" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Pro-Count (2026-09-29)</t>
+          <t>in Yuki: Findajob (2026-09-29)</t>
         </is>
       </c>
       <c r="Q106" s="8" t="inlineStr">
@@ -14410,7 +14402,7 @@
       </c>
       <c r="C107" s="8" t="inlineStr">
         <is>
-          <t>bpost</t>
+          <t>Pro-Count</t>
         </is>
       </c>
       <c r="D107" s="8" t="inlineStr"/>
@@ -14421,12 +14413,12 @@
       </c>
       <c r="F107" s="8" t="inlineStr">
         <is>
-          <t>611030</t>
+          <t>615200</t>
         </is>
       </c>
       <c r="G107" s="8" t="inlineStr">
         <is>
-          <t>PORTKOSTEN</t>
+          <t>Erelonen boekhouders en accountants</t>
         </is>
       </c>
       <c r="H107" s="8" t="inlineStr">
@@ -14440,16 +14432,16 @@
         </is>
       </c>
       <c r="J107" s="9" t="n">
-        <v>5.6</v>
+        <v>200</v>
       </c>
       <c r="K107" s="9" t="n">
-        <v>1.18</v>
+        <v>42</v>
       </c>
       <c r="L107" s="9" t="n">
         <v>0</v>
       </c>
       <c r="M107" s="9" t="n">
-        <v>6.78</v>
+        <v>242</v>
       </c>
       <c r="N107" s="8" t="inlineStr">
         <is>
@@ -14463,7 +14455,7 @@
       </c>
       <c r="P107" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Bpost (2026-09-29)</t>
+          <t>in Yuki: Pro-Count (2026-09-29)</t>
         </is>
       </c>
       <c r="Q107" s="8" t="inlineStr">
@@ -14485,7 +14477,7 @@
       </c>
       <c r="C108" s="8" t="inlineStr">
         <is>
-          <t>Findajob bv</t>
+          <t>bpost</t>
         </is>
       </c>
       <c r="D108" s="8" t="inlineStr"/>
@@ -14496,12 +14488,12 @@
       </c>
       <c r="F108" s="8" t="inlineStr">
         <is>
-          <t>617000</t>
+          <t>611030</t>
         </is>
       </c>
       <c r="G108" s="8" t="inlineStr">
         <is>
-          <t>Uitzendkrachten</t>
+          <t>PORTKOSTEN</t>
         </is>
       </c>
       <c r="H108" s="8" t="inlineStr">
@@ -14515,16 +14507,16 @@
         </is>
       </c>
       <c r="J108" s="9" t="n">
-        <v>197.04</v>
+        <v>5.6</v>
       </c>
       <c r="K108" s="9" t="n">
-        <v>41.38</v>
+        <v>1.18</v>
       </c>
       <c r="L108" s="9" t="n">
         <v>0</v>
       </c>
       <c r="M108" s="9" t="n">
-        <v>238.42</v>
+        <v>6.78</v>
       </c>
       <c r="N108" s="8" t="inlineStr">
         <is>
@@ -14538,7 +14530,7 @@
       </c>
       <c r="P108" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Findajob (2026-09-29)</t>
+          <t>in Yuki: Bpost (2026-09-29)</t>
         </is>
       </c>
       <c r="Q108" s="8" t="inlineStr">
@@ -14555,18 +14547,18 @@
       </c>
       <c r="B109" s="8" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C109" s="8" t="inlineStr">
         <is>
-          <t>Findajob</t>
+          <t>Findajob bv</t>
         </is>
       </c>
       <c r="D109" s="8" t="inlineStr"/>
       <c r="E109" s="8" t="inlineStr">
         <is>
-          <t>F001/202600701</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="F109" s="8" t="inlineStr">
@@ -14590,24 +14582,32 @@
         </is>
       </c>
       <c r="J109" s="9" t="n">
-        <v>123.15</v>
+        <v>197.04</v>
       </c>
       <c r="K109" s="9" t="n">
-        <v>25.86</v>
+        <v>41.38</v>
       </c>
       <c r="L109" s="9" t="n">
         <v>0</v>
       </c>
       <c r="M109" s="9" t="n">
-        <v>149.01</v>
-      </c>
-      <c r="N109" s="8" t="inlineStr"/>
+        <v>238.42</v>
+      </c>
+      <c r="N109" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="O109" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> nog te betalen (vervalt 2026-10-07)</t>
-        </is>
-      </c>
-      <c r="P109" s="8" t="inlineStr"/>
+          <t>550000 KBC zichtrekening</t>
+        </is>
+      </c>
+      <c r="P109" s="8" t="inlineStr">
+        <is>
+          <t>in Yuki: Findajob (2026-09-29)</t>
+        </is>
+      </c>
       <c r="Q109" s="8" t="inlineStr">
         <is>
           <t>Yuki: 21%</t>
@@ -14622,7 +14622,7 @@
       </c>
       <c r="B110" s="8" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C110" s="8" t="inlineStr">
@@ -14633,7 +14633,7 @@
       <c r="D110" s="8" t="inlineStr"/>
       <c r="E110" s="8" t="inlineStr">
         <is>
-          <t>F001/202600711</t>
+          <t>F001/202600701</t>
         </is>
       </c>
       <c r="F110" s="8" t="inlineStr">
@@ -14657,21 +14657,21 @@
         </is>
       </c>
       <c r="J110" s="9" t="n">
-        <v>131.36</v>
+        <v>123.15</v>
       </c>
       <c r="K110" s="9" t="n">
-        <v>27.59</v>
+        <v>25.86</v>
       </c>
       <c r="L110" s="9" t="n">
         <v>0</v>
       </c>
       <c r="M110" s="9" t="n">
-        <v>158.95</v>
+        <v>149.01</v>
       </c>
       <c r="N110" s="8" t="inlineStr"/>
       <c r="O110" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> nog te betalen (vervalt 2026-10-08)</t>
+          <t xml:space="preserve"> nog te betalen (vervalt 2026-10-07)</t>
         </is>
       </c>
       <c r="P110" s="8" t="inlineStr"/>
@@ -14694,23 +14694,23 @@
       </c>
       <c r="C111" s="8" t="inlineStr">
         <is>
-          <t>Widem Logistics</t>
+          <t>Findajob</t>
         </is>
       </c>
       <c r="D111" s="8" t="inlineStr"/>
       <c r="E111" s="8" t="inlineStr">
         <is>
-          <t>26017495</t>
+          <t>F001/202600711</t>
         </is>
       </c>
       <c r="F111" s="8" t="inlineStr">
         <is>
-          <t>612730</t>
+          <t>617000</t>
         </is>
       </c>
       <c r="G111" s="8" t="inlineStr">
         <is>
-          <t>TRANSPORTEN AAN DERDEN</t>
+          <t>Uitzendkrachten</t>
         </is>
       </c>
       <c r="H111" s="8" t="inlineStr">
@@ -14724,21 +14724,21 @@
         </is>
       </c>
       <c r="J111" s="9" t="n">
-        <v>1438.21</v>
+        <v>131.36</v>
       </c>
       <c r="K111" s="9" t="n">
-        <v>302.02</v>
+        <v>27.59</v>
       </c>
       <c r="L111" s="9" t="n">
         <v>0</v>
       </c>
       <c r="M111" s="9" t="n">
-        <v>1740.23</v>
+        <v>158.95</v>
       </c>
       <c r="N111" s="8" t="inlineStr"/>
       <c r="O111" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> nog te betalen (vervalt 2026-10-30)</t>
+          <t xml:space="preserve"> nog te betalen (vervalt 2026-10-08)</t>
         </is>
       </c>
       <c r="P111" s="8" t="inlineStr"/>
@@ -14748,182 +14748,228 @@
         </is>
       </c>
     </row>
-    <row r="113">
-      <c r="A113" s="6" t="inlineStr">
+    <row r="112">
+      <c r="A112" s="8" t="inlineStr">
+        <is>
+          <t>in Yuki</t>
+        </is>
+      </c>
+      <c r="B112" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C112" s="8" t="inlineStr">
+        <is>
+          <t>Widem Logistics</t>
+        </is>
+      </c>
+      <c r="D112" s="8" t="inlineStr"/>
+      <c r="E112" s="8" t="inlineStr">
+        <is>
+          <t>26017495</t>
+        </is>
+      </c>
+      <c r="F112" s="8" t="inlineStr">
+        <is>
+          <t>612730</t>
+        </is>
+      </c>
+      <c r="G112" s="8" t="inlineStr">
+        <is>
+          <t>TRANSPORTEN AAN DERDEN</t>
+        </is>
+      </c>
+      <c r="H112" s="8" t="inlineStr">
+        <is>
+          <t>BE21</t>
+        </is>
+      </c>
+      <c r="I112" s="8" t="inlineStr">
+        <is>
+          <t>82 · 59</t>
+        </is>
+      </c>
+      <c r="J112" s="9" t="n">
+        <v>1438.21</v>
+      </c>
+      <c r="K112" s="9" t="n">
+        <v>302.02</v>
+      </c>
+      <c r="L112" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M112" s="9" t="n">
+        <v>1740.23</v>
+      </c>
+      <c r="N112" s="8" t="inlineStr"/>
+      <c r="O112" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> nog te betalen (vervalt 2026-10-30)</t>
+        </is>
+      </c>
+      <c r="P112" s="8" t="inlineStr"/>
+      <c r="Q112" s="8" t="inlineStr">
+        <is>
+          <t>Yuki: 21%</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="6" t="inlineStr">
         <is>
           <t>Totaal per grootboekrekening</t>
         </is>
       </c>
     </row>
-    <row r="114">
-      <c r="A114" s="7" t="inlineStr">
+    <row r="115">
+      <c r="A115" s="7" t="inlineStr">
         <is>
           <t>Rekening</t>
         </is>
       </c>
-      <c r="B114" s="7" t="inlineStr">
+      <c r="B115" s="7" t="inlineStr">
         <is>
           <t>Naam</t>
         </is>
       </c>
-      <c r="C114" s="7" t="inlineStr">
+      <c r="C115" s="7" t="inlineStr">
         <is>
           <t>Aantal</t>
         </is>
       </c>
-      <c r="D114" s="7" t="inlineStr">
+      <c r="D115" s="7" t="inlineStr">
         <is>
           <t>Maatstaf</t>
         </is>
       </c>
-      <c r="E114" s="7" t="inlineStr">
+      <c r="E115" s="7" t="inlineStr">
         <is>
           <t>Btw aftrekbaar</t>
         </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" s="8" t="inlineStr">
-        <is>
-          <t>616502</t>
-        </is>
-      </c>
-      <c r="B115" s="8" t="inlineStr">
-        <is>
-          <t>RECLAME MET MERK</t>
-        </is>
-      </c>
-      <c r="C115" s="8" t="n">
-        <v>28</v>
-      </c>
-      <c r="D115" s="9" t="n">
-        <v>24441.18</v>
-      </c>
-      <c r="E115" s="9" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="8" t="inlineStr">
         <is>
-          <t>612730</t>
+          <t>616502</t>
         </is>
       </c>
       <c r="B116" s="8" t="inlineStr">
         <is>
-          <t>TRANSPORTEN AAN DERDEN</t>
+          <t>RECLAME MET MERK</t>
         </is>
       </c>
       <c r="C116" s="8" t="n">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="D116" s="9" t="n">
-        <v>12713.44</v>
+        <v>24441.18</v>
       </c>
       <c r="E116" s="9" t="n">
-        <v>2669.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="8" t="inlineStr">
         <is>
-          <t>604000</t>
+          <t>612730</t>
         </is>
       </c>
       <c r="B117" s="8" t="inlineStr">
         <is>
-          <t>Aankopen van handelsgoederen</t>
+          <t>TRANSPORTEN AAN DERDEN</t>
         </is>
       </c>
       <c r="C117" s="8" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D117" s="9" t="n">
-        <v>8637.91</v>
+        <v>12713.44</v>
       </c>
       <c r="E117" s="9" t="n">
-        <v>0</v>
+        <v>2669.8</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="8" t="inlineStr">
         <is>
-          <t>617000</t>
+          <t>604000</t>
         </is>
       </c>
       <c r="B118" s="8" t="inlineStr">
         <is>
-          <t>Uitzendkrachten</t>
+          <t>Aankopen van handelsgoederen</t>
         </is>
       </c>
       <c r="C118" s="8" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="D118" s="9" t="n">
-        <v>1988.17</v>
+        <v>8637.91</v>
       </c>
       <c r="E118" s="9" t="n">
-        <v>417.51</v>
+        <v>0</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="8" t="inlineStr">
         <is>
-          <t>611080</t>
+          <t>617000</t>
         </is>
       </c>
       <c r="B119" s="8" t="inlineStr">
         <is>
-          <t>ABONNEMENTEN</t>
+          <t>Uitzendkrachten</t>
         </is>
       </c>
       <c r="C119" s="8" t="n">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="D119" s="9" t="n">
-        <v>1681.54</v>
+        <v>1988.17</v>
       </c>
       <c r="E119" s="9" t="n">
-        <v>11.17</v>
+        <v>417.51</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="8" t="inlineStr">
         <is>
-          <t>616501</t>
+          <t>611080</t>
         </is>
       </c>
       <c r="B120" s="8" t="inlineStr">
         <is>
-          <t>RECLAME ZONDER MERK</t>
+          <t>ABONNEMENTEN</t>
         </is>
       </c>
       <c r="C120" s="8" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="D120" s="9" t="n">
-        <v>1084.76</v>
+        <v>1681.54</v>
       </c>
       <c r="E120" s="9" t="n">
-        <v>0</v>
+        <v>11.17</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="8" t="inlineStr">
         <is>
-          <t>601000</t>
+          <t>616501</t>
         </is>
       </c>
       <c r="B121" s="8" t="inlineStr">
         <is>
-          <t>Aankopen van hulpstoffen</t>
+          <t>RECLAME ZONDER MERK</t>
         </is>
       </c>
       <c r="C121" s="8" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D121" s="9" t="n">
-        <v>1025</v>
+        <v>1084.76</v>
       </c>
       <c r="E121" s="9" t="n">
         <v>0</v>
@@ -14932,19 +14978,19 @@
     <row r="122">
       <c r="A122" s="8" t="inlineStr">
         <is>
-          <t>616620</t>
+          <t>601000</t>
         </is>
       </c>
       <c r="B122" s="8" t="inlineStr">
         <is>
-          <t>Beurzen en tentoonstellingen</t>
+          <t>Aankopen van hulpstoffen</t>
         </is>
       </c>
       <c r="C122" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D122" s="9" t="n">
-        <v>670</v>
+        <v>1025</v>
       </c>
       <c r="E122" s="9" t="n">
         <v>0</v>
@@ -14953,103 +14999,103 @@
     <row r="123">
       <c r="A123" s="8" t="inlineStr">
         <is>
-          <t>615200</t>
+          <t>616620</t>
         </is>
       </c>
       <c r="B123" s="8" t="inlineStr">
         <is>
-          <t>Erelonen boekhouders en accountants</t>
+          <t>Beurzen en tentoonstellingen</t>
         </is>
       </c>
       <c r="C123" s="8" t="n">
         <v>3</v>
       </c>
       <c r="D123" s="9" t="n">
-        <v>600</v>
+        <v>670</v>
       </c>
       <c r="E123" s="9" t="n">
-        <v>126</v>
+        <v>0</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="8" t="inlineStr">
         <is>
-          <t>615300</t>
+          <t>615200</t>
         </is>
       </c>
       <c r="B124" s="8" t="inlineStr">
         <is>
-          <t>Overige erelonen</t>
+          <t>Erelonen boekhouders en accountants</t>
         </is>
       </c>
       <c r="C124" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D124" s="9" t="n">
-        <v>260</v>
+        <v>600</v>
       </c>
       <c r="E124" s="9" t="n">
-        <v>54.6</v>
+        <v>126</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="8" t="inlineStr">
         <is>
-          <t>611200</t>
+          <t>615300</t>
         </is>
       </c>
       <c r="B125" s="8" t="inlineStr">
         <is>
-          <t>Klein materiaal</t>
+          <t>Overige erelonen</t>
         </is>
       </c>
       <c r="C125" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D125" s="9" t="n">
-        <v>223.04</v>
+        <v>260</v>
       </c>
       <c r="E125" s="9" t="n">
-        <v>10.24</v>
+        <v>54.6</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="8" t="inlineStr">
         <is>
-          <t>616651</t>
+          <t>611200</t>
         </is>
       </c>
       <c r="B126" s="8" t="inlineStr">
         <is>
-          <t>Beroepsbijdragen</t>
+          <t>Klein materiaal</t>
         </is>
       </c>
       <c r="C126" s="8" t="n">
         <v>2</v>
       </c>
       <c r="D126" s="9" t="n">
-        <v>223</v>
+        <v>223.04</v>
       </c>
       <c r="E126" s="9" t="n">
-        <v>0</v>
+        <v>10.24</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="8" t="inlineStr">
         <is>
-          <t>613210</t>
+          <t>616651</t>
         </is>
       </c>
       <c r="B127" s="8" t="inlineStr">
         <is>
-          <t>BURGERLIJKE AANSPRAKELIJKHEID</t>
+          <t>Beroepsbijdragen</t>
         </is>
       </c>
       <c r="C127" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D127" s="9" t="n">
-        <v>55.41</v>
+        <v>223</v>
       </c>
       <c r="E127" s="9" t="n">
         <v>0</v>
@@ -15058,19 +15104,19 @@
     <row r="128">
       <c r="A128" s="8" t="inlineStr">
         <is>
-          <t>616680</t>
+          <t>613210</t>
         </is>
       </c>
       <c r="B128" s="8" t="inlineStr">
         <is>
-          <t>Restaurantkosten</t>
+          <t>BURGERLIJKE AANSPRAKELIJKHEID</t>
         </is>
       </c>
       <c r="C128" s="8" t="n">
         <v>3</v>
       </c>
       <c r="D128" s="9" t="n">
-        <v>50.1</v>
+        <v>55.41</v>
       </c>
       <c r="E128" s="9" t="n">
         <v>0</v>
@@ -15079,47 +15125,68 @@
     <row r="129">
       <c r="A129" s="8" t="inlineStr">
         <is>
-          <t>611030</t>
+          <t>616680</t>
         </is>
       </c>
       <c r="B129" s="8" t="inlineStr">
         <is>
-          <t>PORTKOSTEN</t>
+          <t>Restaurantkosten</t>
         </is>
       </c>
       <c r="C129" s="8" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D129" s="9" t="n">
-        <v>32.92</v>
+        <v>50.1</v>
       </c>
       <c r="E129" s="9" t="n">
-        <v>6.91</v>
+        <v>0</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="8" t="inlineStr">
         <is>
+          <t>611030</t>
+        </is>
+      </c>
+      <c r="B130" s="8" t="inlineStr">
+        <is>
+          <t>PORTKOSTEN</t>
+        </is>
+      </c>
+      <c r="C130" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="D130" s="9" t="n">
+        <v>38.52</v>
+      </c>
+      <c r="E130" s="9" t="n">
+        <v>8.09</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="8" t="inlineStr">
+        <is>
           <t>657000</t>
         </is>
       </c>
-      <c r="B130" s="8" t="inlineStr">
+      <c r="B131" s="8" t="inlineStr">
         <is>
           <t>Diverse financiële kosten</t>
         </is>
       </c>
-      <c r="C130" s="8" t="n">
+      <c r="C131" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="D130" s="9" t="n">
+      <c r="D131" s="9" t="n">
         <v>8.26</v>
       </c>
-      <c r="E130" s="9" t="n">
+      <c r="E131" s="9" t="n">
         <v>1.74</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:Q111"/>
+  <autoFilter ref="A3:Q112"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>